<commit_message>
results/new results for naive
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Zwischenstand.xlsx
+++ b/src/evaluation/data/Zwischenstand.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73A29D4-AED8-42D9-946B-5D9A5BC90153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43783D37-C8E7-4773-92BD-75462FE0035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="15">
   <si>
     <t>run1</t>
   </si>
@@ -459,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67BDA45F-A104-431D-A20F-223D7510156E}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -658,409 +658,642 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="4">
-        <v>0.629</v>
-      </c>
-      <c r="E14" s="2">
-        <f>AVERAGE(B14:D14)</f>
-        <v>0.629</v>
-      </c>
-      <c r="F14" s="2">
-        <f>E14-$E$3</f>
-        <v>-6.0000000000000053E-3</v>
-      </c>
-      <c r="G14">
-        <f>F14*100</f>
-        <v>-0.60000000000000053</v>
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="4">
-        <v>0.65200000000000002</v>
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>0.629</v>
       </c>
       <c r="E15" s="2">
-        <f t="shared" ref="E15:E22" si="1">AVERAGE(B15:D15)</f>
-        <v>0.65200000000000002</v>
+        <f>AVERAGE(B15:D15)</f>
+        <v>0.629</v>
       </c>
       <c r="F15" s="2">
-        <f>E15-$E$4</f>
-        <v>3.2000000000000028E-2</v>
+        <f>E15-$E$3</f>
+        <v>-6.0000000000000053E-3</v>
       </c>
       <c r="G15">
-        <f t="shared" ref="G15:G21" si="2">F15*100</f>
-        <v>3.2000000000000028</v>
+        <f>F15*100</f>
+        <v>-0.60000000000000053</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>0.65200000000000002</v>
+      </c>
+      <c r="E16" s="2">
+        <f t="shared" ref="E16:E23" si="1">AVERAGE(B16:D16)</f>
+        <v>0.65200000000000002</v>
+      </c>
+      <c r="F16" s="2">
+        <f>E16-$E$4</f>
+        <v>3.2000000000000028E-2</v>
+      </c>
+      <c r="G16">
+        <f t="shared" ref="G16:G22" si="2">F16*100</f>
+        <v>3.2000000000000028</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B17">
         <v>0.67200000000000004</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E17" s="2">
         <f t="shared" si="1"/>
         <v>0.67200000000000004</v>
       </c>
-      <c r="F16" s="2">
-        <f>E16-$E$5</f>
+      <c r="F17" s="2">
+        <f>E17-$E$5</f>
         <v>-4.4000000000000039E-2</v>
       </c>
-      <c r="G16">
+      <c r="G17">
         <f t="shared" si="2"/>
         <v>-4.4000000000000039</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B18">
         <v>0.75600000000000001</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E18" s="2">
         <f t="shared" si="1"/>
         <v>0.75600000000000001</v>
       </c>
-      <c r="F17" s="2">
-        <f>E17-$E$6</f>
+      <c r="F18" s="2">
+        <f>E18-$E$6</f>
         <v>-3.3333333333332993E-3</v>
       </c>
-      <c r="G17">
+      <c r="G18">
         <f t="shared" si="2"/>
         <v>-0.33333333333332993</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B19">
         <v>0.14000000000000001</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E19" s="2">
         <f t="shared" si="1"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="F18" s="2">
-        <f>E18-$E$7</f>
+      <c r="F19" s="2">
+        <f>E19-$E$7</f>
         <v>8.6666666666666836E-3</v>
       </c>
-      <c r="G18">
+      <c r="G19">
         <f t="shared" si="2"/>
         <v>0.86666666666666836</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B20">
         <v>0.6</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E20" s="2">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
-      <c r="F19" s="2">
-        <f>E19-$E$8</f>
+      <c r="F20" s="2">
+        <f>E20-$E$8</f>
         <v>1.4333333333333309E-2</v>
       </c>
-      <c r="G19">
+      <c r="G20">
         <f t="shared" si="2"/>
         <v>1.4333333333333309</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B21">
         <v>0.32100000000000001</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E21" s="2">
         <f t="shared" si="1"/>
         <v>0.32100000000000001</v>
       </c>
-      <c r="F20" s="2">
-        <f>E20-$E$9</f>
+      <c r="F21" s="2">
+        <f>E21-$E$9</f>
         <v>1.3000000000000012E-2</v>
       </c>
-      <c r="G20">
+      <c r="G21">
         <f t="shared" si="2"/>
         <v>1.3000000000000012</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B22">
         <v>0.46600000000000003</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E22" s="2">
         <f t="shared" si="1"/>
         <v>0.46600000000000003</v>
       </c>
-      <c r="F21" s="2">
-        <f>E21-$E$10</f>
+      <c r="F22" s="2">
+        <f>E22-$E$10</f>
         <v>5.4333333333333345E-2</v>
       </c>
-      <c r="G21">
+      <c r="G22">
         <f t="shared" si="2"/>
         <v>5.4333333333333345</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B23" s="1">
         <v>12.672000000000001</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E23" s="2">
         <f t="shared" si="1"/>
         <v>12.672000000000001</v>
       </c>
-      <c r="F22" s="2">
-        <f>E22-$E$11</f>
+      <c r="F23" s="2">
+        <f>E23-$E$11</f>
         <v>-19.094999999999995</v>
       </c>
     </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>1500</v>
+      </c>
+      <c r="B25">
+        <v>300</v>
+      </c>
+    </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>1750</v>
-      </c>
-      <c r="B26">
-        <v>300</v>
+      <c r="B26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" t="s">
-        <v>1</v>
-      </c>
-      <c r="D27" t="s">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>3</v>
-      </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" t="s">
-        <v>14</v>
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="C27" s="4">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="E27">
+        <f>AVERAGE(B27:D27)</f>
+        <v>0.63549999999999995</v>
+      </c>
+      <c r="F27">
+        <f>E27-$E$3</f>
+        <v>4.9999999999994493E-4</v>
+      </c>
+      <c r="G27">
+        <f>F27*100</f>
+        <v>4.9999999999994493E-2</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B28">
-        <v>0.61</v>
-      </c>
-      <c r="C28">
-        <v>0.625</v>
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="C28" s="4">
+        <v>0.69899999999999995</v>
       </c>
       <c r="E28">
-        <f>AVERAGE(B28:D28)</f>
-        <v>0.61749999999999994</v>
-      </c>
-      <c r="F28" s="2">
-        <f>E28-$E$3</f>
-        <v>-1.7500000000000071E-2</v>
+        <f t="shared" ref="E28:E35" si="3">AVERAGE(B28:D28)</f>
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="F28">
+        <f>E28-$E$4</f>
+        <v>7.7999999999999958E-2</v>
       </c>
       <c r="G28">
-        <f>F28*100</f>
-        <v>-1.7500000000000071</v>
+        <f t="shared" ref="G28:G34" si="4">F28*100</f>
+        <v>7.7999999999999954</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B29">
-        <v>0.67400000000000004</v>
-      </c>
-      <c r="C29">
-        <v>0.66500000000000004</v>
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="C29" s="4">
+        <v>0.71299999999999997</v>
       </c>
       <c r="E29">
-        <f t="shared" ref="E29:E36" si="3">AVERAGE(B29:D29)</f>
-        <v>0.66949999999999998</v>
-      </c>
-      <c r="F29" s="2">
-        <f>E29-$E$4</f>
-        <v>4.9499999999999988E-2</v>
+        <f t="shared" si="3"/>
+        <v>0.71899999999999997</v>
+      </c>
+      <c r="F29">
+        <f>E29-$E$5</f>
+        <v>2.9999999999998916E-3</v>
       </c>
       <c r="G29">
-        <f t="shared" ref="G29:G35" si="4">F29*100</f>
-        <v>4.9499999999999993</v>
+        <f t="shared" si="4"/>
+        <v>0.29999999999998916</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B30">
-        <v>0.65600000000000003</v>
-      </c>
-      <c r="C30">
-        <v>0.68600000000000005</v>
+        <v>0.75600000000000001</v>
+      </c>
+      <c r="C30" s="4">
+        <v>0.76400000000000001</v>
       </c>
       <c r="E30">
         <f t="shared" si="3"/>
-        <v>0.67100000000000004</v>
-      </c>
-      <c r="F30" s="2">
-        <f>E30-$E$5</f>
-        <v>-4.500000000000004E-2</v>
+        <v>0.76</v>
+      </c>
+      <c r="F30">
+        <f>E30-$E$6</f>
+        <v>6.6666666666670427E-4</v>
       </c>
       <c r="G30">
         <f t="shared" si="4"/>
-        <v>-4.5000000000000036</v>
+        <v>6.6666666666670427E-2</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B31">
-        <v>0.745</v>
-      </c>
-      <c r="C31">
-        <v>0.749</v>
+        <v>0.12</v>
+      </c>
+      <c r="C31" s="4">
+        <v>0.11600000000000001</v>
       </c>
       <c r="E31">
         <f t="shared" si="3"/>
-        <v>0.747</v>
-      </c>
-      <c r="F31" s="2">
-        <f>E31-$E$6</f>
-        <v>-1.2333333333333307E-2</v>
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="F31">
+        <f>E31-$E$7</f>
+        <v>-1.3333333333333336E-2</v>
       </c>
       <c r="G31">
         <f t="shared" si="4"/>
-        <v>-1.2333333333333307</v>
+        <v>-1.3333333333333335</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32">
-        <v>0.113</v>
-      </c>
-      <c r="C32">
-        <v>0.12</v>
+        <v>0.54300000000000004</v>
+      </c>
+      <c r="C32" s="4">
+        <v>0.53500000000000003</v>
       </c>
       <c r="E32">
         <f t="shared" si="3"/>
-        <v>0.11649999999999999</v>
-      </c>
-      <c r="F32" s="2">
-        <f>E32-$E$7</f>
-        <v>-1.4833333333333337E-2</v>
+        <v>0.53900000000000003</v>
+      </c>
+      <c r="F32">
+        <f>E32-$E$8</f>
+        <v>-4.6666666666666634E-2</v>
       </c>
       <c r="G32">
         <f t="shared" si="4"/>
-        <v>-1.4833333333333338</v>
+        <v>-4.6666666666666634</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B33">
-        <v>0.55300000000000005</v>
-      </c>
-      <c r="C33">
-        <v>0.56599999999999995</v>
+        <v>0.34899999999999998</v>
+      </c>
+      <c r="C33" s="4">
+        <v>0.311</v>
       </c>
       <c r="E33">
         <f t="shared" si="3"/>
-        <v>0.5595</v>
-      </c>
-      <c r="F33" s="2">
-        <f>E33-$E$8</f>
-        <v>-2.6166666666666671E-2</v>
+        <v>0.32999999999999996</v>
+      </c>
+      <c r="F33">
+        <f>E33-$E$9</f>
+        <v>2.1999999999999964E-2</v>
       </c>
       <c r="G33">
         <f t="shared" si="4"/>
-        <v>-2.6166666666666671</v>
+        <v>2.1999999999999966</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B34">
-        <v>0.23899999999999999</v>
-      </c>
-      <c r="C34">
-        <v>0.23799999999999999</v>
+        <v>0.52600000000000002</v>
+      </c>
+      <c r="C34" s="4">
+        <v>0.46100000000000002</v>
       </c>
       <c r="E34">
         <f t="shared" si="3"/>
-        <v>0.23849999999999999</v>
-      </c>
-      <c r="F34" s="2">
-        <f>E34-$E$9</f>
-        <v>-6.9500000000000006E-2</v>
+        <v>0.49350000000000005</v>
+      </c>
+      <c r="F34">
+        <f>E34-$E$10</f>
+        <v>8.1833333333333369E-2</v>
       </c>
       <c r="G34">
         <f t="shared" si="4"/>
-        <v>-6.9500000000000011</v>
+        <v>8.1833333333333371</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B35">
-        <v>0.38800000000000001</v>
-      </c>
-      <c r="C35">
-        <v>0.39700000000000002</v>
+        <v>22.539000000000001</v>
+      </c>
+      <c r="C35" s="1">
+        <v>12.643000000000001</v>
       </c>
       <c r="E35">
         <f t="shared" si="3"/>
+        <v>17.591000000000001</v>
+      </c>
+      <c r="F35">
+        <f>E35-$E$11</f>
+        <v>-14.175999999999995</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>1750</v>
+      </c>
+      <c r="B39">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" t="s">
+        <v>2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41">
+        <v>0.61</v>
+      </c>
+      <c r="C41">
+        <v>0.625</v>
+      </c>
+      <c r="E41">
+        <f>AVERAGE(B41:D41)</f>
+        <v>0.61749999999999994</v>
+      </c>
+      <c r="F41" s="2">
+        <f>E41-$E$3</f>
+        <v>-1.7500000000000071E-2</v>
+      </c>
+      <c r="G41">
+        <f>F41*100</f>
+        <v>-1.7500000000000071</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42">
+        <v>0.67400000000000004</v>
+      </c>
+      <c r="C42">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="E42">
+        <f t="shared" ref="E42:E49" si="5">AVERAGE(B42:D42)</f>
+        <v>0.66949999999999998</v>
+      </c>
+      <c r="F42" s="2">
+        <f>E42-$E$4</f>
+        <v>4.9499999999999988E-2</v>
+      </c>
+      <c r="G42">
+        <f t="shared" ref="G42:G48" si="6">F42*100</f>
+        <v>4.9499999999999993</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>0.65600000000000003</v>
+      </c>
+      <c r="C43">
+        <v>0.68600000000000005</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="5"/>
+        <v>0.67100000000000004</v>
+      </c>
+      <c r="F43" s="2">
+        <f>E43-$E$5</f>
+        <v>-4.500000000000004E-2</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="6"/>
+        <v>-4.5000000000000036</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44">
+        <v>0.745</v>
+      </c>
+      <c r="C44">
+        <v>0.749</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="5"/>
+        <v>0.747</v>
+      </c>
+      <c r="F44" s="2">
+        <f>E44-$E$6</f>
+        <v>-1.2333333333333307E-2</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="6"/>
+        <v>-1.2333333333333307</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>8</v>
+      </c>
+      <c r="B45">
+        <v>0.113</v>
+      </c>
+      <c r="C45">
+        <v>0.12</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="5"/>
+        <v>0.11649999999999999</v>
+      </c>
+      <c r="F45" s="2">
+        <f>E45-$E$7</f>
+        <v>-1.4833333333333337E-2</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="6"/>
+        <v>-1.4833333333333338</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46">
+        <v>0.55300000000000005</v>
+      </c>
+      <c r="C46">
+        <v>0.56599999999999995</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="5"/>
+        <v>0.5595</v>
+      </c>
+      <c r="F46" s="2">
+        <f>E46-$E$8</f>
+        <v>-2.6166666666666671E-2</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="6"/>
+        <v>-2.6166666666666671</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="C47">
+        <v>0.23799999999999999</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="5"/>
+        <v>0.23849999999999999</v>
+      </c>
+      <c r="F47" s="2">
+        <f>E47-$E$9</f>
+        <v>-6.9500000000000006E-2</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="6"/>
+        <v>-6.9500000000000011</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48">
+        <v>0.38800000000000001</v>
+      </c>
+      <c r="C48">
+        <v>0.39700000000000002</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="5"/>
         <v>0.39250000000000002</v>
       </c>
-      <c r="F35" s="2">
-        <f>E35-$E$10</f>
+      <c r="F48" s="2">
+        <f>E48-$E$10</f>
         <v>-1.9166666666666665E-2</v>
       </c>
-      <c r="G35">
-        <f t="shared" si="4"/>
+      <c r="G48">
+        <f t="shared" si="6"/>
         <v>-1.9166666666666665</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>12</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B49" s="1">
         <v>11.717000000000001</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C49" s="1">
         <v>25.544</v>
       </c>
-      <c r="E36">
-        <f t="shared" si="3"/>
+      <c r="E49">
+        <f t="shared" si="5"/>
         <v>18.630500000000001</v>
       </c>
-      <c r="F36" s="2">
-        <f>E36-$E$11</f>
+      <c r="F49" s="2">
+        <f>E49-$E$11</f>
         <v>-13.136499999999995</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Results: Neue Ergebnisse + Human Validation (Zwischenstand)
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Zwischenstand.xlsx
+++ b/src/evaluation/data/Zwischenstand.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0709E44E-E0F9-4FED-83A6-0C00AD465487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A751634-B774-4CAA-B635-6306AAEABAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="2" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="naive max_size" sheetId="1" r:id="rId1"/>
+    <sheet name="naive overlap" sheetId="2" r:id="rId2"/>
+    <sheet name="semantic percentile" sheetId="3" r:id="rId3"/>
+    <sheet name="semantic min_size" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="21">
   <si>
     <t>run1</t>
   </si>
@@ -91,13 +94,23 @@
   <si>
     <t>+</t>
   </si>
+  <si>
+    <t>naive</t>
+  </si>
+  <si>
+    <t>semantic</t>
+  </si>
+  <si>
+    <t>differenz</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -133,7 +146,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -705,11 +718,11 @@
       <c r="D15">
         <v>0.67240834386852077</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15">
         <f>AVERAGE(B15:D15)</f>
         <v>0.65438604332409633</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15">
         <f>E15-$E$3</f>
         <v>1.9386043324096325E-2</v>
       </c>
@@ -742,11 +755,11 @@
       <c r="D16">
         <v>0.65999999999999992</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16">
         <f t="shared" ref="E16:E23" si="1">AVERAGE(B16:D16)</f>
         <v>0.6628639846743295</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16">
         <f>E16-$E$4</f>
         <v>4.2863984674329503E-2</v>
       </c>
@@ -759,7 +772,7 @@
         <v>-3.131682968039784E-2</v>
       </c>
       <c r="I16">
-        <f t="shared" ref="I16:I23" si="4">H16*100</f>
+        <f t="shared" ref="I16:I22" si="4">H16*100</f>
         <v>-3.131682968039784</v>
       </c>
       <c r="J16" t="s">
@@ -779,11 +792,11 @@
       <c r="D17">
         <v>0.66101449273140767</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17">
         <f t="shared" si="1"/>
         <v>0.66045230854604076</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17">
         <f>E17-$E$5</f>
         <v>-5.5547691453959325E-2</v>
       </c>
@@ -816,11 +829,11 @@
       <c r="D18">
         <v>0.76358558102811269</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18">
         <f t="shared" si="1"/>
         <v>0.76358558102811269</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18">
         <f>E18-$E$6</f>
         <v>4.2522476947793875E-3</v>
       </c>
@@ -850,11 +863,11 @@
       <c r="D19">
         <v>0.13999108624627049</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19">
         <f t="shared" si="1"/>
         <v>0.13955340864777083</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19">
         <f>E19-$E$7</f>
         <v>8.2200753144374972E-3</v>
       </c>
@@ -887,11 +900,11 @@
       <c r="D20">
         <v>0.60592149549436569</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20">
         <f t="shared" si="1"/>
         <v>0.60494160541305908</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20">
         <f>E20-$E$8</f>
         <v>1.9274938746392412E-2</v>
       </c>
@@ -924,11 +937,11 @@
       <c r="D21">
         <v>0.3271551724137931</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21">
         <f t="shared" si="1"/>
         <v>0.31997126436781609</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21">
         <f>E21-$E$9</f>
         <v>1.1971264367816092E-2</v>
       </c>
@@ -958,11 +971,11 @@
       <c r="D22">
         <v>0.48275862068965519</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22">
         <f t="shared" si="1"/>
         <v>0.47413793103448282</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22">
         <f>E22-$E$10</f>
         <v>6.2471264367816137E-2</v>
       </c>
@@ -995,11 +1008,11 @@
       <c r="D23">
         <v>10.505874237109881</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23">
         <f t="shared" si="1"/>
         <v>11.027337059207348</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23">
         <f>E23-$E$11</f>
         <v>-20.739662940792648</v>
       </c>
@@ -1546,6 +1559,3066 @@
       <c r="F49" s="2">
         <f>E49-$E$11</f>
         <v>-14.673226030777233</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718267C3-91F6-4352-B487-1EEB3C8D4A90}">
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>1500</v>
+      </c>
+      <c r="B1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="C3">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="D3">
+        <v>0.63785624098124105</v>
+      </c>
+      <c r="E3">
+        <f>AVERAGE(B3:D3)</f>
+        <v>0.63628541366041358</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="C4">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="D4">
+        <v>0.68654244306418222</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E11" si="0">AVERAGE(B4:D4)</f>
+        <v>0.69418081435472734</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="C5">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="D5">
+        <v>0.70456521736496258</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>0.71418840578832088</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>0.75600000000000001</v>
+      </c>
+      <c r="C6">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="D6">
+        <v>0.76363038802542538</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.76121012934180854</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>0.12</v>
+      </c>
+      <c r="C7">
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="D7">
+        <v>0.12082725581784701</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.11894241860594901</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>0.54300000000000004</v>
+      </c>
+      <c r="C8">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="D8">
+        <v>0.54221877121649986</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0.54007292373883331</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>0.34899999999999998</v>
+      </c>
+      <c r="C9">
+        <v>0.311</v>
+      </c>
+      <c r="D9">
+        <v>0.31057971014492758</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0.32352657004830915</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>0.52600000000000002</v>
+      </c>
+      <c r="C10">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="D10">
+        <v>0.46086956521739131</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0.48262318840579715</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>22.539000000000001</v>
+      </c>
+      <c r="C11" s="1">
+        <v>12.643000000000001</v>
+      </c>
+      <c r="D11">
+        <v>10.93885221066682</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>15.373617403555608</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>1500</v>
+      </c>
+      <c r="B14">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16">
+        <v>0.62547831632653061</v>
+      </c>
+      <c r="C16">
+        <v>0.62649872448979593</v>
+      </c>
+      <c r="D16">
+        <v>0.60009566326530617</v>
+      </c>
+      <c r="E16">
+        <f>AVERAGE(B16:D16)</f>
+        <v>0.61735756802721087</v>
+      </c>
+      <c r="F16">
+        <f>E16-$E$3</f>
+        <v>-1.8927845633202711E-2</v>
+      </c>
+      <c r="G16">
+        <f>F16*100</f>
+        <v>-1.8927845633202711</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <v>0.67959770114942541</v>
+      </c>
+      <c r="C17">
+        <v>0.67744252873563227</v>
+      </c>
+      <c r="D17">
+        <v>0.6863505747126436</v>
+      </c>
+      <c r="E17">
+        <f t="shared" ref="E17:E24" si="1">AVERAGE(B17:D17)</f>
+        <v>0.68113026819923383</v>
+      </c>
+      <c r="F17">
+        <f>E17-$E$4</f>
+        <v>-1.3050546155493503E-2</v>
+      </c>
+      <c r="G17">
+        <f t="shared" ref="G17:G23" si="2">F17*100</f>
+        <v>-1.3050546155493503</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18">
+        <v>0.6919300766045261</v>
+      </c>
+      <c r="C18">
+        <v>0.68374042143241776</v>
+      </c>
+      <c r="D18">
+        <v>0.68393199231359436</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>0.68653416345017948</v>
+      </c>
+      <c r="F18">
+        <f>E18-$E$5</f>
+        <v>-2.7654242338141399E-2</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="2"/>
+        <v>-2.7654242338141399</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19">
+        <v>0.74649562333714237</v>
+      </c>
+      <c r="C19">
+        <v>0.74649562333714237</v>
+      </c>
+      <c r="D19">
+        <v>0.74649562333714237</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>0.74649562333714237</v>
+      </c>
+      <c r="F19">
+        <f>E19-$E$6</f>
+        <v>-1.4714506004666172E-2</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="2"/>
+        <v>-1.4714506004666172</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20">
+        <v>0.13243422379649381</v>
+      </c>
+      <c r="C20">
+        <v>0.1249492758066641</v>
+      </c>
+      <c r="D20">
+        <v>0.13516733837589159</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>0.13085027932634982</v>
+      </c>
+      <c r="F20">
+        <f>E20-$E$7</f>
+        <v>1.1907860720400815E-2</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="2"/>
+        <v>1.1907860720400816</v>
+      </c>
+      <c r="H20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21">
+        <v>0.50762176039660978</v>
+      </c>
+      <c r="C21">
+        <v>0.50766629049952128</v>
+      </c>
+      <c r="D21">
+        <v>0.50771524184532657</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>0.50766776424715254</v>
+      </c>
+      <c r="F21">
+        <f>E21-$E$8</f>
+        <v>-3.2405159491680768E-2</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="2"/>
+        <v>-3.2405159491680768</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22">
+        <v>0.33146551724137929</v>
+      </c>
+      <c r="C22">
+        <v>0.32284482758620692</v>
+      </c>
+      <c r="D22">
+        <v>0.32715517241379299</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>0.32715517241379305</v>
+      </c>
+      <c r="F22">
+        <f>E22-$E$9</f>
+        <v>3.6286023654839017E-3</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="2"/>
+        <v>0.36286023654839017</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23">
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="C23">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="D23">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>0.5114942528735632</v>
+      </c>
+      <c r="F23">
+        <f>E23-$E$10</f>
+        <v>2.887106446776605E-2</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="2"/>
+        <v>2.8871064467766052</v>
+      </c>
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24">
+        <v>10.864791746797231</v>
+      </c>
+      <c r="C24" s="1">
+        <v>10.36802453624791</v>
+      </c>
+      <c r="D24">
+        <v>10.57495007843807</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>10.60258878716107</v>
+      </c>
+      <c r="F24">
+        <f>E24-$E$11</f>
+        <v>-4.7710286163945383</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>1500</v>
+      </c>
+      <c r="B27">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29">
+        <v>0.61367116168001123</v>
+      </c>
+      <c r="C29">
+        <v>0.59977194303281267</v>
+      </c>
+      <c r="D29">
+        <v>0.60776092147773564</v>
+      </c>
+      <c r="E29">
+        <f>AVERAGE(B29:D29)</f>
+        <v>0.60706800873018663</v>
+      </c>
+      <c r="F29">
+        <f>E29-$E$3</f>
+        <v>-2.9217404930226953E-2</v>
+      </c>
+      <c r="G29">
+        <f>F29*100</f>
+        <v>-2.9217404930226953</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30">
+        <v>0.66752873563218385</v>
+      </c>
+      <c r="C30">
+        <v>0.64712643678160919</v>
+      </c>
+      <c r="D30">
+        <v>0.64985632183908049</v>
+      </c>
+      <c r="E30">
+        <f t="shared" ref="E30:E37" si="3">AVERAGE(B30:D30)</f>
+        <v>0.65483716475095788</v>
+      </c>
+      <c r="F30">
+        <f>E30-$E$4</f>
+        <v>-3.9343649603769459E-2</v>
+      </c>
+      <c r="G30">
+        <f t="shared" ref="G30:G36" si="4">F30*100</f>
+        <v>-3.9343649603769459</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31">
+        <v>0.6571739130208194</v>
+      </c>
+      <c r="C31">
+        <v>0.58146551722274542</v>
+      </c>
+      <c r="D31">
+        <v>0.62525362316846889</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="3"/>
+        <v>0.6212976844706779</v>
+      </c>
+      <c r="F31">
+        <f>E31-$E$5</f>
+        <v>-9.2890721317642977E-2</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="4"/>
+        <v>-9.2890721317642981</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32">
+        <v>0.75996748314060303</v>
+      </c>
+      <c r="C32">
+        <v>0.7565778749617017</v>
+      </c>
+      <c r="D32">
+        <v>0.75996748314060303</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="3"/>
+        <v>0.75883761374763592</v>
+      </c>
+      <c r="F32">
+        <f>E32-$E$6</f>
+        <v>-2.3725155941726195E-3</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="4"/>
+        <v>-0.23725155941726195</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33">
+        <v>0.14570914570883989</v>
+      </c>
+      <c r="C33">
+        <v>0.1088607187809871</v>
+      </c>
+      <c r="D33">
+        <v>0.12909339434045389</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="3"/>
+        <v>0.12788775294342694</v>
+      </c>
+      <c r="F33">
+        <f>E33-$E$7</f>
+        <v>8.9453343374779337E-3</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="4"/>
+        <v>0.89453343374779337</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34">
+        <v>0.61025808321708741</v>
+      </c>
+      <c r="C34">
+        <v>0.58939206857297222</v>
+      </c>
+      <c r="D34">
+        <v>0.61025808321708741</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="3"/>
+        <v>0.60330274500238235</v>
+      </c>
+      <c r="F34">
+        <f>E34-$E$8</f>
+        <v>6.3229821263549035E-2</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="4"/>
+        <v>6.3229821263549031</v>
+      </c>
+      <c r="H34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35">
+        <v>0.26551724137931038</v>
+      </c>
+      <c r="C35">
+        <v>0.24568965517241381</v>
+      </c>
+      <c r="D35">
+        <v>0.25258620689655181</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="3"/>
+        <v>0.25459770114942537</v>
+      </c>
+      <c r="F35">
+        <f>E35-$E$9</f>
+        <v>-6.8928868898883777E-2</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="4"/>
+        <v>-6.8928868898883779</v>
+      </c>
+      <c r="H35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36">
+        <v>0.44827586206896552</v>
+      </c>
+      <c r="C36">
+        <v>0.42241379310344829</v>
+      </c>
+      <c r="D36">
+        <v>0.43103448275862072</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="3"/>
+        <v>0.43390804597701149</v>
+      </c>
+      <c r="F36">
+        <f>E36-$E$10</f>
+        <v>-4.8715142428785663E-2</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="4"/>
+        <v>-4.8715142428785665</v>
+      </c>
+      <c r="H36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37">
+        <v>12.757253385823351</v>
+      </c>
+      <c r="C37" s="1">
+        <v>11.61612859676624</v>
+      </c>
+      <c r="D37">
+        <v>12.433386225124879</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="3"/>
+        <v>12.268922735904823</v>
+      </c>
+      <c r="F37">
+        <f>E37-$E$11</f>
+        <v>-3.1046946676507847</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C2C1CF-AF99-4FC0-A37D-09071864ECF5}">
+  <dimension ref="A1:O67"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1500</v>
+      </c>
+      <c r="B2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.63928167139374037</v>
+      </c>
+      <c r="C4">
+        <v>0.63161098979683061</v>
+      </c>
+      <c r="D4">
+        <v>0.63785624098124105</v>
+      </c>
+      <c r="E4">
+        <f>AVERAGE(B4:D4)</f>
+        <v>0.63624963405727064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0.69714696223316919</v>
+      </c>
+      <c r="C5">
+        <v>0.699296066252588</v>
+      </c>
+      <c r="D5">
+        <v>0.68654244306418222</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E12" si="0">AVERAGE(B5:D5)</f>
+        <v>0.69432849051664647</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>0.72491618771193134</v>
+      </c>
+      <c r="C6">
+        <v>0.71271739127692224</v>
+      </c>
+      <c r="D6">
+        <v>0.70456521736496258</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.71406626545127205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.75592343025572384</v>
+      </c>
+      <c r="C7">
+        <v>0.76445786427386186</v>
+      </c>
+      <c r="D7">
+        <v>0.76363038802542538</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.7613372275183371</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>0.1202172178095338</v>
+      </c>
+      <c r="C8">
+        <v>0.1158506141244314</v>
+      </c>
+      <c r="D8">
+        <v>0.12082725581784701</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0.11896502925060408</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>0.54251985943136916</v>
+      </c>
+      <c r="C9">
+        <v>0.53545989803191707</v>
+      </c>
+      <c r="D9">
+        <v>0.54221877121649986</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0.54006617622659536</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>0.34885057471264369</v>
+      </c>
+      <c r="C10">
+        <v>0.31057971014492758</v>
+      </c>
+      <c r="D10">
+        <v>0.31057971014492758</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0.32333666500083297</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>0.52586206896551724</v>
+      </c>
+      <c r="C11">
+        <v>0.46086956521739131</v>
+      </c>
+      <c r="D11">
+        <v>0.46086956521739131</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0.48253373313343334</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>22.538866022537491</v>
+      </c>
+      <c r="C12">
+        <v>12.643024224820341</v>
+      </c>
+      <c r="D12">
+        <v>10.93885221066682</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>15.37358081934155</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1500</v>
+      </c>
+      <c r="B16">
+        <v>300</v>
+      </c>
+      <c r="C16">
+        <v>400</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>0.63351272621184107</v>
+      </c>
+      <c r="C18">
+        <v>0.62602869107293879</v>
+      </c>
+      <c r="D18">
+        <v>0.63562295404400659</v>
+      </c>
+      <c r="E18">
+        <f t="shared" ref="E18:E26" si="1">AVERAGE(B18:D18)</f>
+        <v>0.63172145710959549</v>
+      </c>
+      <c r="F18">
+        <f>E18-E$4</f>
+        <v>-4.5281769476751554E-3</v>
+      </c>
+      <c r="G18">
+        <f>F18*100</f>
+        <v>-0.45281769476751554</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19">
+        <v>0.63060344827586212</v>
+      </c>
+      <c r="C19">
+        <v>0.62227011494252882</v>
+      </c>
+      <c r="D19">
+        <v>0.63376436781609191</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>0.62887931034482758</v>
+      </c>
+      <c r="F19">
+        <f>E19-E$5</f>
+        <v>-6.5449180171818888E-2</v>
+      </c>
+      <c r="G19">
+        <f t="shared" ref="G19:G25" si="2">F19*100</f>
+        <v>-6.5449180171818888</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>0.70974637678520747</v>
+      </c>
+      <c r="C20">
+        <v>0.72195652171092872</v>
+      </c>
+      <c r="D20">
+        <v>0.7130268198961851</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>0.71490990613077388</v>
+      </c>
+      <c r="F20">
+        <f>E20-E$6</f>
+        <v>8.4364067950182253E-4</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="2"/>
+        <v>8.4364067950182253E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="C21">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="D21">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="F21">
+        <f>E21-E$7</f>
+        <v>-1.2756488019539658E-3</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="2"/>
+        <v>-0.12756488019539658</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22">
+        <v>0.14863753589118131</v>
+      </c>
+      <c r="C22">
+        <v>0.14382413673605429</v>
+      </c>
+      <c r="D22">
+        <v>0.15017526964578171</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>0.14754564742433909</v>
+      </c>
+      <c r="F22">
+        <f>E22-E$8</f>
+        <v>2.8580618173735015E-2</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="2"/>
+        <v>2.8580618173735015</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23">
+        <v>0.5552812872194981</v>
+      </c>
+      <c r="C23">
+        <v>0.55531351804635143</v>
+      </c>
+      <c r="D23">
+        <v>0.55530281878956966</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>0.55529920801847299</v>
+      </c>
+      <c r="F23">
+        <f>E23-E$9</f>
+        <v>1.5233031791877627E-2</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="2"/>
+        <v>1.5233031791877627</v>
+      </c>
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24">
+        <v>0.36206896551724138</v>
+      </c>
+      <c r="C24">
+        <v>0.35344827586206901</v>
+      </c>
+      <c r="D24">
+        <v>0.35344827586206901</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>0.35632183908045983</v>
+      </c>
+      <c r="F24">
+        <f>E24-E$10</f>
+        <v>3.2985174079626867E-2</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="2"/>
+        <v>3.2985174079626867</v>
+      </c>
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="C25">
+        <v>0.5</v>
+      </c>
+      <c r="D25">
+        <v>0.5</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="1"/>
+        <v>0.50287356321839083</v>
+      </c>
+      <c r="F25">
+        <f>E25-E$11</f>
+        <v>2.0339830084957489E-2</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="2"/>
+        <v>2.0339830084957491</v>
+      </c>
+      <c r="H25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26">
+        <v>11.19616421337785</v>
+      </c>
+      <c r="C26" s="1">
+        <v>11.108016953386111</v>
+      </c>
+      <c r="D26">
+        <v>10.89680967659786</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="1"/>
+        <v>11.066996947787274</v>
+      </c>
+      <c r="F26">
+        <f>E26-E$12</f>
+        <v>-4.3065838715542757</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>1500</v>
+      </c>
+      <c r="B30">
+        <v>300</v>
+      </c>
+      <c r="C30">
+        <v>400</v>
+      </c>
+      <c r="D30">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32">
+        <v>0.65619604566972978</v>
+      </c>
+      <c r="C32">
+        <v>0.66472755366560665</v>
+      </c>
+      <c r="D32">
+        <v>0.65075219614693292</v>
+      </c>
+      <c r="E32">
+        <f t="shared" ref="E32:E40" si="3">AVERAGE(B32:D32)</f>
+        <v>0.65722526516075652</v>
+      </c>
+      <c r="F32">
+        <f>E32-E$4</f>
+        <v>2.0975631103485881E-2</v>
+      </c>
+      <c r="G32">
+        <f>F32*100</f>
+        <v>2.0975631103485881</v>
+      </c>
+      <c r="H32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33">
+        <v>0.63069581280788167</v>
+      </c>
+      <c r="C33">
+        <v>0.64793719211822653</v>
+      </c>
+      <c r="D33">
+        <v>0.67092569786535317</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="3"/>
+        <v>0.64985290093048709</v>
+      </c>
+      <c r="F33">
+        <f>E33-E$5</f>
+        <v>-4.4475589586159381E-2</v>
+      </c>
+      <c r="G33">
+        <f t="shared" ref="G33:G39" si="4">F33*100</f>
+        <v>-4.4475589586159376</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34">
+        <v>0.70167874393576857</v>
+      </c>
+      <c r="C34">
+        <v>0.70777059384295604</v>
+      </c>
+      <c r="D34">
+        <v>0.70626811591633665</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="3"/>
+        <v>0.70523915123168701</v>
+      </c>
+      <c r="F34">
+        <f>E34-E$6</f>
+        <v>-8.8271142195850416E-3</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="4"/>
+        <v>-0.88271142195850416</v>
+      </c>
+      <c r="H34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35">
+        <v>0.7645731722938216</v>
+      </c>
+      <c r="C35">
+        <v>0.7645731722938216</v>
+      </c>
+      <c r="D35">
+        <v>0.7645731722938216</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="3"/>
+        <v>0.76457317229382171</v>
+      </c>
+      <c r="F35">
+        <f>E35-E$7</f>
+        <v>3.2359447754846116E-3</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="4"/>
+        <v>0.32359447754846116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36">
+        <v>0.14562855618653209</v>
+      </c>
+      <c r="C36">
+        <v>0.13882559465945099</v>
+      </c>
+      <c r="D36">
+        <v>0.141336252868936</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="3"/>
+        <v>0.14193013457163969</v>
+      </c>
+      <c r="F36">
+        <f>E36-E$8</f>
+        <v>2.2965105321035614E-2</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="4"/>
+        <v>2.2965105321035613</v>
+      </c>
+      <c r="H36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37">
+        <v>0.56955904715958205</v>
+      </c>
+      <c r="C37">
+        <v>0.56969008919932784</v>
+      </c>
+      <c r="D37">
+        <v>0.56955904715958205</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="3"/>
+        <v>0.56960272783949728</v>
+      </c>
+      <c r="F37">
+        <f>E37-E$9</f>
+        <v>2.9536551612901918E-2</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="4"/>
+        <v>2.9536551612901918</v>
+      </c>
+      <c r="H37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38">
+        <v>0.33477011494252867</v>
+      </c>
+      <c r="C38">
+        <v>0.33477011494252867</v>
+      </c>
+      <c r="D38">
+        <v>0.33477011494252867</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="3"/>
+        <v>0.33477011494252867</v>
+      </c>
+      <c r="F38">
+        <f>E38-E$10</f>
+        <v>1.1433449941695706E-2</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="4"/>
+        <v>1.1433449941695706</v>
+      </c>
+      <c r="H38" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39">
+        <v>0.46551724137931028</v>
+      </c>
+      <c r="C39">
+        <v>0.46551724137931028</v>
+      </c>
+      <c r="D39">
+        <v>0.46551724137931028</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="3"/>
+        <v>0.46551724137931028</v>
+      </c>
+      <c r="F39">
+        <f>E39-E$11</f>
+        <v>-1.7016491754123064E-2</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="4"/>
+        <v>-1.7016491754123064</v>
+      </c>
+      <c r="H39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40">
+        <v>10.31293877034352</v>
+      </c>
+      <c r="C40" s="1">
+        <v>10.39542101786054</v>
+      </c>
+      <c r="D40">
+        <v>9.8157314329311767</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="3"/>
+        <v>10.174697073711746</v>
+      </c>
+      <c r="F40">
+        <f>E40-E$12</f>
+        <v>-5.1988837456298036</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>19</v>
+      </c>
+      <c r="I43" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>1500</v>
+      </c>
+      <c r="B44">
+        <v>300</v>
+      </c>
+      <c r="C44">
+        <v>400</v>
+      </c>
+      <c r="D44">
+        <v>15</v>
+      </c>
+      <c r="I44">
+        <v>1500</v>
+      </c>
+      <c r="J44">
+        <v>300</v>
+      </c>
+      <c r="K44">
+        <v>600</v>
+      </c>
+      <c r="L44">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G45" t="s">
+        <v>14</v>
+      </c>
+      <c r="J45" t="s">
+        <v>0</v>
+      </c>
+      <c r="K45" t="s">
+        <v>1</v>
+      </c>
+      <c r="L45" t="s">
+        <v>2</v>
+      </c>
+      <c r="M45" t="s">
+        <v>3</v>
+      </c>
+      <c r="N45" t="s">
+        <v>20</v>
+      </c>
+      <c r="O45" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46">
+        <v>0.62861930998294635</v>
+      </c>
+      <c r="C46">
+        <v>0.65029679916043548</v>
+      </c>
+      <c r="D46">
+        <v>0.65322656446509653</v>
+      </c>
+      <c r="E46">
+        <f>AVERAGE(B46:D46)</f>
+        <v>0.64404755786949275</v>
+      </c>
+      <c r="F46">
+        <f>E46-$E$4</f>
+        <v>7.7979238122221073E-3</v>
+      </c>
+      <c r="G46">
+        <f>F46*100</f>
+        <v>0.77979238122221073</v>
+      </c>
+      <c r="I46" t="s">
+        <v>4</v>
+      </c>
+      <c r="J46">
+        <v>0.58116975211111632</v>
+      </c>
+      <c r="K46">
+        <v>0.60617751589973801</v>
+      </c>
+      <c r="L46">
+        <v>0.60536153891758193</v>
+      </c>
+      <c r="M46">
+        <f>AVERAGE(J46:L46)</f>
+        <v>0.59756960230947875</v>
+      </c>
+      <c r="N46">
+        <f>M46-E46</f>
+        <v>-4.6477955560013995E-2</v>
+      </c>
+      <c r="O46">
+        <f>N46*100</f>
+        <v>-4.6477955560013999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>5</v>
+      </c>
+      <c r="B47">
+        <v>0.63048029556650242</v>
+      </c>
+      <c r="C47">
+        <v>0.62315270935960587</v>
+      </c>
+      <c r="D47">
+        <v>0.6411124794745483</v>
+      </c>
+      <c r="E47">
+        <f t="shared" ref="E47:E54" si="5">AVERAGE(B47:D47)</f>
+        <v>0.63158182813355213</v>
+      </c>
+      <c r="F47">
+        <f>E47-$E$5</f>
+        <v>-6.2746662383094343E-2</v>
+      </c>
+      <c r="G47">
+        <f t="shared" ref="G47:G53" si="6">F47*100</f>
+        <v>-6.2746662383094343</v>
+      </c>
+      <c r="I47" t="s">
+        <v>5</v>
+      </c>
+      <c r="J47">
+        <v>0.60849753694581277</v>
+      </c>
+      <c r="K47">
+        <v>0.62516420361247937</v>
+      </c>
+      <c r="L47">
+        <v>0.60921592775041045</v>
+      </c>
+      <c r="M47">
+        <f t="shared" ref="M47:M54" si="7">AVERAGE(J47:L47)</f>
+        <v>0.6142925561029009</v>
+      </c>
+      <c r="N47">
+        <f t="shared" ref="N47:N54" si="8">M47-E47</f>
+        <v>-1.7289272030651226E-2</v>
+      </c>
+      <c r="O47">
+        <f t="shared" ref="O47:O53" si="9">N47*100</f>
+        <v>-1.7289272030651226</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48">
+        <v>0.64956896549431453</v>
+      </c>
+      <c r="C48">
+        <v>0.68018438694906547</v>
+      </c>
+      <c r="D48">
+        <v>0.67041427200661396</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="5"/>
+        <v>0.66672254148333143</v>
+      </c>
+      <c r="F48">
+        <f>E48-$E$6</f>
+        <v>-4.7343723967940621E-2</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="6"/>
+        <v>-4.7343723967940621</v>
+      </c>
+      <c r="I48" t="s">
+        <v>6</v>
+      </c>
+      <c r="J48">
+        <v>0.63952346741104926</v>
+      </c>
+      <c r="K48">
+        <v>0.67476053637439981</v>
+      </c>
+      <c r="L48">
+        <v>0.6631345785201086</v>
+      </c>
+      <c r="M48">
+        <f t="shared" si="7"/>
+        <v>0.65913952743518589</v>
+      </c>
+      <c r="N48">
+        <f t="shared" si="8"/>
+        <v>-7.5830140481455421E-3</v>
+      </c>
+      <c r="O48">
+        <f t="shared" si="9"/>
+        <v>-0.75830140481455421</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49">
+        <v>0.76165258772505207</v>
+      </c>
+      <c r="C49">
+        <v>0.76165258772505207</v>
+      </c>
+      <c r="D49">
+        <v>0.76165258772505207</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="5"/>
+        <v>0.76165258772505207</v>
+      </c>
+      <c r="F49">
+        <f>E49-$E$7</f>
+        <v>3.1536020671496523E-4</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="6"/>
+        <v>3.1536020671496523E-2</v>
+      </c>
+      <c r="I49" t="s">
+        <v>7</v>
+      </c>
+      <c r="J49">
+        <v>0.75484597742695825</v>
+      </c>
+      <c r="K49">
+        <v>0.75484597742695825</v>
+      </c>
+      <c r="L49">
+        <v>0.75484597742695825</v>
+      </c>
+      <c r="M49">
+        <f t="shared" si="7"/>
+        <v>0.75484597742695814</v>
+      </c>
+      <c r="N49">
+        <f t="shared" si="8"/>
+        <v>-6.8066102980939291E-3</v>
+      </c>
+      <c r="O49">
+        <f t="shared" si="9"/>
+        <v>-0.68066102980939291</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>8</v>
+      </c>
+      <c r="B50">
+        <v>0.12228882773438179</v>
+      </c>
+      <c r="C50">
+        <v>0.130548145035601</v>
+      </c>
+      <c r="D50">
+        <v>0.1235946086697287</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="5"/>
+        <v>0.12547719381323716</v>
+      </c>
+      <c r="F50">
+        <f>E50-$E$8</f>
+        <v>6.5121645626330799E-3</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="6"/>
+        <v>0.65121645626330804</v>
+      </c>
+      <c r="I50" t="s">
+        <v>8</v>
+      </c>
+      <c r="J50">
+        <v>0.12039097349345269</v>
+      </c>
+      <c r="K50">
+        <v>0.1208664797934889</v>
+      </c>
+      <c r="L50">
+        <v>0.1127508406541232</v>
+      </c>
+      <c r="M50">
+        <f t="shared" si="7"/>
+        <v>0.1180027646470216</v>
+      </c>
+      <c r="N50">
+        <f t="shared" si="8"/>
+        <v>-7.4744291662155599E-3</v>
+      </c>
+      <c r="O50">
+        <f t="shared" si="9"/>
+        <v>-0.74744291662155593</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51">
+        <v>0.53661076583489509</v>
+      </c>
+      <c r="C51">
+        <v>0.53599105026958216</v>
+      </c>
+      <c r="D51">
+        <v>0.53583428166634284</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="5"/>
+        <v>0.53614536592360673</v>
+      </c>
+      <c r="F51">
+        <f>E51-$E$9</f>
+        <v>-3.920810302988631E-3</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="6"/>
+        <v>-0.3920810302988631</v>
+      </c>
+      <c r="I51" t="s">
+        <v>9</v>
+      </c>
+      <c r="J51">
+        <v>0.54799313232763169</v>
+      </c>
+      <c r="K51">
+        <v>0.55503114084071004</v>
+      </c>
+      <c r="L51">
+        <v>0.55535068561869882</v>
+      </c>
+      <c r="M51">
+        <f t="shared" si="7"/>
+        <v>0.55279165292901355</v>
+      </c>
+      <c r="N51">
+        <f t="shared" si="8"/>
+        <v>1.6646287005406823E-2</v>
+      </c>
+      <c r="O51">
+        <f t="shared" si="9"/>
+        <v>1.6646287005406823</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>10</v>
+      </c>
+      <c r="B52">
+        <v>0.32241379310344831</v>
+      </c>
+      <c r="C52">
+        <v>0.32241379310344831</v>
+      </c>
+      <c r="D52">
+        <v>0.31379310344827582</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="5"/>
+        <v>0.31954022988505748</v>
+      </c>
+      <c r="F52">
+        <f>E52-$E$10</f>
+        <v>-3.7964351157754872E-3</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="6"/>
+        <v>-0.37964351157754872</v>
+      </c>
+      <c r="I52" t="s">
+        <v>10</v>
+      </c>
+      <c r="J52">
+        <v>0.31422413793103449</v>
+      </c>
+      <c r="K52">
+        <v>0.32284482758620692</v>
+      </c>
+      <c r="L52">
+        <v>0.31853448275862067</v>
+      </c>
+      <c r="M52">
+        <f t="shared" si="7"/>
+        <v>0.31853448275862073</v>
+      </c>
+      <c r="N52">
+        <f t="shared" si="8"/>
+        <v>-1.0057471264367512E-3</v>
+      </c>
+      <c r="O52">
+        <f t="shared" si="9"/>
+        <v>-0.10057471264367512</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53">
+        <v>0.43103448275862072</v>
+      </c>
+      <c r="C53">
+        <v>0.43103448275862072</v>
+      </c>
+      <c r="D53">
+        <v>0.42241379310344829</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="5"/>
+        <v>0.42816091954022989</v>
+      </c>
+      <c r="F53">
+        <f>E53-$E$11</f>
+        <v>-5.4372813593203451E-2</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="6"/>
+        <v>-5.4372813593203446</v>
+      </c>
+      <c r="I53" t="s">
+        <v>11</v>
+      </c>
+      <c r="J53">
+        <v>0.42241379310344829</v>
+      </c>
+      <c r="K53">
+        <v>0.43103448275862072</v>
+      </c>
+      <c r="L53">
+        <v>0.42241379310344829</v>
+      </c>
+      <c r="M53">
+        <f t="shared" si="7"/>
+        <v>0.42528735632183912</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="8"/>
+        <v>-2.8735632183907733E-3</v>
+      </c>
+      <c r="O53">
+        <f t="shared" si="9"/>
+        <v>-0.28735632183907733</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54">
+        <v>11.24697343028825</v>
+      </c>
+      <c r="C54" s="1">
+        <v>10.637627139173709</v>
+      </c>
+      <c r="D54">
+        <v>11.093879611327729</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="5"/>
+        <v>10.992826726929897</v>
+      </c>
+      <c r="F54">
+        <f>E54-$E$12</f>
+        <v>-4.380754092411653</v>
+      </c>
+      <c r="I54" t="s">
+        <v>12</v>
+      </c>
+      <c r="J54">
+        <v>10.782622464771929</v>
+      </c>
+      <c r="K54" s="1">
+        <v>10.95228897086505</v>
+      </c>
+      <c r="L54">
+        <v>11.172789222207561</v>
+      </c>
+      <c r="M54">
+        <f t="shared" si="7"/>
+        <v>10.969233552614847</v>
+      </c>
+      <c r="N54">
+        <f t="shared" si="8"/>
+        <v>-2.3593174315049481E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>1500</v>
+      </c>
+      <c r="B57">
+        <v>300</v>
+      </c>
+      <c r="C57">
+        <v>400</v>
+      </c>
+      <c r="D57">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>0</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1</v>
+      </c>
+      <c r="D58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F58" t="s">
+        <v>20</v>
+      </c>
+      <c r="G58" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>4</v>
+      </c>
+      <c r="B59">
+        <v>0.61555959331188681</v>
+      </c>
+      <c r="C59">
+        <v>0.65158730158730149</v>
+      </c>
+      <c r="D59">
+        <v>0.65265971402335043</v>
+      </c>
+      <c r="E59">
+        <f>AVERAGE(B59:D59)</f>
+        <v>0.63993553630751299</v>
+      </c>
+      <c r="F59">
+        <f>E59-E$4</f>
+        <v>3.6859022502423455E-3</v>
+      </c>
+      <c r="G59">
+        <f>F59*100</f>
+        <v>0.36859022502423455</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>5</v>
+      </c>
+      <c r="B60">
+        <v>0.67097701149425282</v>
+      </c>
+      <c r="C60">
+        <v>0.66939655172413781</v>
+      </c>
+      <c r="D60">
+        <v>0.67054597701149421</v>
+      </c>
+      <c r="E60">
+        <f t="shared" ref="E60:E67" si="10">AVERAGE(B60:D60)</f>
+        <v>0.67030651340996161</v>
+      </c>
+      <c r="F60">
+        <f>E60-E$5</f>
+        <v>-2.4021977106684855E-2</v>
+      </c>
+      <c r="G60">
+        <f t="shared" ref="G60:G66" si="11">F60*100</f>
+        <v>-2.4021977106684855</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61">
+        <v>0.64281400963976165</v>
+      </c>
+      <c r="C61">
+        <v>0.65427536229576322</v>
+      </c>
+      <c r="D61">
+        <v>0.65949473177800511</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="10"/>
+        <v>0.65219470123784329</v>
+      </c>
+      <c r="F61">
+        <f>E61-E$6</f>
+        <v>-6.1871564213428765E-2</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="11"/>
+        <v>-6.1871564213428769</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62">
+        <v>0.76950864952882647</v>
+      </c>
+      <c r="C62">
+        <v>0.7707857655317053</v>
+      </c>
+      <c r="D62">
+        <v>0.77190141442109028</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="10"/>
+        <v>0.77073194316054072</v>
+      </c>
+      <c r="F62">
+        <f>E62-E$7</f>
+        <v>9.3947156422036215E-3</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="11"/>
+        <v>0.93947156422036215</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>8</v>
+      </c>
+      <c r="B63">
+        <v>0.11081178003243131</v>
+      </c>
+      <c r="C63">
+        <v>0.122654639095896</v>
+      </c>
+      <c r="D63">
+        <v>0.1153495195865346</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="10"/>
+        <v>0.11627197957162062</v>
+      </c>
+      <c r="F63">
+        <f>E63-E$8</f>
+        <v>-2.6930496789834557E-3</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="11"/>
+        <v>-0.26930496789834557</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>9</v>
+      </c>
+      <c r="B64">
+        <v>0.60866933546773316</v>
+      </c>
+      <c r="C64">
+        <v>0.59323477226513066</v>
+      </c>
+      <c r="D64">
+        <v>0.56796815813713286</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="10"/>
+        <v>0.58995742195666556</v>
+      </c>
+      <c r="F64">
+        <f>E64-E$9</f>
+        <v>4.9891245730070199E-2</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="11"/>
+        <v>4.9891245730070199</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>10</v>
+      </c>
+      <c r="B65">
+        <v>0.28893678160919539</v>
+      </c>
+      <c r="C65">
+        <v>0.28864942528735632</v>
+      </c>
+      <c r="D65">
+        <v>0.30373563218390798</v>
+      </c>
+      <c r="E65">
+        <f t="shared" si="10"/>
+        <v>0.29377394636015325</v>
+      </c>
+      <c r="F65">
+        <f>E65-E$10</f>
+        <v>-2.9562718640679719E-2</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="11"/>
+        <v>-2.9562718640679719</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>11</v>
+      </c>
+      <c r="B66">
+        <v>0.44827586206896552</v>
+      </c>
+      <c r="C66">
+        <v>0.43103448275862072</v>
+      </c>
+      <c r="D66">
+        <v>0.44827586206896552</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="10"/>
+        <v>0.44252873563218392</v>
+      </c>
+      <c r="F66">
+        <f>E66-E$11</f>
+        <v>-4.0004997501249417E-2</v>
+      </c>
+      <c r="G66">
+        <f t="shared" si="11"/>
+        <v>-4.0004997501249413</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67">
+        <v>37.130805184101227</v>
+      </c>
+      <c r="C67" s="1">
+        <v>12.481576933942989</v>
+      </c>
+      <c r="D67">
+        <v>12.33926722099041</v>
+      </c>
+      <c r="E67">
+        <f t="shared" si="10"/>
+        <v>20.650549779678208</v>
+      </c>
+      <c r="F67">
+        <f>E67-E$12</f>
+        <v>5.2769689603366583</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C64D6A0-67B0-420F-B472-231F769BBEC3}">
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1500</v>
+      </c>
+      <c r="B2">
+        <v>300</v>
+      </c>
+      <c r="C2">
+        <v>400</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0.63351272621184107</v>
+      </c>
+      <c r="C4">
+        <v>0.62602869107293879</v>
+      </c>
+      <c r="D4">
+        <v>0.63562295404400659</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E12" si="0">AVERAGE(B4:D4)</f>
+        <v>0.63172145710959549</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0.63060344827586212</v>
+      </c>
+      <c r="C5">
+        <v>0.62227011494252882</v>
+      </c>
+      <c r="D5">
+        <v>0.63376436781609191</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>0.62887931034482758</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>0.70974637678520747</v>
+      </c>
+      <c r="C6">
+        <v>0.72195652171092872</v>
+      </c>
+      <c r="D6">
+        <v>0.7130268198961851</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.71490990613077388</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="C7">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="D7">
+        <v>0.76006157871638313</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.76006157871638313</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>0.14863753589118131</v>
+      </c>
+      <c r="C8">
+        <v>0.14382413673605429</v>
+      </c>
+      <c r="D8">
+        <v>0.15017526964578171</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0.14754564742433909</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>0.5552812872194981</v>
+      </c>
+      <c r="C9">
+        <v>0.55531351804635143</v>
+      </c>
+      <c r="D9">
+        <v>0.55530281878956966</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0.55529920801847299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>0.36206896551724138</v>
+      </c>
+      <c r="C10">
+        <v>0.35344827586206901</v>
+      </c>
+      <c r="D10">
+        <v>0.35344827586206901</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0.35632183908045983</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="C11">
+        <v>0.5</v>
+      </c>
+      <c r="D11">
+        <v>0.5</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0.50287356321839083</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>11.19616421337785</v>
+      </c>
+      <c r="C12" s="1">
+        <v>11.108016953386111</v>
+      </c>
+      <c r="D12">
+        <v>10.89680967659786</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>11.066996947787274</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1500</v>
+      </c>
+      <c r="B16">
+        <v>300</v>
+      </c>
+      <c r="C16">
+        <v>500</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.59221648557931739</v>
+      </c>
+      <c r="C18">
+        <v>0.59493776204302518</v>
+      </c>
+      <c r="D18">
+        <v>0.61003051529367314</v>
+      </c>
+      <c r="E18">
+        <f t="shared" ref="E18:E26" si="1">AVERAGE(B18:D18)</f>
+        <v>0.5990615876386719</v>
+      </c>
+      <c r="F18">
+        <f>E18-E$4</f>
+        <v>-3.2659869470923586E-2</v>
+      </c>
+      <c r="G18">
+        <f>F18*100</f>
+        <v>-3.2659869470923586</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.61408045977011494</v>
+      </c>
+      <c r="C19">
+        <v>0.64928160919540223</v>
+      </c>
+      <c r="D19">
+        <v>0.64382183908045965</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>0.63572796934865894</v>
+      </c>
+      <c r="F19">
+        <f>E19-E$5</f>
+        <v>6.8486590038313588E-3</v>
+      </c>
+      <c r="G19">
+        <f t="shared" ref="G19:G25" si="2">F19*100</f>
+        <v>0.68486590038313588</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0.70400966180911884</v>
+      </c>
+      <c r="C20">
+        <v>0.71094348656380024</v>
+      </c>
+      <c r="D20">
+        <v>0.70604645591214499</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>0.70699986809502136</v>
+      </c>
+      <c r="F20">
+        <f>E20-E$6</f>
+        <v>-7.9100380357525202E-3</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="2"/>
+        <v>-0.79100380357525202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="4">
+        <v>0.7560400178544624</v>
+      </c>
+      <c r="C21">
+        <v>0.7560400178544624</v>
+      </c>
+      <c r="D21">
+        <v>0.7560400178544624</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>0.7560400178544624</v>
+      </c>
+      <c r="F21">
+        <f>E21-E$7</f>
+        <v>-4.0215608619207366E-3</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="2"/>
+        <v>-0.40215608619207366</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="4">
+        <v>0.13995621720847409</v>
+      </c>
+      <c r="C22">
+        <v>0.1411203399061548</v>
+      </c>
+      <c r="D22">
+        <v>0.1494549052335897</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>0.1435104874494062</v>
+      </c>
+      <c r="F22">
+        <f>E22-E$8</f>
+        <v>-4.0351599749328948E-3</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="2"/>
+        <v>-0.40351599749328948</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="4">
+        <v>0.55506857152178457</v>
+      </c>
+      <c r="C23">
+        <v>0.55503634069493146</v>
+      </c>
+      <c r="D23">
+        <v>0.55506857152178457</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>0.55505782791283353</v>
+      </c>
+      <c r="F23">
+        <f>E23-E$9</f>
+        <v>-2.4138010563945489E-4</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="2"/>
+        <v>-2.4138010563945489E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="4">
+        <v>0.31867816091954032</v>
+      </c>
+      <c r="C24">
+        <v>0.33160919540229888</v>
+      </c>
+      <c r="D24">
+        <v>0.3445402298850575</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>0.33160919540229888</v>
+      </c>
+      <c r="F24">
+        <f>E24-E$10</f>
+        <v>-2.471264367816095E-2</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="2"/>
+        <v>-2.471264367816095</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.45689655172413801</v>
+      </c>
+      <c r="C25">
+        <v>0.46551724137931028</v>
+      </c>
+      <c r="D25">
+        <v>0.48275862068965519</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="1"/>
+        <v>0.46839080459770116</v>
+      </c>
+      <c r="F25">
+        <f>E25-E$11</f>
+        <v>-3.4482758620689669E-2</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="2"/>
+        <v>-3.4482758620689671</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="4">
+        <v>11.706257104873661</v>
+      </c>
+      <c r="C26" s="1">
+        <v>10.99899522189436</v>
+      </c>
+      <c r="D26">
+        <v>11.138804086323439</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="1"/>
+        <v>11.281352137697153</v>
+      </c>
+      <c r="F26">
+        <f>E26-E$12</f>
+        <v>0.21435518990987923</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>1500</v>
+      </c>
+      <c r="B30">
+        <v>300</v>
+      </c>
+      <c r="C30">
+        <v>600</v>
+      </c>
+      <c r="D30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32">
+        <v>0.58637347500983861</v>
+      </c>
+      <c r="C32" s="4">
+        <v>0.58366840866840863</v>
+      </c>
+      <c r="D32">
+        <v>0.58937131050767411</v>
+      </c>
+      <c r="E32">
+        <f t="shared" ref="E32:E40" si="3">AVERAGE(C32:D32)</f>
+        <v>0.58651985958804143</v>
+      </c>
+      <c r="F32">
+        <f>E32-E$4</f>
+        <v>-4.520159752155406E-2</v>
+      </c>
+      <c r="G32">
+        <f>F32*100</f>
+        <v>-4.520159752155406</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33">
+        <v>0.62635467980295567</v>
+      </c>
+      <c r="C33" s="4">
+        <v>0.62943349753694577</v>
+      </c>
+      <c r="D33">
+        <v>0.61988916256157633</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="3"/>
+        <v>0.62466133004926105</v>
+      </c>
+      <c r="F33">
+        <f>E33-E$5</f>
+        <v>-4.2179802955665258E-3</v>
+      </c>
+      <c r="G33">
+        <f t="shared" ref="G33:G39" si="4">F33*100</f>
+        <v>-0.42179802955665258</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34">
+        <v>0.70331384013056886</v>
+      </c>
+      <c r="C34" s="4">
+        <v>0.71747584538549414</v>
+      </c>
+      <c r="D34">
+        <v>0.70080409354121465</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="3"/>
+        <v>0.70913996946335445</v>
+      </c>
+      <c r="F34">
+        <f>E34-E$6</f>
+        <v>-5.7699366674194286E-3</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="4"/>
+        <v>-0.57699366674194286</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35">
+        <v>0.76039935416643756</v>
+      </c>
+      <c r="C35" s="4">
+        <v>0.76039935416643756</v>
+      </c>
+      <c r="D35">
+        <v>0.76039935416643756</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="3"/>
+        <v>0.76039935416643756</v>
+      </c>
+      <c r="F35">
+        <f>E35-E$7</f>
+        <v>3.3777545005442278E-4</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="4"/>
+        <v>3.3777545005442278E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36">
+        <v>0.123175505660665</v>
+      </c>
+      <c r="C36" s="4">
+        <v>0.13378200496323939</v>
+      </c>
+      <c r="D36">
+        <v>0.1391438137885227</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="3"/>
+        <v>0.13646290937588104</v>
+      </c>
+      <c r="F36">
+        <f>E36-E$8</f>
+        <v>-1.1082738048458052E-2</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="4"/>
+        <v>-1.1082738048458052</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37">
+        <v>0.55192605413259055</v>
+      </c>
+      <c r="C37" s="4">
+        <v>0.55189382330573733</v>
+      </c>
+      <c r="D37">
+        <v>0.551859992206436</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="3"/>
+        <v>0.55187690775608667</v>
+      </c>
+      <c r="F37">
+        <f>E37-E$9</f>
+        <v>-3.4223002623863241E-3</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="4"/>
+        <v>-0.34223002623863241</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38">
+        <v>0.31264367816091948</v>
+      </c>
+      <c r="C38" s="4">
+        <v>0.31264367816091948</v>
+      </c>
+      <c r="D38">
+        <v>0.32557471264367821</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="3"/>
+        <v>0.31910919540229887</v>
+      </c>
+      <c r="F38">
+        <f>E38-E$10</f>
+        <v>-3.7212643678160962E-2</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="4"/>
+        <v>-3.7212643678160964</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39">
+        <v>0.43965517241379309</v>
+      </c>
+      <c r="C39" s="4">
+        <v>0.43965517241379309</v>
+      </c>
+      <c r="D39">
+        <v>0.45689655172413801</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="3"/>
+        <v>0.44827586206896552</v>
+      </c>
+      <c r="F39">
+        <f>E39-E$11</f>
+        <v>-5.4597701149425304E-2</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="4"/>
+        <v>-5.4597701149425308</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40">
+        <v>11.802332791788819</v>
+      </c>
+      <c r="C40" s="4">
+        <v>11.505953823697981</v>
+      </c>
+      <c r="D40">
+        <v>10.9318431841916</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="3"/>
+        <v>11.218898503944789</v>
+      </c>
+      <c r="F40">
+        <f>E40-E$12</f>
+        <v>0.15190155615751522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results: adding new files
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Zwischenstand.xlsx
+++ b/src/evaluation/data/Zwischenstand.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A751634-B774-4CAA-B635-6306AAEABAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38FD6E6-4BDD-4FB9-9C45-085677519544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="2" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="naive max_size" sheetId="1" r:id="rId1"/>
-    <sheet name="naive overlap" sheetId="2" r:id="rId2"/>
-    <sheet name="semantic percentile" sheetId="3" r:id="rId3"/>
-    <sheet name="semantic min_size" sheetId="4" r:id="rId4"/>
+    <sheet name="gpt_naive max_size" sheetId="5" r:id="rId2"/>
+    <sheet name="naive overlap" sheetId="2" r:id="rId3"/>
+    <sheet name="semantic percentile" sheetId="3" r:id="rId4"/>
+    <sheet name="semantic min_size" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="21">
   <si>
     <t>run1</t>
   </si>
@@ -1567,6 +1568,902 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0763B57-AFAE-4268-833F-1978FDE50B6B}">
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>1000</v>
+      </c>
+      <c r="B1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="2" t="e">
+        <f>AVERAGE(B3:D3)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="e">
+        <f t="shared" ref="E4:E11" si="0">AVERAGE(B4:D4)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="2" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1250</v>
+      </c>
+      <c r="B13">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>0.69945357716701795</v>
+      </c>
+      <c r="C15">
+        <v>0.6795021277889991</v>
+      </c>
+      <c r="D15">
+        <v>0.69120162991966927</v>
+      </c>
+      <c r="E15">
+        <f>AVERAGE(B15:D15)</f>
+        <v>0.69005244495856211</v>
+      </c>
+      <c r="F15" t="e">
+        <f>E15-$E$3</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G15" t="e">
+        <f>F15*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>0.61134057971014499</v>
+      </c>
+      <c r="C16">
+        <v>0.60628591954023003</v>
+      </c>
+      <c r="D16">
+        <v>0.62047413793103456</v>
+      </c>
+      <c r="E16">
+        <f t="shared" ref="E16:E23" si="1">AVERAGE(B16:D16)</f>
+        <v>0.61270021239380312</v>
+      </c>
+      <c r="F16" t="e">
+        <f>E16-$E$4</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G16" t="e">
+        <f t="shared" ref="G16:G22" si="2">F16*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17">
+        <v>0.57977828743671855</v>
+      </c>
+      <c r="C17">
+        <v>0.5693366857997334</v>
+      </c>
+      <c r="D17">
+        <v>0.58335727966791828</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="1"/>
+        <v>0.57749075096812341</v>
+      </c>
+      <c r="F17" t="e">
+        <f>E17-$E$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G17" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18">
+        <v>0.76445431250814044</v>
+      </c>
+      <c r="C18">
+        <v>0.76445431250814044</v>
+      </c>
+      <c r="D18">
+        <v>0.76394038159581756</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>0.76428300220403278</v>
+      </c>
+      <c r="F18" t="e">
+        <f>E18-$E$6</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G18" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19">
+        <v>0.25233225683849669</v>
+      </c>
+      <c r="C19">
+        <v>0.25233470207780773</v>
+      </c>
+      <c r="D19">
+        <v>0.25556369724652522</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>0.25341021872094321</v>
+      </c>
+      <c r="F19" t="e">
+        <f>E19-$E$7</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G19" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20">
+        <v>0.62712365568616846</v>
+      </c>
+      <c r="C20">
+        <v>0.60685930765855134</v>
+      </c>
+      <c r="D20">
+        <v>0.59911507491363925</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>0.61103267941945294</v>
+      </c>
+      <c r="F20" t="e">
+        <f>E20-$E$8</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G20" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>0.33721264367816078</v>
+      </c>
+      <c r="C21">
+        <v>0.32859195402298852</v>
+      </c>
+      <c r="D21">
+        <v>0.33721264367816078</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>0.33433908045977007</v>
+      </c>
+      <c r="F21" t="e">
+        <f>E21-$E$9</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G21" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>0.48275862068965519</v>
+      </c>
+      <c r="C22">
+        <v>0.47413793103448282</v>
+      </c>
+      <c r="D22">
+        <v>0.48275862068965519</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>0.47988505747126436</v>
+      </c>
+      <c r="F22" t="e">
+        <f>E22-$E$10</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G22" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="1">
+        <v>11.411141514778141</v>
+      </c>
+      <c r="C23">
+        <v>11.46074738584716</v>
+      </c>
+      <c r="D23">
+        <v>12.08357310089572</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>11.651820667173673</v>
+      </c>
+      <c r="F23" t="e">
+        <f>E23-$E$11</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>1500</v>
+      </c>
+      <c r="B25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27">
+        <v>0.66156887149880883</v>
+      </c>
+      <c r="C27">
+        <v>0.64893983549723111</v>
+      </c>
+      <c r="D27">
+        <v>0.67855384785151807</v>
+      </c>
+      <c r="E27">
+        <f>AVERAGE(B27:D27)</f>
+        <v>0.66302085161585267</v>
+      </c>
+      <c r="F27" t="e">
+        <f>E27-$E$3</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G27" t="e">
+        <f>F27*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28">
+        <v>0.62444581280788181</v>
+      </c>
+      <c r="C28">
+        <v>0.63594006568144501</v>
+      </c>
+      <c r="D28">
+        <v>0.6361076604554865</v>
+      </c>
+      <c r="E28">
+        <f t="shared" ref="E28:E35" si="3">AVERAGE(B28:D28)</f>
+        <v>0.63216451298160448</v>
+      </c>
+      <c r="F28" t="e">
+        <f>E28-$E$4</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G28" t="e">
+        <f t="shared" ref="G28:G34" si="4">F28*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29">
+        <v>0.62411398464630641</v>
+      </c>
+      <c r="C29">
+        <v>0.63705699230932189</v>
+      </c>
+      <c r="D29">
+        <v>0.6270169081827085</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="3"/>
+        <v>0.6293959617127789</v>
+      </c>
+      <c r="F29" t="e">
+        <f>E29-$E$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G29" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30">
+        <v>0.75828297912577958</v>
+      </c>
+      <c r="C30">
+        <v>0.75921113559346654</v>
+      </c>
+      <c r="D30">
+        <v>0.76194123225598731</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="3"/>
+        <v>0.75981178232507796</v>
+      </c>
+      <c r="F30" t="e">
+        <f>E30-$E$6</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G30" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31">
+        <v>0.27292447328324371</v>
+      </c>
+      <c r="C31">
+        <v>0.26747226671678082</v>
+      </c>
+      <c r="D31">
+        <v>0.27978722808894241</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="3"/>
+        <v>0.27339465602965562</v>
+      </c>
+      <c r="F31" t="e">
+        <f>E31-$E$7</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G31" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32">
+        <v>0.59892572244511921</v>
+      </c>
+      <c r="C32">
+        <v>0.59085822927043607</v>
+      </c>
+      <c r="D32">
+        <v>0.63535731636781256</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="3"/>
+        <v>0.60838042269445591</v>
+      </c>
+      <c r="F32" t="e">
+        <f>E32-$E$8</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G32" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33">
+        <v>0.3466954022988506</v>
+      </c>
+      <c r="C33">
+        <v>0.34885057471264369</v>
+      </c>
+      <c r="D33">
+        <v>0.3603448275862069</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="3"/>
+        <v>0.35196360153256706</v>
+      </c>
+      <c r="F33" t="e">
+        <f>E33-$E$9</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G33" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="C34">
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="D34">
+        <v>0.52586206896551724</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="3"/>
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="F34" t="e">
+        <f>E34-$E$10</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G34" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35">
+        <v>12.829803801816089</v>
+      </c>
+      <c r="C35" s="1">
+        <v>13.84695393052594</v>
+      </c>
+      <c r="D35">
+        <v>12.0599361699203</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="3"/>
+        <v>12.91223130075411</v>
+      </c>
+      <c r="F35" t="e">
+        <f>E35-$E$11</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>1750</v>
+      </c>
+      <c r="B39">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1</v>
+      </c>
+      <c r="D40" t="s">
+        <v>2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41">
+        <v>0.62963137009189651</v>
+      </c>
+      <c r="C41">
+        <v>0.62900901409001886</v>
+      </c>
+      <c r="D41">
+        <v>0.64225496854746966</v>
+      </c>
+      <c r="E41">
+        <f>AVERAGE(B41:D41)</f>
+        <v>0.63363178424312838</v>
+      </c>
+      <c r="F41" s="2" t="e">
+        <f>E41-$E$3</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G41" t="e">
+        <f>F41*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42">
+        <v>0.6554187192118226</v>
+      </c>
+      <c r="C42">
+        <v>0.656568144499179</v>
+      </c>
+      <c r="D42">
+        <v>0.69250208855472017</v>
+      </c>
+      <c r="E42">
+        <f t="shared" ref="E42:E49" si="5">AVERAGE(B42:D42)</f>
+        <v>0.66816298408857389</v>
+      </c>
+      <c r="F42" s="2" t="e">
+        <f>E42-$E$4</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G42" t="e">
+        <f t="shared" ref="G42:G48" si="6">F42*100</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>0.58686542143005738</v>
+      </c>
+      <c r="C43">
+        <v>0.61296695399601808</v>
+      </c>
+      <c r="D43">
+        <v>0.62757201643333771</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="5"/>
+        <v>0.60913479728647102</v>
+      </c>
+      <c r="F43" s="2" t="e">
+        <f>E43-$E$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G43" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44">
+        <v>0.75326889799614516</v>
+      </c>
+      <c r="C44">
+        <v>0.7523646340895267</v>
+      </c>
+      <c r="D44">
+        <v>0.75326889799614516</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="5"/>
+        <v>0.75296747669393904</v>
+      </c>
+      <c r="F44" s="2" t="e">
+        <f>E44-$E$6</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G44" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>8</v>
+      </c>
+      <c r="B45">
+        <v>0.24553750941061361</v>
+      </c>
+      <c r="C45">
+        <v>0.26164240439793229</v>
+      </c>
+      <c r="D45">
+        <v>0.2483463938670056</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="5"/>
+        <v>0.25184210255851719</v>
+      </c>
+      <c r="F45" s="2" t="e">
+        <f>E45-$E$7</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G45" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46">
+        <v>0.60933495101680679</v>
+      </c>
+      <c r="C46">
+        <v>0.63147614145716247</v>
+      </c>
+      <c r="D46">
+        <v>0.62695548999659645</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="5"/>
+        <v>0.62258886082352183</v>
+      </c>
+      <c r="F46" s="2" t="e">
+        <f>E46-$E$8</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G46" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47">
+        <v>0.26307471264367821</v>
+      </c>
+      <c r="C47">
+        <v>0.25445402298850572</v>
+      </c>
+      <c r="D47">
+        <v>0.26307471264367821</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="5"/>
+        <v>0.26020114942528738</v>
+      </c>
+      <c r="F47" s="2" t="e">
+        <f>E47-$E$9</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G47" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48">
+        <v>0.41379310344827591</v>
+      </c>
+      <c r="C48">
+        <v>0.40517241379310343</v>
+      </c>
+      <c r="D48">
+        <v>0.41379310344827591</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="5"/>
+        <v>0.41091954022988508</v>
+      </c>
+      <c r="F48" s="2" t="e">
+        <f>E48-$E$10</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G48" t="e">
+        <f t="shared" si="6"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="1">
+        <v>11.927592316578171</v>
+      </c>
+      <c r="C49" s="1">
+        <v>11.35648157267735</v>
+      </c>
+      <c r="D49">
+        <v>11.18512282289308</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="5"/>
+        <v>11.489732237382867</v>
+      </c>
+      <c r="F49" s="2" t="e">
+        <f>E49-$E$11</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718267C3-91F6-4352-B487-1EEB3C8D4A90}">
   <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2321,7 +3218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C2C1CF-AF99-4FC0-A37D-09071864ECF5}">
   <dimension ref="A1:O67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3883,7 +4780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C64D6A0-67B0-420F-B472-231F769BBEC3}">
   <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Results: erste Ergebnisse advanced-setup
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Zwischenstand.xlsx
+++ b/src/evaluation/data/Zwischenstand.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C113B8C-E8A2-4B2A-BB82-71962342467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45A46EC-D076-462F-BCC3-0B067E39E460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="7" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="12" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="naive max_size" sheetId="1" state="hidden" r:id="rId1"/>
@@ -25,7 +25,8 @@
     <sheet name="gpt_hybrid" sheetId="12" r:id="rId10"/>
     <sheet name="gpt_context-window" sheetId="11" r:id="rId11"/>
     <sheet name="gpt_deduplication" sheetId="9" r:id="rId12"/>
-    <sheet name="semantic min_size" sheetId="4" state="hidden" r:id="rId13"/>
+    <sheet name="Advanced" sheetId="14" r:id="rId13"/>
+    <sheet name="semantic min_size" sheetId="4" state="hidden" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="59">
   <si>
     <t>run1</t>
   </si>
@@ -213,6 +214,18 @@
   </si>
   <si>
     <t>lokal</t>
+  </si>
+  <si>
+    <t>advanced</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>Durchschnitt</t>
+  </si>
+  <si>
+    <t>Differenz zu advanced-voyage</t>
   </si>
 </sst>
 </file>
@@ -5671,6 +5684,2363 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2812793-DBB4-41C8-A6C8-004B2B5D4FF1}">
+  <dimension ref="A1:U55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1">
+        <v>1500</v>
+      </c>
+      <c r="C1">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>0.66156887149880894</v>
+      </c>
+      <c r="C3">
+        <v>0.64893983549723122</v>
+      </c>
+      <c r="D3">
+        <v>0.67855384785151796</v>
+      </c>
+      <c r="E3">
+        <f>AVERAGE(B3:D3)</f>
+        <v>0.66302085161585278</v>
+      </c>
+      <c r="G3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>0.72093318610841095</v>
+      </c>
+      <c r="I3">
+        <v>0.72920821290496773</v>
+      </c>
+      <c r="J3">
+        <v>0.74600730940974624</v>
+      </c>
+      <c r="K3">
+        <f>AVERAGE(H3:J3)</f>
+        <v>0.73204956947437505</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>0.62444581280788181</v>
+      </c>
+      <c r="C4">
+        <v>0.6359400656814449</v>
+      </c>
+      <c r="D4">
+        <v>0.63349753694581279</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E17" si="0">AVERAGE(B4:D4)</f>
+        <v>0.63129447181171316</v>
+      </c>
+      <c r="G4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>0.80114942528735633</v>
+      </c>
+      <c r="I4">
+        <v>0.79784482758620701</v>
+      </c>
+      <c r="J4">
+        <v>0.80158045977011516</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:K17" si="1">AVERAGE(H4:J4)</f>
+        <v>0.80019157088122617</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>0.62411398464630674</v>
+      </c>
+      <c r="C5">
+        <v>0.63705699230932178</v>
+      </c>
+      <c r="D5">
+        <v>0.63023227966371942</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>0.63046775220644935</v>
+      </c>
+      <c r="G5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>0.82098898464300618</v>
+      </c>
+      <c r="I5">
+        <v>0.82521551720923469</v>
+      </c>
+      <c r="J5">
+        <v>0.81385296931803208</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="1"/>
+        <v>0.82001915705675765</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>0.75927595016951388</v>
+      </c>
+      <c r="C6">
+        <v>0.75921113559346654</v>
+      </c>
+      <c r="D6">
+        <v>0.7619412322559872</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.76014277267298924</v>
+      </c>
+      <c r="G6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6">
+        <v>0.77957780726490122</v>
+      </c>
+      <c r="I6">
+        <v>0.77957780726490122</v>
+      </c>
+      <c r="J6">
+        <v>0.77776832922414518</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="1"/>
+        <v>0.77897464791798254</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>0.27292447328324371</v>
+      </c>
+      <c r="C7">
+        <v>0.27091359774604223</v>
+      </c>
+      <c r="D7">
+        <v>0.27978722808894224</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.27454176637274275</v>
+      </c>
+      <c r="G7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <v>0.33484660455304061</v>
+      </c>
+      <c r="I7">
+        <v>0.32623183411420348</v>
+      </c>
+      <c r="J7">
+        <v>0.344758727709434</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="1"/>
+        <v>0.33527905545889269</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>0.59892572244511921</v>
+      </c>
+      <c r="C8">
+        <v>0.59085822927043607</v>
+      </c>
+      <c r="D8">
+        <v>0.63535731636781256</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0.60838042269445591</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8">
+        <v>0.5978723254348659</v>
+      </c>
+      <c r="I8">
+        <v>0.60885923528497021</v>
+      </c>
+      <c r="J8">
+        <v>0.62617798594169338</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="1"/>
+        <v>0.61096984888717654</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>0.24309878051280981</v>
+      </c>
+      <c r="C9">
+        <v>0.23840367794036871</v>
+      </c>
+      <c r="D9">
+        <v>0.24638800323009491</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0.24263015389442447</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9">
+        <v>0.26685631275177002</v>
+      </c>
+      <c r="I9">
+        <v>0.26685631275177002</v>
+      </c>
+      <c r="J9">
+        <v>0.27435976266860962</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="1"/>
+        <v>0.26935746272404987</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>0.19543476402759549</v>
+      </c>
+      <c r="C10">
+        <v>0.18611909449100489</v>
+      </c>
+      <c r="D10">
+        <v>0.19965597987174991</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0.19373661279678342</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10">
+        <v>0.21834114193916321</v>
+      </c>
+      <c r="I10">
+        <v>0.21834114193916321</v>
+      </c>
+      <c r="J10">
+        <v>0.2285752147436142</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="1"/>
+        <v>0.22175249954064688</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11">
+        <v>0.29144790768623352</v>
+      </c>
+      <c r="C11">
+        <v>0.29186853766441351</v>
+      </c>
+      <c r="D11">
+        <v>0.2941862940788269</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0.29250091314315796</v>
+      </c>
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11">
+        <v>0.31574171781539923</v>
+      </c>
+      <c r="I11">
+        <v>0.31574171781539923</v>
+      </c>
+      <c r="J11">
+        <v>0.32069301605224609</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="1"/>
+        <v>0.31739215056101483</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0.3466954022988506</v>
+      </c>
+      <c r="C12">
+        <v>0.34885057471264369</v>
+      </c>
+      <c r="D12">
+        <v>0.3603448275862069</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0.35196360153256706</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12">
+        <v>0.50172413793103454</v>
+      </c>
+      <c r="I12">
+        <v>0.50172413793103454</v>
+      </c>
+      <c r="J12">
+        <v>0.50488505747126433</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="1"/>
+        <v>0.50277777777777777</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>0.50862068965517238</v>
+      </c>
+      <c r="C13">
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="D13">
+        <v>0.52586206896551724</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="G13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <v>0.65517241379310343</v>
+      </c>
+      <c r="I13">
+        <v>0.65517241379310343</v>
+      </c>
+      <c r="J13">
+        <v>0.65517241379310343</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="1"/>
+        <v>0.65517241379310343</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>12.829803801816089</v>
+      </c>
+      <c r="C14" s="1">
+        <v>13.84695393052594</v>
+      </c>
+      <c r="D14">
+        <v>12.0599361699203</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>12.91223130075411</v>
+      </c>
+      <c r="G14" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14">
+        <v>12.24515574553917</v>
+      </c>
+      <c r="I14">
+        <v>11.68563891895886</v>
+      </c>
+      <c r="J14">
+        <v>14.27650121573744</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="1"/>
+        <v>12.735765293411824</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <f>258300/116</f>
+        <v>2226.7241379310344</v>
+      </c>
+      <c r="C15" s="1">
+        <f>250500/116</f>
+        <v>2159.4827586206898</v>
+      </c>
+      <c r="D15">
+        <f>250700/116</f>
+        <v>2161.2068965517242</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>2182.4712643678163</v>
+      </c>
+      <c r="G15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15">
+        <v>2171.879310344827</v>
+      </c>
+      <c r="I15">
+        <v>2179.6465517241381</v>
+      </c>
+      <c r="J15">
+        <v>2216.6637931034479</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="1"/>
+        <v>2189.3965517241377</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16">
+        <f>25826/116</f>
+        <v>222.63793103448276</v>
+      </c>
+      <c r="C16" s="1">
+        <v>221.81034482758622</v>
+      </c>
+      <c r="D16">
+        <f>24957/116</f>
+        <v>215.14655172413794</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>219.86494252873561</v>
+      </c>
+      <c r="G16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16">
+        <v>218.43103448275861</v>
+      </c>
+      <c r="I16">
+        <v>218.33620689655169</v>
+      </c>
+      <c r="J16">
+        <v>218.42241379310349</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="1"/>
+        <v>218.39655172413791</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17">
+        <f>284126/116</f>
+        <v>2449.3620689655172</v>
+      </c>
+      <c r="C17" s="1">
+        <f>276230/116</f>
+        <v>2381.2931034482758</v>
+      </c>
+      <c r="D17">
+        <f>275657/116</f>
+        <v>2376.3534482758619</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>2402.3362068965521</v>
+      </c>
+      <c r="G17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H17">
+        <v>2390.3103448275861</v>
+      </c>
+      <c r="I17">
+        <v>2397.9827586206902</v>
+      </c>
+      <c r="J17">
+        <v>2435.0862068965521</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="1"/>
+        <v>2407.7931034482758</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18">
+        <v>14413.73275862069</v>
+      </c>
+      <c r="I18">
+        <v>14372.456896551719</v>
+      </c>
+      <c r="J18">
+        <v>14552.26724137931</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
+        <v>35</v>
+      </c>
+      <c r="I20" t="s">
+        <v>14</v>
+      </c>
+      <c r="K20" t="s">
+        <v>51</v>
+      </c>
+      <c r="L20" t="s">
+        <v>14</v>
+      </c>
+      <c r="N20" t="s">
+        <v>37</v>
+      </c>
+      <c r="O20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21">
+        <v>0.77264215244812295</v>
+      </c>
+      <c r="C21">
+        <v>0.76778544190469022</v>
+      </c>
+      <c r="D21">
+        <v>0.76245881609211952</v>
+      </c>
+      <c r="E21">
+        <f>AVERAGE(B21:D21)</f>
+        <v>0.7676288034816442</v>
+      </c>
+      <c r="F21">
+        <f>E21-E3</f>
+        <v>0.10460795186579142</v>
+      </c>
+      <c r="G21">
+        <f>F21*100</f>
+        <v>10.460795186579141</v>
+      </c>
+      <c r="H21">
+        <f>F21/E3</f>
+        <v>0.15777475415871256</v>
+      </c>
+      <c r="I21">
+        <f>H21*100</f>
+        <v>15.777475415871256</v>
+      </c>
+      <c r="K21">
+        <f>E21-K3</f>
+        <v>3.5579234007269145E-2</v>
+      </c>
+      <c r="L21">
+        <f>K21*100</f>
+        <v>3.5579234007269145</v>
+      </c>
+      <c r="M21" t="s">
+        <v>17</v>
+      </c>
+      <c r="N21">
+        <f>K21/K3</f>
+        <v>4.8602219700526132E-2</v>
+      </c>
+      <c r="O21">
+        <f>N21*100</f>
+        <v>4.8602219700526135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22">
+        <v>0.84123563218390796</v>
+      </c>
+      <c r="C22">
+        <v>0.84037356321839096</v>
+      </c>
+      <c r="D22">
+        <v>0.83511904761904754</v>
+      </c>
+      <c r="E22">
+        <f t="shared" ref="E22:E36" si="2">AVERAGE(B22:D22)</f>
+        <v>0.83890941434044886</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22:F35" si="3">E22-E4</f>
+        <v>0.20761494252873569</v>
+      </c>
+      <c r="G22">
+        <f t="shared" ref="G22:G35" si="4">F22*100</f>
+        <v>20.761494252873568</v>
+      </c>
+      <c r="H22">
+        <f t="shared" ref="H22:H35" si="5">F22/E4</f>
+        <v>0.32887178931396999</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22:I35" si="6">H22*100</f>
+        <v>32.887178931396996</v>
+      </c>
+      <c r="K22">
+        <f t="shared" ref="K22:K35" si="7">E22-K4</f>
+        <v>3.8717843459222689E-2</v>
+      </c>
+      <c r="L22">
+        <f t="shared" ref="L22:L31" si="8">K22*100</f>
+        <v>3.8717843459222689</v>
+      </c>
+      <c r="M22" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22">
+        <f t="shared" ref="N22:N35" si="9">K22/K4</f>
+        <v>4.8385717705803785E-2</v>
+      </c>
+      <c r="O22">
+        <f t="shared" ref="O22:O35" si="10">N22*100</f>
+        <v>4.8385717705803781</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23">
+        <v>0.82298850570998738</v>
+      </c>
+      <c r="C23">
+        <v>0.80753113023231093</v>
+      </c>
+      <c r="D23">
+        <v>0.81069204977200204</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="2"/>
+        <v>0.81373722857143349</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="3"/>
+        <v>0.18326947636498414</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="4"/>
+        <v>18.326947636498414</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="5"/>
+        <v>0.2906881053370225</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="6"/>
+        <v>29.068810533702248</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="7"/>
+        <v>-6.2819284853241619E-3</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="8"/>
+        <v>-0.62819284853241619</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="9"/>
+        <v>-7.6607094252181696E-3</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="10"/>
+        <v>-0.76607094252181696</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24">
+        <v>0.77034003281154162</v>
+      </c>
+      <c r="C24">
+        <v>0.77034003281154162</v>
+      </c>
+      <c r="D24">
+        <v>0.77034003281154162</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="2"/>
+        <v>0.77034003281154162</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="3"/>
+        <v>1.0197260138552378E-2</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="4"/>
+        <v>1.0197260138552378</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="5"/>
+        <v>1.3414927438821026E-2</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="6"/>
+        <v>1.3414927438821027</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="7"/>
+        <v>-8.6346151064409238E-3</v>
+      </c>
+      <c r="L24">
+        <f t="shared" si="8"/>
+        <v>-0.86346151064409238</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="9"/>
+        <v>-1.1084590659682231E-2</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="10"/>
+        <v>-1.1084590659682232</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25">
+        <v>0.36834198288425296</v>
+      </c>
+      <c r="C25">
+        <v>0.37274607102431823</v>
+      </c>
+      <c r="D25">
+        <v>0.37256031244034138</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="2"/>
+        <v>0.37121612211630417</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="3"/>
+        <v>9.6674355743561424E-2</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="4"/>
+        <v>9.6674355743561424</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="5"/>
+        <v>0.35212986723596573</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="6"/>
+        <v>35.212986723596572</v>
+      </c>
+      <c r="K25">
+        <f t="shared" si="7"/>
+        <v>3.5937066657411476E-2</v>
+      </c>
+      <c r="L25">
+        <f t="shared" si="8"/>
+        <v>3.5937066657411476</v>
+      </c>
+      <c r="M25" t="s">
+        <v>17</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="9"/>
+        <v>0.10718554014125581</v>
+      </c>
+      <c r="O25">
+        <f t="shared" si="10"/>
+        <v>10.71855401412558</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26">
+        <v>0.67413042896192743</v>
+      </c>
+      <c r="C26">
+        <v>0.67076490948923384</v>
+      </c>
+      <c r="D26">
+        <v>0.68029604900521856</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="2"/>
+        <v>0.67506379581879328</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="3"/>
+        <v>6.6683373124337364E-2</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>6.6683373124337368</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="5"/>
+        <v>0.10960801931956224</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="6"/>
+        <v>10.960801931956224</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="7"/>
+        <v>6.4093946931616741E-2</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="8"/>
+        <v>6.4093946931616745</v>
+      </c>
+      <c r="M26" t="s">
+        <v>17</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="9"/>
+        <v>0.10490525358715781</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="10"/>
+        <v>10.490525358715781</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27">
+        <v>0.27271312627748684</v>
+      </c>
+      <c r="C27">
+        <v>0.27271312475204468</v>
+      </c>
+      <c r="D27">
+        <v>0.27271312475204468</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="2"/>
+        <v>0.27271312526052544</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="3"/>
+        <v>3.0082971366100969E-2</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="4"/>
+        <v>3.0082971366100968</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="5"/>
+        <v>0.12398694425751779</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="6"/>
+        <v>12.398694425751779</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="7"/>
+        <v>3.3556625364755677E-3</v>
+      </c>
+      <c r="L27">
+        <f t="shared" si="8"/>
+        <v>0.33556625364755677</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="9"/>
+        <v>1.2458026974783921E-2</v>
+      </c>
+      <c r="O27">
+        <f t="shared" si="10"/>
+        <v>1.245802697478392</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28">
+        <v>0.2192579662961211</v>
+      </c>
+      <c r="C28">
+        <v>0.21925795078277591</v>
+      </c>
+      <c r="D28">
+        <v>0.21925795078277591</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="2"/>
+        <v>0.21925795595389097</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="3"/>
+        <v>2.5521343157107551E-2</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="4"/>
+        <v>2.552134315710755</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="5"/>
+        <v>0.13173216352181047</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="6"/>
+        <v>13.173216352181047</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="7"/>
+        <v>-2.4945435867559096E-3</v>
+      </c>
+      <c r="L28">
+        <f t="shared" si="8"/>
+        <v>-0.24945435867559096</v>
+      </c>
+      <c r="N28">
+        <f t="shared" si="9"/>
+        <v>-1.1249224211331442E-2</v>
+      </c>
+      <c r="O28">
+        <f t="shared" si="10"/>
+        <v>-1.1249224211331443</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29">
+        <v>0.3277924655583398</v>
+      </c>
+      <c r="C29">
+        <v>0.3277924656867981</v>
+      </c>
+      <c r="D29">
+        <v>0.3277924656867981</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="2"/>
+        <v>0.32779246564397863</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="3"/>
+        <v>3.5291552500820667E-2</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="4"/>
+        <v>3.5291552500820664</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="5"/>
+        <v>0.12065450367858514</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="6"/>
+        <v>12.065450367858514</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="7"/>
+        <v>1.0400315082963796E-2</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="8"/>
+        <v>1.0400315082963796</v>
+      </c>
+      <c r="M29" t="s">
+        <v>17</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="9"/>
+        <v>3.2768028650300408E-2</v>
+      </c>
+      <c r="O29">
+        <f t="shared" si="10"/>
+        <v>3.2768028650300409</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30">
+        <v>0.55244252873563227</v>
+      </c>
+      <c r="C30">
+        <v>0.55244252873563215</v>
+      </c>
+      <c r="D30">
+        <v>0.54382183908045978</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="2"/>
+        <v>0.54956896551724144</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="3"/>
+        <v>0.19760536398467438</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="4"/>
+        <v>19.760536398467437</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="5"/>
+        <v>0.5614369301945844</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="6"/>
+        <v>56.143693019458439</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="7"/>
+        <v>4.6791187739463669E-2</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="8"/>
+        <v>4.6791187739463673</v>
+      </c>
+      <c r="M30" t="s">
+        <v>17</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="9"/>
+        <v>9.3065345780148731E-2</v>
+      </c>
+      <c r="O30">
+        <f t="shared" si="10"/>
+        <v>9.3065345780148725</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31">
+        <v>0.7068965517241379</v>
+      </c>
+      <c r="C31">
+        <v>0.7068965517241379</v>
+      </c>
+      <c r="D31">
+        <v>0.69827586206896552</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="2"/>
+        <v>0.70402298850574707</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="3"/>
+        <v>0.18678160919540221</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="4"/>
+        <v>18.678160919540222</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="5"/>
+        <v>0.36111111111111094</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="6"/>
+        <v>36.111111111111093</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="7"/>
+        <v>4.8850574712643646E-2</v>
+      </c>
+      <c r="L31">
+        <f t="shared" si="8"/>
+        <v>4.8850574712643642</v>
+      </c>
+      <c r="M31" t="s">
+        <v>17</v>
+      </c>
+      <c r="N31">
+        <f t="shared" si="9"/>
+        <v>7.4561403508771884E-2</v>
+      </c>
+      <c r="O31">
+        <f t="shared" si="10"/>
+        <v>7.4561403508771882</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32">
+        <v>13.379221959360709</v>
+      </c>
+      <c r="C32">
+        <v>13.379414190506109</v>
+      </c>
+      <c r="D32">
+        <v>13.921241846577869</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="2"/>
+        <v>13.55995933214823</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="3"/>
+        <v>0.64772803139412005</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="4"/>
+        <v>64.772803139412005</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="5"/>
+        <v>5.0163911744385413E-2</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="6"/>
+        <v>5.0163911744385414</v>
+      </c>
+      <c r="K32">
+        <f t="shared" si="7"/>
+        <v>0.8241940387364064</v>
+      </c>
+      <c r="N32">
+        <f t="shared" si="9"/>
+        <v>6.4714920520933264E-2</v>
+      </c>
+      <c r="O32">
+        <f t="shared" si="10"/>
+        <v>6.4714920520933266</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33">
+        <v>2201.1034482758619</v>
+      </c>
+      <c r="C33">
+        <v>2213.6120689655172</v>
+      </c>
+      <c r="D33">
+        <v>2202.0775862068972</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="2"/>
+        <v>2205.5977011494251</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="3"/>
+        <v>23.126436781608845</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="4"/>
+        <v>2312.6436781608845</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="5"/>
+        <v>1.0596445029624592E-2</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="6"/>
+        <v>1.0596445029624593</v>
+      </c>
+      <c r="K33">
+        <f t="shared" si="7"/>
+        <v>16.20114942528744</v>
+      </c>
+      <c r="N33">
+        <f t="shared" si="9"/>
+        <v>7.3998241262091717E-3</v>
+      </c>
+      <c r="O33">
+        <f t="shared" si="10"/>
+        <v>0.73998241262091713</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34">
+        <v>222.25</v>
+      </c>
+      <c r="C34">
+        <v>223.73275862068971</v>
+      </c>
+      <c r="D34">
+        <v>220</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="2"/>
+        <v>221.99425287356325</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="3"/>
+        <v>2.129310344827644</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="4"/>
+        <v>212.9310344827644</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="5"/>
+        <v>9.6846287558979543E-3</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="6"/>
+        <v>0.96846287558979538</v>
+      </c>
+      <c r="K34">
+        <f t="shared" si="7"/>
+        <v>3.5977011494253475</v>
+      </c>
+      <c r="N34">
+        <f t="shared" si="9"/>
+        <v>1.6473250703929122E-2</v>
+      </c>
+      <c r="O34">
+        <f t="shared" si="10"/>
+        <v>1.6473250703929121</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35">
+        <v>2423.3534482758619</v>
+      </c>
+      <c r="C35">
+        <v>2437.344827586207</v>
+      </c>
+      <c r="D35">
+        <v>2422.0775862068972</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="2"/>
+        <v>2427.5919540229884</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="3"/>
+        <v>25.25574712643629</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="4"/>
+        <v>2525.574712643629</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="5"/>
+        <v>1.0512994415158411E-2</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="6"/>
+        <v>1.051299441515841</v>
+      </c>
+      <c r="K35">
+        <f t="shared" si="7"/>
+        <v>19.79885057471256</v>
+      </c>
+      <c r="N35">
+        <f t="shared" si="9"/>
+        <v>8.2228205348532681E-3</v>
+      </c>
+      <c r="O35">
+        <f t="shared" si="10"/>
+        <v>0.82228205348532679</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36">
+        <v>13057.560344827591</v>
+      </c>
+      <c r="C36">
+        <v>12947.78448275862</v>
+      </c>
+      <c r="D36">
+        <v>12960.474137931031</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="2"/>
+        <v>12988.606321839079</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D39" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>57</v>
+      </c>
+      <c r="F39" t="s">
+        <v>34</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" t="s">
+        <v>35</v>
+      </c>
+      <c r="I39" t="s">
+        <v>14</v>
+      </c>
+      <c r="K39" t="s">
+        <v>58</v>
+      </c>
+      <c r="L39" t="s">
+        <v>14</v>
+      </c>
+      <c r="N39" t="s">
+        <v>37</v>
+      </c>
+      <c r="O39" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>51</v>
+      </c>
+      <c r="R39" t="s">
+        <v>14</v>
+      </c>
+      <c r="T39" t="s">
+        <v>37</v>
+      </c>
+      <c r="U39" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40">
+        <v>0.73745520382817531</v>
+      </c>
+      <c r="E40">
+        <f>AVERAGE(B40:D40)</f>
+        <v>0.73745520382817531</v>
+      </c>
+      <c r="F40">
+        <f>E40-E3</f>
+        <v>7.443435221232253E-2</v>
+      </c>
+      <c r="G40">
+        <f>F40*100</f>
+        <v>7.443435221232253</v>
+      </c>
+      <c r="H40">
+        <f>F40/E3</f>
+        <v>0.11226547706745278</v>
+      </c>
+      <c r="I40">
+        <f>H40*100</f>
+        <v>11.226547706745277</v>
+      </c>
+      <c r="K40">
+        <f>E40-E21</f>
+        <v>-3.0173599653468886E-2</v>
+      </c>
+      <c r="L40">
+        <f>K40*100</f>
+        <v>-3.0173599653468886</v>
+      </c>
+      <c r="N40">
+        <f>K40/E21</f>
+        <v>-3.9307539681437201E-2</v>
+      </c>
+      <c r="O40">
+        <f>N40*100</f>
+        <v>-3.93075396814372</v>
+      </c>
+      <c r="Q40">
+        <f>E40-K3</f>
+        <v>5.4056343538002594E-3</v>
+      </c>
+      <c r="R40">
+        <f>Q40*100</f>
+        <v>0.54056343538002594</v>
+      </c>
+      <c r="T40">
+        <f>Q40/K3</f>
+        <v>7.3842463396045759E-3</v>
+      </c>
+      <c r="U40">
+        <f>T40*100</f>
+        <v>0.73842463396045754</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41">
+        <v>0.76327996715927759</v>
+      </c>
+      <c r="E41">
+        <f t="shared" ref="E41:E55" si="11">AVERAGE(B41:D41)</f>
+        <v>0.76327996715927759</v>
+      </c>
+      <c r="F41">
+        <f t="shared" ref="F41:F54" si="12">E41-E4</f>
+        <v>0.13198549534756443</v>
+      </c>
+      <c r="G41">
+        <f t="shared" ref="G41:G54" si="13">F41*100</f>
+        <v>13.198549534756443</v>
+      </c>
+      <c r="H41">
+        <f t="shared" ref="H41:H54" si="14">F41/E4</f>
+        <v>0.20907120407499749</v>
+      </c>
+      <c r="I41">
+        <f t="shared" ref="I41:I54" si="15">H41*100</f>
+        <v>20.90712040749975</v>
+      </c>
+      <c r="K41">
+        <f t="shared" ref="K41:K54" si="16">E41-E22</f>
+        <v>-7.5629447181171261E-2</v>
+      </c>
+      <c r="L41">
+        <f t="shared" ref="L41:L50" si="17">K41*100</f>
+        <v>-7.5629447181171265</v>
+      </c>
+      <c r="N41">
+        <f t="shared" ref="N41:N54" si="18">K41/E22</f>
+        <v>-9.0152102108224857E-2</v>
+      </c>
+      <c r="O41">
+        <f t="shared" ref="O41:O54" si="19">N41*100</f>
+        <v>-9.0152102108224863</v>
+      </c>
+      <c r="Q41">
+        <f>E41-K4</f>
+        <v>-3.6911603721948572E-2</v>
+      </c>
+      <c r="R41">
+        <f t="shared" ref="R41:R50" si="20">Q41*100</f>
+        <v>-3.6911603721948572</v>
+      </c>
+      <c r="T41">
+        <f>Q41/K4</f>
+        <v>-4.6128458565614441E-2</v>
+      </c>
+      <c r="U41">
+        <f t="shared" ref="U41:U54" si="21">T41*100</f>
+        <v>-4.6128458565614441</v>
+      </c>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42">
+        <v>0.72266522985235537</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="11"/>
+        <v>0.72266522985235537</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="12"/>
+        <v>9.2197477645906023E-2</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="13"/>
+        <v>9.2197477645906023</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="14"/>
+        <v>0.14623662720772365</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="15"/>
+        <v>14.623662720772366</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="16"/>
+        <v>-9.1071998719078118E-2</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="17"/>
+        <v>-9.1071998719078113</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="18"/>
+        <v>-0.11191819118188889</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="19"/>
+        <v>-11.191819118188889</v>
+      </c>
+      <c r="Q42">
+        <f>E42-K5</f>
+        <v>-9.735392720440228E-2</v>
+      </c>
+      <c r="R42">
+        <f t="shared" si="20"/>
+        <v>-9.7353927204402275</v>
+      </c>
+      <c r="S42" t="s">
+        <v>16</v>
+      </c>
+      <c r="T42">
+        <f>Q42/K5</f>
+        <v>-0.1187215278650666</v>
+      </c>
+      <c r="U42">
+        <f t="shared" si="21"/>
+        <v>-11.872152786506659</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43">
+        <v>0.78235877899259454</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="11"/>
+        <v>0.78235877899259454</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="12"/>
+        <v>2.2216006319605297E-2</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="13"/>
+        <v>2.2216006319605297</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="14"/>
+        <v>2.9226096883726533E-2</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="15"/>
+        <v>2.9226096883726531</v>
+      </c>
+      <c r="K43">
+        <f t="shared" si="16"/>
+        <v>1.2018746181052919E-2</v>
+      </c>
+      <c r="L43">
+        <f t="shared" si="17"/>
+        <v>1.2018746181052919</v>
+      </c>
+      <c r="N43">
+        <f t="shared" si="18"/>
+        <v>1.560187147120942E-2</v>
+      </c>
+      <c r="O43">
+        <f t="shared" si="19"/>
+        <v>1.5601871471209421</v>
+      </c>
+      <c r="Q43">
+        <f>E43-K6</f>
+        <v>3.3841310746119957E-3</v>
+      </c>
+      <c r="R43">
+        <f t="shared" si="20"/>
+        <v>0.33841310746119957</v>
+      </c>
+      <c r="T43">
+        <f>Q43/K6</f>
+        <v>4.3443404527438584E-3</v>
+      </c>
+      <c r="U43">
+        <f t="shared" si="21"/>
+        <v>0.43443404527438584</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>8</v>
+      </c>
+      <c r="B44">
+        <v>0.32017835358857871</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="11"/>
+        <v>0.32017835358857871</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="12"/>
+        <v>4.5636587215835966E-2</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="13"/>
+        <v>4.5636587215835966</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="14"/>
+        <v>0.16622821299210119</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="15"/>
+        <v>16.62282129921012</v>
+      </c>
+      <c r="K44">
+        <f t="shared" si="16"/>
+        <v>-5.1037768527725458E-2</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="17"/>
+        <v>-5.1037768527725458</v>
+      </c>
+      <c r="N44">
+        <f t="shared" si="18"/>
+        <v>-0.13748801705259728</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="19"/>
+        <v>-13.748801705259728</v>
+      </c>
+      <c r="Q44">
+        <f>E44-K7</f>
+        <v>-1.5100701870313982E-2</v>
+      </c>
+      <c r="R44">
+        <f t="shared" si="20"/>
+        <v>-1.5100701870313982</v>
+      </c>
+      <c r="T44">
+        <f>Q44/K7</f>
+        <v>-4.5039204282074287E-2</v>
+      </c>
+      <c r="U44">
+        <f t="shared" si="21"/>
+        <v>-4.5039204282074286</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45">
+        <v>0.67979355968595312</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="11"/>
+        <v>0.67979355968595312</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="12"/>
+        <v>7.1413136991497206E-2</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="13"/>
+        <v>7.1413136991497206</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="14"/>
+        <v>0.11738237183112432</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="15"/>
+        <v>11.738237183112432</v>
+      </c>
+      <c r="K45">
+        <f t="shared" si="16"/>
+        <v>4.7297638671598419E-3</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="17"/>
+        <v>0.47297638671598419</v>
+      </c>
+      <c r="N45">
+        <f t="shared" si="18"/>
+        <v>7.0063953902653785E-3</v>
+      </c>
+      <c r="O45">
+        <f t="shared" si="19"/>
+        <v>0.70063953902653786</v>
+      </c>
+      <c r="Q45">
+        <f>E45-K8</f>
+        <v>6.8823710798776583E-2</v>
+      </c>
+      <c r="R45">
+        <f t="shared" si="20"/>
+        <v>6.8823710798776583</v>
+      </c>
+      <c r="S45" t="s">
+        <v>17</v>
+      </c>
+      <c r="T45">
+        <f>Q45/K8</f>
+        <v>0.11264665666257087</v>
+      </c>
+      <c r="U45">
+        <f t="shared" si="21"/>
+        <v>11.264665666257088</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46">
+        <v>0.28677049279212952</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="11"/>
+        <v>0.28677049279212952</v>
+      </c>
+      <c r="F46">
+        <f t="shared" si="12"/>
+        <v>4.414033889770505E-2</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="13"/>
+        <v>4.4140338897705051</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="14"/>
+        <v>0.18192437415224083</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="15"/>
+        <v>18.192437415224084</v>
+      </c>
+      <c r="K46">
+        <f t="shared" si="16"/>
+        <v>1.4057367531604081E-2</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="17"/>
+        <v>1.4057367531604081</v>
+      </c>
+      <c r="N46">
+        <f t="shared" si="18"/>
+        <v>5.1546354867133527E-2</v>
+      </c>
+      <c r="O46">
+        <f t="shared" si="19"/>
+        <v>5.154635486713353</v>
+      </c>
+      <c r="Q46">
+        <f>E46-K9</f>
+        <v>1.7413030068079649E-2</v>
+      </c>
+      <c r="R46">
+        <f t="shared" si="20"/>
+        <v>1.7413030068079649</v>
+      </c>
+      <c r="S46" t="s">
+        <v>17</v>
+      </c>
+      <c r="T46">
+        <f>Q46/K9</f>
+        <v>6.4646547721303987E-2</v>
+      </c>
+      <c r="U46">
+        <f t="shared" si="21"/>
+        <v>6.4646547721303991</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47">
+        <v>0.23999802768230441</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="11"/>
+        <v>0.23999802768230441</v>
+      </c>
+      <c r="F47">
+        <f t="shared" si="12"/>
+        <v>4.6261414885520991E-2</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="13"/>
+        <v>4.6261414885520988</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="14"/>
+        <v>0.23878509187133401</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="15"/>
+        <v>23.8785091871334</v>
+      </c>
+      <c r="K47">
+        <f t="shared" si="16"/>
+        <v>2.0740071728413439E-2</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="17"/>
+        <v>2.0740071728413438</v>
+      </c>
+      <c r="N47">
+        <f t="shared" si="18"/>
+        <v>9.4592105623638081E-2</v>
+      </c>
+      <c r="O47">
+        <f t="shared" si="19"/>
+        <v>9.4592105623638076</v>
+      </c>
+      <c r="Q47">
+        <f>E47-K10</f>
+        <v>1.824552814165753E-2</v>
+      </c>
+      <c r="R47">
+        <f t="shared" si="20"/>
+        <v>1.824552814165753</v>
+      </c>
+      <c r="S47" t="s">
+        <v>17</v>
+      </c>
+      <c r="T47">
+        <f>Q47/K10</f>
+        <v>8.2278793607524381E-2</v>
+      </c>
+      <c r="U47">
+        <f t="shared" si="21"/>
+        <v>8.2278793607524374</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48">
+        <v>0.33447659015655518</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="11"/>
+        <v>0.33447659015655518</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="12"/>
+        <v>4.1975677013397217E-2</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="13"/>
+        <v>4.1975677013397217</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="14"/>
+        <v>0.1435061400743497</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="15"/>
+        <v>14.35061400743497</v>
+      </c>
+      <c r="K48">
+        <f t="shared" si="16"/>
+        <v>6.6841245125765503E-3</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="17"/>
+        <v>0.66841245125765503</v>
+      </c>
+      <c r="N48">
+        <f t="shared" si="18"/>
+        <v>2.0391330531179138E-2</v>
+      </c>
+      <c r="O48">
+        <f t="shared" si="19"/>
+        <v>2.0391330531179137</v>
+      </c>
+      <c r="Q48">
+        <f>E48-K11</f>
+        <v>1.7084439595540346E-2</v>
+      </c>
+      <c r="R48">
+        <f t="shared" si="20"/>
+        <v>1.7084439595540346</v>
+      </c>
+      <c r="S48" t="s">
+        <v>17</v>
+      </c>
+      <c r="T48">
+        <f>Q48/K11</f>
+        <v>5.3827542884542973E-2</v>
+      </c>
+      <c r="U48">
+        <f t="shared" si="21"/>
+        <v>5.3827542884542972</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B49">
+        <v>0.4653735632183908</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="11"/>
+        <v>0.4653735632183908</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="12"/>
+        <v>0.11340996168582373</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="13"/>
+        <v>11.340996168582373</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="14"/>
+        <v>0.32222071030072114</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="15"/>
+        <v>32.222071030072115</v>
+      </c>
+      <c r="K49">
+        <f t="shared" si="16"/>
+        <v>-8.4195402298850641E-2</v>
+      </c>
+      <c r="L49">
+        <f t="shared" si="17"/>
+        <v>-8.4195402298850635</v>
+      </c>
+      <c r="N49">
+        <f t="shared" si="18"/>
+        <v>-0.15320261437908508</v>
+      </c>
+      <c r="O49">
+        <f t="shared" si="19"/>
+        <v>-15.320261437908508</v>
+      </c>
+      <c r="Q49">
+        <f>E49-K12</f>
+        <v>-3.7404214559386972E-2</v>
+      </c>
+      <c r="R49">
+        <f t="shared" si="20"/>
+        <v>-3.740421455938697</v>
+      </c>
+      <c r="T49">
+        <f>Q49/K12</f>
+        <v>-7.439512288054867E-2</v>
+      </c>
+      <c r="U49">
+        <f t="shared" si="21"/>
+        <v>-7.4395122880548668</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50">
+        <v>0.62931034482758619</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="11"/>
+        <v>0.62931034482758619</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="12"/>
+        <v>0.11206896551724133</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="13"/>
+        <v>11.206896551724132</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="14"/>
+        <v>0.21666666666666654</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="15"/>
+        <v>21.666666666666654</v>
+      </c>
+      <c r="K50">
+        <f t="shared" si="16"/>
+        <v>-7.4712643678160884E-2</v>
+      </c>
+      <c r="L50">
+        <f t="shared" si="17"/>
+        <v>-7.4712643678160884</v>
+      </c>
+      <c r="N50">
+        <f t="shared" si="18"/>
+        <v>-0.10612244897959179</v>
+      </c>
+      <c r="O50">
+        <f t="shared" si="19"/>
+        <v>-10.612244897959179</v>
+      </c>
+      <c r="Q50">
+        <f>E50-K13</f>
+        <v>-2.5862068965517238E-2</v>
+      </c>
+      <c r="R50">
+        <f t="shared" si="20"/>
+        <v>-2.5862068965517238</v>
+      </c>
+      <c r="T50">
+        <f>Q50/K13</f>
+        <v>-3.9473684210526314E-2</v>
+      </c>
+      <c r="U50">
+        <f t="shared" si="21"/>
+        <v>-3.9473684210526314</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51">
+        <v>13.829238024251209</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="11"/>
+        <v>13.829238024251209</v>
+      </c>
+      <c r="F51">
+        <f t="shared" si="12"/>
+        <v>0.91700672349709933</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="13"/>
+        <v>91.700672349709933</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="14"/>
+        <v>7.1018455458085203E-2</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="15"/>
+        <v>7.1018455458085201</v>
+      </c>
+      <c r="K51">
+        <f t="shared" si="16"/>
+        <v>0.26927869210297928</v>
+      </c>
+      <c r="N51">
+        <f t="shared" si="18"/>
+        <v>1.9858370184383065E-2</v>
+      </c>
+      <c r="O51">
+        <f t="shared" si="19"/>
+        <v>1.9858370184383065</v>
+      </c>
+      <c r="Q51">
+        <f>E51-K14</f>
+        <v>1.0934727308393857</v>
+      </c>
+      <c r="T51">
+        <f>Q51/K14</f>
+        <v>8.5858423553473937E-2</v>
+      </c>
+      <c r="U51">
+        <f t="shared" si="21"/>
+        <v>8.5858423553473937</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>31</v>
+      </c>
+      <c r="B52">
+        <v>2185.9396551724139</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="11"/>
+        <v>2185.9396551724139</v>
+      </c>
+      <c r="F52">
+        <f t="shared" si="12"/>
+        <v>3.468390804597675</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="13"/>
+        <v>346.8390804597675</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="14"/>
+        <v>1.5892034233047937E-3</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="15"/>
+        <v>0.15892034233047939</v>
+      </c>
+      <c r="K52">
+        <f t="shared" si="16"/>
+        <v>-19.65804597701117</v>
+      </c>
+      <c r="N52">
+        <f t="shared" si="18"/>
+        <v>-8.9127976361086051E-3</v>
+      </c>
+      <c r="O52">
+        <f t="shared" si="19"/>
+        <v>-0.89127976361086048</v>
+      </c>
+      <c r="Q52">
+        <f>E52-K15</f>
+        <v>-3.4568965517237302</v>
+      </c>
+      <c r="T52">
+        <f>Q52/K15</f>
+        <v>-1.5789266448791304E-3</v>
+      </c>
+      <c r="U52">
+        <f t="shared" si="21"/>
+        <v>-0.15789266448791303</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>32</v>
+      </c>
+      <c r="B53">
+        <v>214.4568965517241</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="11"/>
+        <v>214.4568965517241</v>
+      </c>
+      <c r="F53">
+        <f t="shared" si="12"/>
+        <v>-5.4080459770115112</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="13"/>
+        <v>-540.80459770115112</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="14"/>
+        <v>-2.4597127285559395E-2</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="15"/>
+        <v>-2.4597127285559397</v>
+      </c>
+      <c r="K53">
+        <f t="shared" si="16"/>
+        <v>-7.5373563218391553</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="18"/>
+        <v>-3.3952934475885078E-2</v>
+      </c>
+      <c r="O53">
+        <f t="shared" si="19"/>
+        <v>-3.3952934475885077</v>
+      </c>
+      <c r="Q53">
+        <f>E53-K16</f>
+        <v>-3.9396551724138078</v>
+      </c>
+      <c r="T53">
+        <f>Q53/K16</f>
+        <v>-1.8038998973711286E-2</v>
+      </c>
+      <c r="U53">
+        <f t="shared" si="21"/>
+        <v>-1.8038998973711287</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>33</v>
+      </c>
+      <c r="B54">
+        <v>2400.3965517241381</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="11"/>
+        <v>2400.3965517241381</v>
+      </c>
+      <c r="F54">
+        <f t="shared" si="12"/>
+        <v>-1.9396551724139499</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="13"/>
+        <v>-193.96551724139499</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="14"/>
+        <v>-8.0740371262175885E-4</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="15"/>
+        <v>-8.0740371262175883E-2</v>
+      </c>
+      <c r="K54">
+        <f t="shared" si="16"/>
+        <v>-27.19540229885024</v>
+      </c>
+      <c r="N54">
+        <f t="shared" si="18"/>
+        <v>-1.1202624993785389E-2</v>
+      </c>
+      <c r="O54">
+        <f t="shared" si="19"/>
+        <v>-1.1202624993785388</v>
+      </c>
+      <c r="Q54">
+        <f>E54-K17</f>
+        <v>-7.3965517241376801</v>
+      </c>
+      <c r="T54">
+        <f>Q54/K17</f>
+        <v>-3.0719216337752805E-3</v>
+      </c>
+      <c r="U54">
+        <f t="shared" si="21"/>
+        <v>-0.30719216337752808</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>45</v>
+      </c>
+      <c r="B55">
+        <v>11011.8275862069</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="11"/>
+        <v>11011.8275862069</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C64D6A0-67B0-420F-B472-231F769BBEC3}">
   <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Results: multiple reruns and final conclusion
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Zwischenstand.xlsx
+++ b/src/evaluation/data/Zwischenstand.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45A46EC-D076-462F-BCC3-0B067E39E460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B9A0F8-D127-41B6-901F-E381D0E240F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="12" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{D3F11DAE-F554-4455-8ED3-B07E6EB1D3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="naive max_size" sheetId="1" state="hidden" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="59">
   <si>
     <t>run1</t>
   </si>
@@ -5687,6 +5687,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2812793-DBB4-41C8-A6C8-004B2B5D4FF1}">
   <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="11" max="11" width="27.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -7147,57 +7150,63 @@
       <c r="B40">
         <v>0.73745520382817531</v>
       </c>
+      <c r="C40">
+        <v>0.74461169948414752</v>
+      </c>
+      <c r="D40">
+        <v>0.7385652513758495</v>
+      </c>
       <c r="E40">
         <f>AVERAGE(B40:D40)</f>
-        <v>0.73745520382817531</v>
+        <v>0.74021071822939077</v>
       </c>
       <c r="F40">
         <f>E40-E3</f>
-        <v>7.443435221232253E-2</v>
+        <v>7.7189866613537994E-2</v>
       </c>
       <c r="G40">
         <f>F40*100</f>
-        <v>7.443435221232253</v>
+        <v>7.7189866613537994</v>
       </c>
       <c r="H40">
         <f>F40/E3</f>
-        <v>0.11226547706745278</v>
+        <v>0.11642147667817389</v>
       </c>
       <c r="I40">
         <f>H40*100</f>
-        <v>11.226547706745277</v>
+        <v>11.642147667817389</v>
       </c>
       <c r="K40">
         <f>E40-E21</f>
-        <v>-3.0173599653468886E-2</v>
+        <v>-2.7418085252253421E-2</v>
       </c>
       <c r="L40">
         <f>K40*100</f>
-        <v>-3.0173599653468886</v>
+        <v>-2.7418085252253421</v>
       </c>
       <c r="N40">
         <f>K40/E21</f>
-        <v>-3.9307539681437201E-2</v>
+        <v>-3.5717895326356199E-2</v>
       </c>
       <c r="O40">
         <f>N40*100</f>
-        <v>-3.93075396814372</v>
+        <v>-3.5717895326356199</v>
       </c>
       <c r="Q40">
-        <f>E40-K3</f>
-        <v>5.4056343538002594E-3</v>
+        <f t="shared" ref="Q40:Q54" si="11">E40-K3</f>
+        <v>8.1611487550157236E-3</v>
       </c>
       <c r="R40">
         <f>Q40*100</f>
-        <v>0.54056343538002594</v>
+        <v>0.81611487550157236</v>
       </c>
       <c r="T40">
-        <f>Q40/K3</f>
-        <v>7.3842463396045759E-3</v>
+        <f t="shared" ref="T40:T54" si="12">Q40/K3</f>
+        <v>1.1148355378277974E-2</v>
       </c>
       <c r="U40">
         <f>T40*100</f>
-        <v>0.73842463396045754</v>
+        <v>1.1148355378277974</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -7207,57 +7216,63 @@
       <c r="B41">
         <v>0.76327996715927759</v>
       </c>
+      <c r="C41">
+        <v>0.76522988505747114</v>
+      </c>
+      <c r="D41">
+        <v>0.77169540229885059</v>
+      </c>
       <c r="E41">
-        <f t="shared" ref="E41:E55" si="11">AVERAGE(B41:D41)</f>
-        <v>0.76327996715927759</v>
+        <f t="shared" ref="E41:E55" si="13">AVERAGE(B41:D41)</f>
+        <v>0.76673508483853314</v>
       </c>
       <c r="F41">
-        <f t="shared" ref="F41:F54" si="12">E41-E4</f>
-        <v>0.13198549534756443</v>
+        <f t="shared" ref="F41:F54" si="14">E41-E4</f>
+        <v>0.13544061302681998</v>
       </c>
       <c r="G41">
-        <f t="shared" ref="G41:G54" si="13">F41*100</f>
-        <v>13.198549534756443</v>
+        <f t="shared" ref="G41:G54" si="15">F41*100</f>
+        <v>13.544061302681998</v>
       </c>
       <c r="H41">
-        <f t="shared" ref="H41:H54" si="14">F41/E4</f>
-        <v>0.20907120407499749</v>
+        <f t="shared" ref="H41:H54" si="16">F41/E4</f>
+        <v>0.21454427224449993</v>
       </c>
       <c r="I41">
-        <f t="shared" ref="I41:I54" si="15">H41*100</f>
-        <v>20.90712040749975</v>
+        <f t="shared" ref="I41:I54" si="17">H41*100</f>
+        <v>21.454427224449994</v>
       </c>
       <c r="K41">
-        <f t="shared" ref="K41:K54" si="16">E41-E22</f>
-        <v>-7.5629447181171261E-2</v>
+        <f t="shared" ref="K41:K54" si="18">E41-E22</f>
+        <v>-7.2174329501915713E-2</v>
       </c>
       <c r="L41">
-        <f t="shared" ref="L41:L50" si="17">K41*100</f>
-        <v>-7.5629447181171265</v>
+        <f t="shared" ref="L41:L50" si="19">K41*100</f>
+        <v>-7.2174329501915713</v>
       </c>
       <c r="N41">
-        <f t="shared" ref="N41:N54" si="18">K41/E22</f>
-        <v>-9.0152102108224857E-2</v>
+        <f t="shared" ref="N41:N54" si="20">K41/E22</f>
+        <v>-8.6033519553072632E-2</v>
       </c>
       <c r="O41">
-        <f t="shared" ref="O41:O54" si="19">N41*100</f>
-        <v>-9.0152102108224863</v>
+        <f t="shared" ref="O41:O54" si="21">N41*100</f>
+        <v>-8.6033519553072626</v>
       </c>
       <c r="Q41">
-        <f>E41-K4</f>
-        <v>-3.6911603721948572E-2</v>
+        <f t="shared" si="11"/>
+        <v>-3.3456486042693023E-2</v>
       </c>
       <c r="R41">
-        <f t="shared" ref="R41:R50" si="20">Q41*100</f>
-        <v>-3.6911603721948572</v>
+        <f t="shared" ref="R41:R50" si="22">Q41*100</f>
+        <v>-3.3456486042693023</v>
       </c>
       <c r="T41">
-        <f>Q41/K4</f>
-        <v>-4.6128458565614441E-2</v>
+        <f t="shared" si="12"/>
+        <v>-4.1810595437600566E-2</v>
       </c>
       <c r="U41">
-        <f t="shared" ref="U41:U54" si="21">T41*100</f>
-        <v>-4.6128458565614441</v>
+        <f t="shared" ref="U41:U54" si="23">T41*100</f>
+        <v>-4.1810595437600568</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -7267,60 +7282,66 @@
       <c r="B42">
         <v>0.72266522985235537</v>
       </c>
+      <c r="C42">
+        <v>0.70678879307098252</v>
+      </c>
+      <c r="D42">
+        <v>0.72523946356658919</v>
+      </c>
       <c r="E42">
+        <f t="shared" si="13"/>
+        <v>0.71823116216330896</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="14"/>
+        <v>8.7763409956859606E-2</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="15"/>
+        <v>8.7763409956859597</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="16"/>
+        <v>0.13920364626059589</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="17"/>
+        <v>13.920364626059589</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="18"/>
+        <v>-9.5506066408124535E-2</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="19"/>
+        <v>-9.5506066408124539</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="20"/>
+        <v>-0.11736720780956697</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="21"/>
+        <v>-11.736720780956697</v>
+      </c>
+      <c r="Q42">
         <f t="shared" si="11"/>
-        <v>0.72266522985235537</v>
-      </c>
-      <c r="F42">
-        <f t="shared" si="12"/>
-        <v>9.2197477645906023E-2</v>
-      </c>
-      <c r="G42">
-        <f t="shared" si="13"/>
-        <v>9.2197477645906023</v>
-      </c>
-      <c r="H42">
-        <f t="shared" si="14"/>
-        <v>0.14623662720772365</v>
-      </c>
-      <c r="I42">
-        <f t="shared" si="15"/>
-        <v>14.623662720772366</v>
-      </c>
-      <c r="K42">
-        <f t="shared" si="16"/>
-        <v>-9.1071998719078118E-2</v>
-      </c>
-      <c r="L42">
-        <f t="shared" si="17"/>
-        <v>-9.1071998719078113</v>
-      </c>
-      <c r="N42">
-        <f t="shared" si="18"/>
-        <v>-0.11191819118188889</v>
-      </c>
-      <c r="O42">
-        <f t="shared" si="19"/>
-        <v>-11.191819118188889</v>
-      </c>
-      <c r="Q42">
-        <f>E42-K5</f>
-        <v>-9.735392720440228E-2</v>
+        <v>-0.1017879948934487</v>
       </c>
       <c r="R42">
-        <f t="shared" si="20"/>
-        <v>-9.7353927204402275</v>
+        <f t="shared" si="22"/>
+        <v>-10.17879948934487</v>
       </c>
       <c r="S42" t="s">
         <v>16</v>
       </c>
       <c r="T42">
-        <f>Q42/K5</f>
-        <v>-0.1187215278650666</v>
+        <f t="shared" si="12"/>
+        <v>-0.12412880115970686</v>
       </c>
       <c r="U42">
-        <f t="shared" si="21"/>
-        <v>-11.872152786506659</v>
+        <f t="shared" si="23"/>
+        <v>-12.412880115970685</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -7330,57 +7351,63 @@
       <c r="B43">
         <v>0.78235877899259454</v>
       </c>
+      <c r="C43">
+        <v>0.78235877899259454</v>
+      </c>
+      <c r="D43">
+        <v>0.78235877899259476</v>
+      </c>
       <c r="E43">
+        <f t="shared" si="13"/>
+        <v>0.78235877899259465</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="14"/>
+        <v>2.2216006319605408E-2</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="15"/>
+        <v>2.2216006319605408</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="16"/>
+        <v>2.9226096883726679E-2</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="17"/>
+        <v>2.9226096883726678</v>
+      </c>
+      <c r="K43">
+        <f t="shared" si="18"/>
+        <v>1.201874618105303E-2</v>
+      </c>
+      <c r="L43">
+        <f t="shared" si="19"/>
+        <v>1.201874618105303</v>
+      </c>
+      <c r="N43">
+        <f t="shared" si="20"/>
+        <v>1.5601871471209564E-2</v>
+      </c>
+      <c r="O43">
+        <f t="shared" si="21"/>
+        <v>1.5601871471209565</v>
+      </c>
+      <c r="Q43">
         <f t="shared" si="11"/>
-        <v>0.78235877899259454</v>
-      </c>
-      <c r="F43">
+        <v>3.3841310746121067E-3</v>
+      </c>
+      <c r="R43">
+        <f t="shared" si="22"/>
+        <v>0.33841310746121067</v>
+      </c>
+      <c r="T43">
         <f t="shared" si="12"/>
-        <v>2.2216006319605297E-2</v>
-      </c>
-      <c r="G43">
-        <f t="shared" si="13"/>
-        <v>2.2216006319605297</v>
-      </c>
-      <c r="H43">
-        <f t="shared" si="14"/>
-        <v>2.9226096883726533E-2</v>
-      </c>
-      <c r="I43">
-        <f t="shared" si="15"/>
-        <v>2.9226096883726531</v>
-      </c>
-      <c r="K43">
-        <f t="shared" si="16"/>
-        <v>1.2018746181052919E-2</v>
-      </c>
-      <c r="L43">
-        <f t="shared" si="17"/>
-        <v>1.2018746181052919</v>
-      </c>
-      <c r="N43">
-        <f t="shared" si="18"/>
-        <v>1.560187147120942E-2</v>
-      </c>
-      <c r="O43">
-        <f t="shared" si="19"/>
-        <v>1.5601871471209421</v>
-      </c>
-      <c r="Q43">
-        <f>E43-K6</f>
-        <v>3.3841310746119957E-3</v>
-      </c>
-      <c r="R43">
-        <f t="shared" si="20"/>
-        <v>0.33841310746119957</v>
-      </c>
-      <c r="T43">
-        <f>Q43/K6</f>
-        <v>4.3443404527438584E-3</v>
+        <v>4.3443404527440006E-3</v>
       </c>
       <c r="U43">
-        <f t="shared" si="21"/>
-        <v>0.43443404527438584</v>
+        <f t="shared" si="23"/>
+        <v>0.43443404527440005</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -7390,57 +7417,63 @@
       <c r="B44">
         <v>0.32017835358857871</v>
       </c>
+      <c r="C44">
+        <v>0.32961473783399581</v>
+      </c>
+      <c r="D44">
+        <v>0.33286277736459546</v>
+      </c>
       <c r="E44">
+        <f t="shared" si="13"/>
+        <v>0.32755195626238998</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="14"/>
+        <v>5.301018988964723E-2</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="15"/>
+        <v>5.3010189889647226</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="16"/>
+        <v>0.19308606697632957</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="17"/>
+        <v>19.308606697632957</v>
+      </c>
+      <c r="K44">
+        <f t="shared" si="18"/>
+        <v>-4.3664165853914194E-2</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="19"/>
+        <v>-4.3664165853914199</v>
+      </c>
+      <c r="N44">
+        <f t="shared" si="20"/>
+        <v>-0.11762464842578674</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="21"/>
+        <v>-11.762464842578673</v>
+      </c>
+      <c r="Q44">
         <f t="shared" si="11"/>
-        <v>0.32017835358857871</v>
-      </c>
-      <c r="F44">
+        <v>-7.727099196502718E-3</v>
+      </c>
+      <c r="R44">
+        <f t="shared" si="22"/>
+        <v>-0.7727099196502718</v>
+      </c>
+      <c r="T44">
         <f t="shared" si="12"/>
-        <v>4.5636587215835966E-2</v>
-      </c>
-      <c r="G44">
-        <f t="shared" si="13"/>
-        <v>4.5636587215835966</v>
-      </c>
-      <c r="H44">
-        <f t="shared" si="14"/>
-        <v>0.16622821299210119</v>
-      </c>
-      <c r="I44">
-        <f t="shared" si="15"/>
-        <v>16.62282129921012</v>
-      </c>
-      <c r="K44">
-        <f t="shared" si="16"/>
-        <v>-5.1037768527725458E-2</v>
-      </c>
-      <c r="L44">
-        <f t="shared" si="17"/>
-        <v>-5.1037768527725458</v>
-      </c>
-      <c r="N44">
-        <f t="shared" si="18"/>
-        <v>-0.13748801705259728</v>
-      </c>
-      <c r="O44">
-        <f t="shared" si="19"/>
-        <v>-13.748801705259728</v>
-      </c>
-      <c r="Q44">
-        <f>E44-K7</f>
-        <v>-1.5100701870313982E-2</v>
-      </c>
-      <c r="R44">
-        <f t="shared" si="20"/>
-        <v>-1.5100701870313982</v>
-      </c>
-      <c r="T44">
-        <f>Q44/K7</f>
-        <v>-4.5039204282074287E-2</v>
+        <v>-2.3046769759974193E-2</v>
       </c>
       <c r="U44">
-        <f t="shared" si="21"/>
-        <v>-4.5039204282074286</v>
+        <f t="shared" si="23"/>
+        <v>-2.3046769759974195</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -7450,60 +7483,66 @@
       <c r="B45">
         <v>0.67979355968595312</v>
       </c>
+      <c r="C45">
+        <v>0.68091892819859112</v>
+      </c>
+      <c r="D45">
+        <v>0.68116646643667378</v>
+      </c>
       <c r="E45">
+        <f t="shared" si="13"/>
+        <v>0.68062631810707275</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="14"/>
+        <v>7.2245895412616834E-2</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="15"/>
+        <v>7.2245895412616834</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="16"/>
+        <v>0.11875118382778822</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="17"/>
+        <v>11.875118382778822</v>
+      </c>
+      <c r="K45">
+        <f t="shared" si="18"/>
+        <v>5.56252228827947E-3</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="19"/>
+        <v>0.556252228827947</v>
+      </c>
+      <c r="N45">
+        <f t="shared" si="20"/>
+        <v>8.2399949793376462E-3</v>
+      </c>
+      <c r="O45">
+        <f t="shared" si="21"/>
+        <v>0.82399949793376459</v>
+      </c>
+      <c r="Q45">
         <f t="shared" si="11"/>
-        <v>0.67979355968595312</v>
-      </c>
-      <c r="F45">
-        <f t="shared" si="12"/>
-        <v>7.1413136991497206E-2</v>
-      </c>
-      <c r="G45">
-        <f t="shared" si="13"/>
-        <v>7.1413136991497206</v>
-      </c>
-      <c r="H45">
-        <f t="shared" si="14"/>
-        <v>0.11738237183112432</v>
-      </c>
-      <c r="I45">
-        <f t="shared" si="15"/>
-        <v>11.738237183112432</v>
-      </c>
-      <c r="K45">
-        <f t="shared" si="16"/>
-        <v>4.7297638671598419E-3</v>
-      </c>
-      <c r="L45">
-        <f t="shared" si="17"/>
-        <v>0.47297638671598419</v>
-      </c>
-      <c r="N45">
-        <f t="shared" si="18"/>
-        <v>7.0063953902653785E-3</v>
-      </c>
-      <c r="O45">
-        <f t="shared" si="19"/>
-        <v>0.70063953902653786</v>
-      </c>
-      <c r="Q45">
-        <f>E45-K8</f>
-        <v>6.8823710798776583E-2</v>
+        <v>6.9656469219896211E-2</v>
       </c>
       <c r="R45">
-        <f t="shared" si="20"/>
-        <v>6.8823710798776583</v>
+        <f t="shared" si="22"/>
+        <v>6.9656469219896211</v>
       </c>
       <c r="S45" t="s">
         <v>17</v>
       </c>
       <c r="T45">
-        <f>Q45/K8</f>
-        <v>0.11264665666257087</v>
+        <f t="shared" si="12"/>
+        <v>0.11400966732935977</v>
       </c>
       <c r="U45">
-        <f t="shared" si="21"/>
-        <v>11.264665666257088</v>
+        <f t="shared" si="23"/>
+        <v>11.400966732935977</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -7513,59 +7552,65 @@
       <c r="B46">
         <v>0.28677049279212952</v>
       </c>
+      <c r="C46">
+        <v>0.28677049279212952</v>
+      </c>
+      <c r="D46">
+        <v>0.28677049279212952</v>
+      </c>
       <c r="E46">
+        <f t="shared" si="13"/>
+        <v>0.28677049279212952</v>
+      </c>
+      <c r="F46">
+        <f t="shared" si="14"/>
+        <v>4.414033889770505E-2</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="15"/>
+        <v>4.4140338897705051</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="16"/>
+        <v>0.18192437415224083</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="17"/>
+        <v>18.192437415224084</v>
+      </c>
+      <c r="K46">
+        <f t="shared" si="18"/>
+        <v>1.4057367531604081E-2</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="19"/>
+        <v>1.4057367531604081</v>
+      </c>
+      <c r="N46">
+        <f t="shared" si="20"/>
+        <v>5.1546354867133527E-2</v>
+      </c>
+      <c r="O46">
+        <f t="shared" si="21"/>
+        <v>5.154635486713353</v>
+      </c>
+      <c r="Q46">
         <f t="shared" si="11"/>
-        <v>0.28677049279212952</v>
-      </c>
-      <c r="F46">
-        <f t="shared" si="12"/>
-        <v>4.414033889770505E-2</v>
-      </c>
-      <c r="G46">
-        <f t="shared" si="13"/>
-        <v>4.4140338897705051</v>
-      </c>
-      <c r="H46">
-        <f t="shared" si="14"/>
-        <v>0.18192437415224083</v>
-      </c>
-      <c r="I46">
-        <f t="shared" si="15"/>
-        <v>18.192437415224084</v>
-      </c>
-      <c r="K46">
-        <f t="shared" si="16"/>
-        <v>1.4057367531604081E-2</v>
-      </c>
-      <c r="L46">
-        <f t="shared" si="17"/>
-        <v>1.4057367531604081</v>
-      </c>
-      <c r="N46">
-        <f t="shared" si="18"/>
-        <v>5.1546354867133527E-2</v>
-      </c>
-      <c r="O46">
-        <f t="shared" si="19"/>
-        <v>5.154635486713353</v>
-      </c>
-      <c r="Q46">
-        <f>E46-K9</f>
         <v>1.7413030068079649E-2</v>
       </c>
       <c r="R46">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>1.7413030068079649</v>
       </c>
       <c r="S46" t="s">
         <v>17</v>
       </c>
       <c r="T46">
-        <f>Q46/K9</f>
+        <f t="shared" si="12"/>
         <v>6.4646547721303987E-2</v>
       </c>
       <c r="U46">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>6.4646547721303991</v>
       </c>
     </row>
@@ -7576,59 +7621,65 @@
       <c r="B47">
         <v>0.23999802768230441</v>
       </c>
+      <c r="C47">
+        <v>0.23999802768230441</v>
+      </c>
+      <c r="D47">
+        <v>0.23999802768230441</v>
+      </c>
       <c r="E47">
+        <f t="shared" si="13"/>
+        <v>0.23999802768230441</v>
+      </c>
+      <c r="F47">
+        <f t="shared" si="14"/>
+        <v>4.6261414885520991E-2</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="15"/>
+        <v>4.6261414885520988</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="16"/>
+        <v>0.23878509187133401</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="17"/>
+        <v>23.8785091871334</v>
+      </c>
+      <c r="K47">
+        <f t="shared" si="18"/>
+        <v>2.0740071728413439E-2</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="19"/>
+        <v>2.0740071728413438</v>
+      </c>
+      <c r="N47">
+        <f t="shared" si="20"/>
+        <v>9.4592105623638081E-2</v>
+      </c>
+      <c r="O47">
+        <f t="shared" si="21"/>
+        <v>9.4592105623638076</v>
+      </c>
+      <c r="Q47">
         <f t="shared" si="11"/>
-        <v>0.23999802768230441</v>
-      </c>
-      <c r="F47">
-        <f t="shared" si="12"/>
-        <v>4.6261414885520991E-2</v>
-      </c>
-      <c r="G47">
-        <f t="shared" si="13"/>
-        <v>4.6261414885520988</v>
-      </c>
-      <c r="H47">
-        <f t="shared" si="14"/>
-        <v>0.23878509187133401</v>
-      </c>
-      <c r="I47">
-        <f t="shared" si="15"/>
-        <v>23.8785091871334</v>
-      </c>
-      <c r="K47">
-        <f t="shared" si="16"/>
-        <v>2.0740071728413439E-2</v>
-      </c>
-      <c r="L47">
-        <f t="shared" si="17"/>
-        <v>2.0740071728413438</v>
-      </c>
-      <c r="N47">
-        <f t="shared" si="18"/>
-        <v>9.4592105623638081E-2</v>
-      </c>
-      <c r="O47">
-        <f t="shared" si="19"/>
-        <v>9.4592105623638076</v>
-      </c>
-      <c r="Q47">
-        <f>E47-K10</f>
         <v>1.824552814165753E-2</v>
       </c>
       <c r="R47">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>1.824552814165753</v>
       </c>
       <c r="S47" t="s">
         <v>17</v>
       </c>
       <c r="T47">
-        <f>Q47/K10</f>
+        <f t="shared" si="12"/>
         <v>8.2278793607524381E-2</v>
       </c>
       <c r="U47">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>8.2278793607524374</v>
       </c>
     </row>
@@ -7639,59 +7690,65 @@
       <c r="B48">
         <v>0.33447659015655518</v>
       </c>
+      <c r="C48">
+        <v>0.33447659015655518</v>
+      </c>
+      <c r="D48">
+        <v>0.33447659015655518</v>
+      </c>
       <c r="E48">
+        <f t="shared" si="13"/>
+        <v>0.33447659015655518</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="14"/>
+        <v>4.1975677013397217E-2</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="15"/>
+        <v>4.1975677013397217</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="16"/>
+        <v>0.1435061400743497</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="17"/>
+        <v>14.35061400743497</v>
+      </c>
+      <c r="K48">
+        <f t="shared" si="18"/>
+        <v>6.6841245125765503E-3</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="19"/>
+        <v>0.66841245125765503</v>
+      </c>
+      <c r="N48">
+        <f t="shared" si="20"/>
+        <v>2.0391330531179138E-2</v>
+      </c>
+      <c r="O48">
+        <f t="shared" si="21"/>
+        <v>2.0391330531179137</v>
+      </c>
+      <c r="Q48">
         <f t="shared" si="11"/>
-        <v>0.33447659015655518</v>
-      </c>
-      <c r="F48">
-        <f t="shared" si="12"/>
-        <v>4.1975677013397217E-2</v>
-      </c>
-      <c r="G48">
-        <f t="shared" si="13"/>
-        <v>4.1975677013397217</v>
-      </c>
-      <c r="H48">
-        <f t="shared" si="14"/>
-        <v>0.1435061400743497</v>
-      </c>
-      <c r="I48">
-        <f t="shared" si="15"/>
-        <v>14.35061400743497</v>
-      </c>
-      <c r="K48">
-        <f t="shared" si="16"/>
-        <v>6.6841245125765503E-3</v>
-      </c>
-      <c r="L48">
-        <f t="shared" si="17"/>
-        <v>0.66841245125765503</v>
-      </c>
-      <c r="N48">
-        <f t="shared" si="18"/>
-        <v>2.0391330531179138E-2</v>
-      </c>
-      <c r="O48">
-        <f t="shared" si="19"/>
-        <v>2.0391330531179137</v>
-      </c>
-      <c r="Q48">
-        <f>E48-K11</f>
         <v>1.7084439595540346E-2</v>
       </c>
       <c r="R48">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>1.7084439595540346</v>
       </c>
       <c r="S48" t="s">
         <v>17</v>
       </c>
       <c r="T48">
-        <f>Q48/K11</f>
+        <f t="shared" si="12"/>
         <v>5.3827542884542973E-2</v>
       </c>
       <c r="U48">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>5.3827542884542972</v>
       </c>
     </row>
@@ -7702,56 +7759,62 @@
       <c r="B49">
         <v>0.4653735632183908</v>
       </c>
+      <c r="C49">
+        <v>0.4653735632183908</v>
+      </c>
+      <c r="D49">
+        <v>0.4653735632183908</v>
+      </c>
       <c r="E49">
+        <f t="shared" si="13"/>
+        <v>0.4653735632183908</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="14"/>
+        <v>0.11340996168582373</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="15"/>
+        <v>11.340996168582373</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="16"/>
+        <v>0.32222071030072114</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="17"/>
+        <v>32.222071030072115</v>
+      </c>
+      <c r="K49">
+        <f t="shared" si="18"/>
+        <v>-8.4195402298850641E-2</v>
+      </c>
+      <c r="L49">
+        <f t="shared" si="19"/>
+        <v>-8.4195402298850635</v>
+      </c>
+      <c r="N49">
+        <f t="shared" si="20"/>
+        <v>-0.15320261437908508</v>
+      </c>
+      <c r="O49">
+        <f t="shared" si="21"/>
+        <v>-15.320261437908508</v>
+      </c>
+      <c r="Q49">
         <f t="shared" si="11"/>
-        <v>0.4653735632183908</v>
-      </c>
-      <c r="F49">
+        <v>-3.7404214559386972E-2</v>
+      </c>
+      <c r="R49">
+        <f t="shared" si="22"/>
+        <v>-3.740421455938697</v>
+      </c>
+      <c r="T49">
         <f t="shared" si="12"/>
-        <v>0.11340996168582373</v>
-      </c>
-      <c r="G49">
-        <f t="shared" si="13"/>
-        <v>11.340996168582373</v>
-      </c>
-      <c r="H49">
-        <f t="shared" si="14"/>
-        <v>0.32222071030072114</v>
-      </c>
-      <c r="I49">
-        <f t="shared" si="15"/>
-        <v>32.222071030072115</v>
-      </c>
-      <c r="K49">
-        <f t="shared" si="16"/>
-        <v>-8.4195402298850641E-2</v>
-      </c>
-      <c r="L49">
-        <f t="shared" si="17"/>
-        <v>-8.4195402298850635</v>
-      </c>
-      <c r="N49">
-        <f t="shared" si="18"/>
-        <v>-0.15320261437908508</v>
-      </c>
-      <c r="O49">
-        <f t="shared" si="19"/>
-        <v>-15.320261437908508</v>
-      </c>
-      <c r="Q49">
-        <f>E49-K12</f>
-        <v>-3.7404214559386972E-2</v>
-      </c>
-      <c r="R49">
-        <f t="shared" si="20"/>
-        <v>-3.740421455938697</v>
-      </c>
-      <c r="T49">
-        <f>Q49/K12</f>
         <v>-7.439512288054867E-2</v>
       </c>
       <c r="U49">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-7.4395122880548668</v>
       </c>
     </row>
@@ -7762,56 +7825,62 @@
       <c r="B50">
         <v>0.62931034482758619</v>
       </c>
+      <c r="C50">
+        <v>0.62931034482758619</v>
+      </c>
+      <c r="D50">
+        <v>0.62931034482758619</v>
+      </c>
       <c r="E50">
+        <f t="shared" si="13"/>
+        <v>0.62931034482758619</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="14"/>
+        <v>0.11206896551724133</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="15"/>
+        <v>11.206896551724132</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="16"/>
+        <v>0.21666666666666654</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="17"/>
+        <v>21.666666666666654</v>
+      </c>
+      <c r="K50">
+        <f t="shared" si="18"/>
+        <v>-7.4712643678160884E-2</v>
+      </c>
+      <c r="L50">
+        <f t="shared" si="19"/>
+        <v>-7.4712643678160884</v>
+      </c>
+      <c r="N50">
+        <f t="shared" si="20"/>
+        <v>-0.10612244897959179</v>
+      </c>
+      <c r="O50">
+        <f t="shared" si="21"/>
+        <v>-10.612244897959179</v>
+      </c>
+      <c r="Q50">
         <f t="shared" si="11"/>
-        <v>0.62931034482758619</v>
-      </c>
-      <c r="F50">
+        <v>-2.5862068965517238E-2</v>
+      </c>
+      <c r="R50">
+        <f t="shared" si="22"/>
+        <v>-2.5862068965517238</v>
+      </c>
+      <c r="T50">
         <f t="shared" si="12"/>
-        <v>0.11206896551724133</v>
-      </c>
-      <c r="G50">
-        <f t="shared" si="13"/>
-        <v>11.206896551724132</v>
-      </c>
-      <c r="H50">
-        <f t="shared" si="14"/>
-        <v>0.21666666666666654</v>
-      </c>
-      <c r="I50">
-        <f t="shared" si="15"/>
-        <v>21.666666666666654</v>
-      </c>
-      <c r="K50">
-        <f t="shared" si="16"/>
-        <v>-7.4712643678160884E-2</v>
-      </c>
-      <c r="L50">
-        <f t="shared" si="17"/>
-        <v>-7.4712643678160884</v>
-      </c>
-      <c r="N50">
-        <f t="shared" si="18"/>
-        <v>-0.10612244897959179</v>
-      </c>
-      <c r="O50">
-        <f t="shared" si="19"/>
-        <v>-10.612244897959179</v>
-      </c>
-      <c r="Q50">
-        <f>E50-K13</f>
-        <v>-2.5862068965517238E-2</v>
-      </c>
-      <c r="R50">
-        <f t="shared" si="20"/>
-        <v>-2.5862068965517238</v>
-      </c>
-      <c r="T50">
-        <f>Q50/K13</f>
         <v>-3.9473684210526314E-2</v>
       </c>
       <c r="U50">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>-3.9473684210526314</v>
       </c>
     </row>
@@ -7822,49 +7891,55 @@
       <c r="B51">
         <v>13.829238024251209</v>
       </c>
+      <c r="C51">
+        <v>13.240400398599689</v>
+      </c>
+      <c r="D51">
+        <v>13.17877932458088</v>
+      </c>
       <c r="E51">
+        <f t="shared" si="13"/>
+        <v>13.416139249143926</v>
+      </c>
+      <c r="F51">
+        <f t="shared" si="14"/>
+        <v>0.50390794838981634</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="15"/>
+        <v>50.390794838981634</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="16"/>
+        <v>3.9025629006536361E-2</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="17"/>
+        <v>3.9025629006536362</v>
+      </c>
+      <c r="K51">
+        <f t="shared" si="18"/>
+        <v>-0.14382008300430371</v>
+      </c>
+      <c r="N51">
+        <f t="shared" si="20"/>
+        <v>-1.0606232620722697E-2</v>
+      </c>
+      <c r="O51">
+        <f t="shared" si="21"/>
+        <v>-1.0606232620722698</v>
+      </c>
+      <c r="Q51">
         <f t="shared" si="11"/>
-        <v>13.829238024251209</v>
-      </c>
-      <c r="F51">
+        <v>0.68037395573210269</v>
+      </c>
+      <c r="T51">
         <f t="shared" si="12"/>
-        <v>0.91700672349709933</v>
-      </c>
-      <c r="G51">
-        <f t="shared" si="13"/>
-        <v>91.700672349709933</v>
-      </c>
-      <c r="H51">
-        <f t="shared" si="14"/>
-        <v>7.1018455458085203E-2</v>
-      </c>
-      <c r="I51">
-        <f t="shared" si="15"/>
-        <v>7.1018455458085201</v>
-      </c>
-      <c r="K51">
-        <f t="shared" si="16"/>
-        <v>0.26927869210297928</v>
-      </c>
-      <c r="N51">
-        <f t="shared" si="18"/>
-        <v>1.9858370184383065E-2</v>
-      </c>
-      <c r="O51">
-        <f t="shared" si="19"/>
-        <v>1.9858370184383065</v>
-      </c>
-      <c r="Q51">
-        <f>E51-K14</f>
-        <v>1.0934727308393857</v>
-      </c>
-      <c r="T51">
-        <f>Q51/K14</f>
-        <v>8.5858423553473937E-2</v>
+        <v>5.3422306399133965E-2</v>
       </c>
       <c r="U51">
-        <f t="shared" si="21"/>
-        <v>8.5858423553473937</v>
+        <f t="shared" si="23"/>
+        <v>5.3422306399133968</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -7874,49 +7949,55 @@
       <c r="B52">
         <v>2185.9396551724139</v>
       </c>
+      <c r="C52">
+        <v>2154.629310344827</v>
+      </c>
+      <c r="D52">
+        <v>2172.53448275862</v>
+      </c>
       <c r="E52">
+        <f t="shared" si="13"/>
+        <v>2171.03448275862</v>
+      </c>
+      <c r="F52">
+        <f t="shared" si="14"/>
+        <v>-11.43678160919626</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="15"/>
+        <v>-1143.678160919626</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="16"/>
+        <v>-5.2402896642531902E-3</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="17"/>
+        <v>-0.52402896642531904</v>
+      </c>
+      <c r="K52">
+        <f t="shared" si="18"/>
+        <v>-34.563218390805105</v>
+      </c>
+      <c r="N52">
+        <f t="shared" si="20"/>
+        <v>-1.5670681182154311E-2</v>
+      </c>
+      <c r="O52">
+        <f t="shared" si="21"/>
+        <v>-1.5670681182154311</v>
+      </c>
+      <c r="Q52">
         <f t="shared" si="11"/>
-        <v>2185.9396551724139</v>
-      </c>
-      <c r="F52">
+        <v>-18.362068965517665</v>
+      </c>
+      <c r="T52">
         <f t="shared" si="12"/>
-        <v>3.468390804597675</v>
-      </c>
-      <c r="G52">
-        <f t="shared" si="13"/>
-        <v>346.8390804597675</v>
-      </c>
-      <c r="H52">
-        <f t="shared" si="14"/>
-        <v>1.5892034233047937E-3</v>
-      </c>
-      <c r="I52">
-        <f t="shared" si="15"/>
-        <v>0.15892034233047939</v>
-      </c>
-      <c r="K52">
-        <f t="shared" si="16"/>
-        <v>-19.65804597701117</v>
-      </c>
-      <c r="N52">
-        <f t="shared" si="18"/>
-        <v>-8.9127976361086051E-3</v>
-      </c>
-      <c r="O52">
-        <f t="shared" si="19"/>
-        <v>-0.89127976361086048</v>
-      </c>
-      <c r="Q52">
-        <f>E52-K15</f>
-        <v>-3.4568965517237302</v>
-      </c>
-      <c r="T52">
-        <f>Q52/K15</f>
-        <v>-1.5789266448791304E-3</v>
+        <v>-8.3868173406309778E-3</v>
       </c>
       <c r="U52">
-        <f t="shared" si="21"/>
-        <v>-0.15789266448791303</v>
+        <f t="shared" si="23"/>
+        <v>-0.83868173406309776</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -7926,49 +8007,55 @@
       <c r="B53">
         <v>214.4568965517241</v>
       </c>
+      <c r="C53">
+        <v>211.55172413793099</v>
+      </c>
+      <c r="D53">
+        <v>214.66379310344831</v>
+      </c>
       <c r="E53">
+        <f t="shared" si="13"/>
+        <v>213.55747126436782</v>
+      </c>
+      <c r="F53">
+        <f t="shared" si="14"/>
+        <v>-6.3074712643677913</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="15"/>
+        <v>-630.74712643677913</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="16"/>
+        <v>-2.8687935383529487E-2</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="17"/>
+        <v>-2.8687935383529486</v>
+      </c>
+      <c r="K53">
+        <f t="shared" si="18"/>
+        <v>-8.4367816091954353</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="20"/>
+        <v>-3.8004504621120087E-2</v>
+      </c>
+      <c r="O53">
+        <f t="shared" si="21"/>
+        <v>-3.8004504621120088</v>
+      </c>
+      <c r="Q53">
         <f t="shared" si="11"/>
-        <v>214.4568965517241</v>
-      </c>
-      <c r="F53">
+        <v>-4.8390804597700878</v>
+      </c>
+      <c r="T53">
         <f t="shared" si="12"/>
-        <v>-5.4080459770115112</v>
-      </c>
-      <c r="G53">
-        <f t="shared" si="13"/>
-        <v>-540.80459770115112</v>
-      </c>
-      <c r="H53">
-        <f t="shared" si="14"/>
-        <v>-2.4597127285559395E-2</v>
-      </c>
-      <c r="I53">
-        <f t="shared" si="15"/>
-        <v>-2.4597127285559397</v>
-      </c>
-      <c r="K53">
-        <f t="shared" si="16"/>
-        <v>-7.5373563218391553</v>
-      </c>
-      <c r="N53">
-        <f t="shared" si="18"/>
-        <v>-3.3952934475885078E-2</v>
-      </c>
-      <c r="O53">
-        <f t="shared" si="19"/>
-        <v>-3.3952934475885077</v>
-      </c>
-      <c r="Q53">
-        <f>E53-K16</f>
-        <v>-3.9396551724138078</v>
-      </c>
-      <c r="T53">
-        <f>Q53/K16</f>
-        <v>-1.8038998973711286E-2</v>
+        <v>-2.2157311649693309E-2</v>
       </c>
       <c r="U53">
-        <f t="shared" si="21"/>
-        <v>-1.8038998973711287</v>
+        <f t="shared" si="23"/>
+        <v>-2.215731164969331</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -7978,49 +8065,55 @@
       <c r="B54">
         <v>2400.3965517241381</v>
       </c>
+      <c r="C54">
+        <v>2366.1810344827591</v>
+      </c>
+      <c r="D54">
+        <v>2387.1982758620688</v>
+      </c>
       <c r="E54">
+        <f t="shared" si="13"/>
+        <v>2384.5919540229884</v>
+      </c>
+      <c r="F54">
+        <f t="shared" si="14"/>
+        <v>-17.74425287356371</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="15"/>
+        <v>-1774.425287356371</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="16"/>
+        <v>-7.3862487784282903E-3</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="17"/>
+        <v>-0.73862487784282904</v>
+      </c>
+      <c r="K54">
+        <f t="shared" si="18"/>
+        <v>-43</v>
+      </c>
+      <c r="N54">
+        <f t="shared" si="20"/>
+        <v>-1.7713026247570436E-2</v>
+      </c>
+      <c r="O54">
+        <f t="shared" si="21"/>
+        <v>-1.7713026247570436</v>
+      </c>
+      <c r="Q54">
         <f t="shared" si="11"/>
-        <v>2400.3965517241381</v>
-      </c>
-      <c r="F54">
+        <v>-23.20114942528744</v>
+      </c>
+      <c r="T54">
         <f t="shared" si="12"/>
-        <v>-1.9396551724139499</v>
-      </c>
-      <c r="G54">
-        <f t="shared" si="13"/>
-        <v>-193.96551724139499</v>
-      </c>
-      <c r="H54">
-        <f t="shared" si="14"/>
-        <v>-8.0740371262175885E-4</v>
-      </c>
-      <c r="I54">
-        <f t="shared" si="15"/>
-        <v>-8.0740371262175883E-2</v>
-      </c>
-      <c r="K54">
-        <f t="shared" si="16"/>
-        <v>-27.19540229885024</v>
-      </c>
-      <c r="N54">
-        <f t="shared" si="18"/>
-        <v>-1.1202624993785389E-2</v>
-      </c>
-      <c r="O54">
-        <f t="shared" si="19"/>
-        <v>-1.1202624993785388</v>
-      </c>
-      <c r="Q54">
-        <f>E54-K17</f>
-        <v>-7.3965517241376801</v>
-      </c>
-      <c r="T54">
-        <f>Q54/K17</f>
-        <v>-3.0719216337752805E-3</v>
+        <v>-9.6358567486800866E-3</v>
       </c>
       <c r="U54">
-        <f t="shared" si="21"/>
-        <v>-0.30719216337752808</v>
+        <f t="shared" si="23"/>
+        <v>-0.96358567486800861</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -8030,9 +8123,15 @@
       <c r="B55">
         <v>11011.8275862069</v>
       </c>
+      <c r="C55">
+        <v>10804.71551724138</v>
+      </c>
+      <c r="D55">
+        <v>11011.8275862069</v>
+      </c>
       <c r="E55">
-        <f t="shared" si="11"/>
-        <v>11011.8275862069</v>
+        <f t="shared" si="13"/>
+        <v>10942.79022988506</v>
       </c>
     </row>
   </sheetData>
@@ -8785,7 +8884,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0763B57-AFAE-4268-833F-1978FDE50B6B}">
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -8793,7 +8892,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1">
-        <v>1000</v>
+        <v>1250</v>
       </c>
       <c r="B1">
         <v>300</v>
@@ -8817,1251 +8916,1142 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2" t="e">
+      <c r="B3">
+        <v>0.6948605865592562</v>
+      </c>
+      <c r="C3">
+        <v>0.6795021277889991</v>
+      </c>
+      <c r="D3">
+        <v>0.69120162991966927</v>
+      </c>
+      <c r="E3">
         <f>AVERAGE(B3:D3)</f>
-        <v>#DIV/0!</v>
+        <v>0.68852144808930815</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="e">
-        <f t="shared" ref="E4:E11" si="0">AVERAGE(B4:D4)</f>
-        <v>#DIV/0!</v>
+      <c r="B4">
+        <v>0.61038074712643686</v>
+      </c>
+      <c r="C4">
+        <v>0.60628591954023003</v>
+      </c>
+      <c r="D4">
+        <v>0.62047413793103445</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E17" si="0">AVERAGE(B4:D4)</f>
+        <v>0.61238026819923375</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="2" t="e">
+      <c r="B5">
+        <v>0.58406369729270291</v>
+      </c>
+      <c r="C5">
+        <v>0.5693366857997334</v>
+      </c>
+      <c r="D5">
+        <v>0.58335727966791839</v>
+      </c>
+      <c r="E5">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.57891922092011827</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="e">
+      <c r="B6">
+        <v>0.76445431250814044</v>
+      </c>
+      <c r="C6">
+        <v>0.76445431250814044</v>
+      </c>
+      <c r="D6">
+        <v>0.76445431250814044</v>
+      </c>
+      <c r="E6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.76445431250814044</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="2" t="e">
+      <c r="B7">
+        <v>0.24970583861541903</v>
+      </c>
+      <c r="C7">
+        <v>0.25233470207780773</v>
+      </c>
+      <c r="D7">
+        <v>0.25556369724652511</v>
+      </c>
+      <c r="E7">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.25253474597991726</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="2" t="e">
+      <c r="B8">
+        <v>0.62712365568616835</v>
+      </c>
+      <c r="C8">
+        <v>0.60685930765855134</v>
+      </c>
+      <c r="D8">
+        <v>0.59911507491363925</v>
+      </c>
+      <c r="E8">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.61103267941945294</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="2" t="e">
+      <c r="B9">
+        <v>0.33721264367816084</v>
+      </c>
+      <c r="C9">
+        <v>0.32859195402298852</v>
+      </c>
+      <c r="D9">
+        <v>0.33721264367816084</v>
+      </c>
+      <c r="E9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.33433908045977007</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="2" t="e">
+      <c r="B10">
+        <v>0.48275862068965519</v>
+      </c>
+      <c r="C10">
+        <v>0.47413793103448282</v>
+      </c>
+      <c r="D10">
+        <v>0.48275862068965519</v>
+      </c>
+      <c r="E10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.47988505747126436</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2" t="e">
+      <c r="B11" s="1">
+        <v>11.411141514778137</v>
+      </c>
+      <c r="C11">
+        <v>11.46074738584716</v>
+      </c>
+      <c r="D11">
+        <v>12.083573100895718</v>
+      </c>
+      <c r="E11">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>11.651820667173672</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12">
+        <v>0.24375483393669131</v>
+      </c>
+      <c r="C12">
+        <v>0.24375483393669131</v>
+      </c>
+      <c r="D12">
+        <v>0.24375483393669131</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0.24375483393669131</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>1250</v>
+      <c r="A13" t="s">
+        <v>22</v>
       </c>
       <c r="B13">
-        <v>300</v>
+        <v>0.18719576299190521</v>
+      </c>
+      <c r="C13">
+        <v>0.18719576299190521</v>
+      </c>
+      <c r="D13">
+        <v>0.18719576299190521</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0.18719576299190521</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D14" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" t="s">
-        <v>3</v>
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14">
+        <v>0.30106881260871893</v>
+      </c>
+      <c r="C14">
+        <v>0.30106881260871893</v>
+      </c>
+      <c r="D14">
+        <v>0.30106881260871893</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>0.30106881260871893</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B15">
-        <v>0.6948605865592562</v>
+        <v>286147</v>
       </c>
       <c r="C15">
-        <v>0.6795021277889991</v>
+        <v>276425</v>
       </c>
       <c r="D15">
-        <v>0.69120162991966927</v>
+        <v>276425</v>
       </c>
       <c r="E15">
-        <f>AVERAGE(B15:D15)</f>
-        <v>0.68852144808930815</v>
+        <f t="shared" si="0"/>
+        <v>279665.66666666669</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16">
+        <v>259700</v>
+      </c>
+      <c r="C16">
+        <v>250900</v>
+      </c>
+      <c r="D16">
+        <v>250900</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>253833.33333333334</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17">
+        <v>26447</v>
+      </c>
+      <c r="C17">
+        <f>C15-C16</f>
+        <v>25525</v>
+      </c>
+      <c r="D17">
+        <v>25525</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>25832.333333333332</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>1500</v>
+      </c>
+      <c r="B19">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>27</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21">
+        <v>0.66156887149880894</v>
+      </c>
+      <c r="C21">
+        <v>0.64893983549723122</v>
+      </c>
+      <c r="D21">
+        <v>0.67855384785151796</v>
+      </c>
+      <c r="E21">
+        <f>AVERAGE(B21:D21)</f>
+        <v>0.66302085161585278</v>
+      </c>
+      <c r="F21">
+        <f>E21-E3</f>
+        <v>-2.5500596473455373E-2</v>
+      </c>
+      <c r="G21">
+        <f>F21*100</f>
+        <v>-2.5500596473455373</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21">
+        <f>E21-E39</f>
+        <v>3.0136476105413368E-2</v>
+      </c>
+      <c r="J21">
+        <f>I21*100</f>
+        <v>3.0136476105413368</v>
+      </c>
+      <c r="K21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>5</v>
       </c>
-      <c r="B16">
-        <v>0.61038074712643686</v>
-      </c>
-      <c r="C16">
-        <v>0.60628591954023003</v>
-      </c>
-      <c r="D16">
-        <v>0.62047413793103445</v>
-      </c>
-      <c r="E16">
-        <f t="shared" ref="E16:E29" si="1">AVERAGE(B16:D16)</f>
-        <v>0.61238026819923375</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B22">
+        <v>0.62444581280788181</v>
+      </c>
+      <c r="C22">
+        <v>0.6359400656814449</v>
+      </c>
+      <c r="D22">
+        <v>0.63349753694581279</v>
+      </c>
+      <c r="E22">
+        <f t="shared" ref="E22:E35" si="1">AVERAGE(B22:D22)</f>
+        <v>0.63129447181171316</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22:F35" si="2">E22-E4</f>
+        <v>1.8914203612479419E-2</v>
+      </c>
+      <c r="G22">
+        <f t="shared" ref="G22:G32" si="3">F22*100</f>
+        <v>1.8914203612479419</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22:I35" si="4">E22-E40</f>
+        <v>-3.4325396825396925E-2</v>
+      </c>
+      <c r="J22">
+        <f t="shared" ref="J22:J32" si="5">I22*100</f>
+        <v>-3.4325396825396925</v>
+      </c>
+      <c r="K22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>6</v>
       </c>
-      <c r="B17">
-        <v>0.58406369729270291</v>
-      </c>
-      <c r="C17">
-        <v>0.5693366857997334</v>
-      </c>
-      <c r="D17">
-        <v>0.58335727966791839</v>
-      </c>
-      <c r="E17">
-        <f t="shared" si="1"/>
-        <v>0.57891922092011827</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18">
-        <v>0.76445431250814044</v>
-      </c>
-      <c r="C18">
-        <v>0.76445431250814044</v>
-      </c>
-      <c r="D18">
-        <v>0.76445431250814044</v>
-      </c>
-      <c r="E18">
-        <f t="shared" si="1"/>
-        <v>0.76445431250814044</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19">
-        <v>0.24970583861541903</v>
-      </c>
-      <c r="C19">
-        <v>0.25233470207780773</v>
-      </c>
-      <c r="D19">
-        <v>0.25556369724652511</v>
-      </c>
-      <c r="E19">
-        <f t="shared" si="1"/>
-        <v>0.25253474597991726</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20">
-        <v>0.62712365568616835</v>
-      </c>
-      <c r="C20">
-        <v>0.60685930765855134</v>
-      </c>
-      <c r="D20">
-        <v>0.59911507491363925</v>
-      </c>
-      <c r="E20">
-        <f t="shared" si="1"/>
-        <v>0.61103267941945294</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21">
-        <v>0.33721264367816084</v>
-      </c>
-      <c r="C21">
-        <v>0.32859195402298852</v>
-      </c>
-      <c r="D21">
-        <v>0.33721264367816084</v>
-      </c>
-      <c r="E21">
-        <f t="shared" si="1"/>
-        <v>0.33433908045977007</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22">
-        <v>0.48275862068965519</v>
-      </c>
-      <c r="C22">
-        <v>0.47413793103448282</v>
-      </c>
-      <c r="D22">
-        <v>0.48275862068965519</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="1"/>
-        <v>0.47988505747126436</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="1">
-        <v>11.411141514778137</v>
+      <c r="B23">
+        <v>0.62411398464630674</v>
       </c>
       <c r="C23">
-        <v>11.46074738584716</v>
+        <v>0.63705699230932178</v>
       </c>
       <c r="D23">
-        <v>12.083573100895718</v>
+        <v>0.63023227966371942</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
-        <v>11.651820667173672</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.63046775220644935</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="2"/>
+        <v>5.1548531286331079E-2</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="3"/>
+        <v>5.1548531286331079</v>
+      </c>
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="4"/>
+        <v>2.7009134319842976E-2</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="5"/>
+        <v>2.7009134319842976</v>
+      </c>
+      <c r="K23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B24">
-        <v>0.24375483393669131</v>
+        <v>0.75927595016951388</v>
       </c>
       <c r="C24">
-        <v>0.24375483393669131</v>
+        <v>0.75921113559346654</v>
       </c>
       <c r="D24">
-        <v>0.24375483393669131</v>
+        <v>0.7619412322559872</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
-        <v>0.24375483393669131</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.76014277267298924</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="2"/>
+        <v>-4.3115398351512013E-3</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="3"/>
+        <v>-0.43115398351512013</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="4"/>
+        <v>6.8738746768439718E-3</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="5"/>
+        <v>0.68738746768439718</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B25">
-        <v>0.18719576299190521</v>
+        <v>0.27292447328324371</v>
       </c>
       <c r="C25">
-        <v>0.18719576299190521</v>
+        <v>0.27091359774604223</v>
       </c>
       <c r="D25">
-        <v>0.18719576299190521</v>
+        <v>0.27978722808894224</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
-        <v>0.18719576299190521</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.27454176637274275</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="2"/>
+        <v>2.2007020392825483E-2</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="3"/>
+        <v>2.2007020392825485</v>
+      </c>
+      <c r="H25" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="4"/>
+        <v>2.2588670506993092E-2</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="5"/>
+        <v>2.2588670506993092</v>
+      </c>
+      <c r="K25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B26">
-        <v>0.30106881260871893</v>
+        <v>0.59892572244511921</v>
       </c>
       <c r="C26">
-        <v>0.30106881260871893</v>
+        <v>0.59085822927043607</v>
       </c>
       <c r="D26">
-        <v>0.30106881260871893</v>
+        <v>0.63535731636781256</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
-        <v>0.30106881260871893</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.60838042269445591</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="2"/>
+        <v>-2.6522567249970264E-3</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="3"/>
+        <v>-0.26522567249970264</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="4"/>
+        <v>-1.5621164082773253E-2</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="5"/>
+        <v>-1.5621164082773253</v>
+      </c>
+      <c r="K26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="B27">
-        <v>286147</v>
+        <v>0.3466954022988506</v>
       </c>
       <c r="C27">
-        <v>276425</v>
+        <v>0.34885057471264369</v>
       </c>
       <c r="D27">
-        <v>276425</v>
+        <v>0.3603448275862069</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
-        <v>279665.66666666669</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.35196360153256706</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="2"/>
+        <v>1.7624521072796995E-2</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="3"/>
+        <v>1.7624521072796995</v>
+      </c>
+      <c r="H27" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="4"/>
+        <v>9.1762452107279679E-2</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="5"/>
+        <v>9.1762452107279682</v>
+      </c>
+      <c r="K27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B28">
-        <v>259700</v>
+        <v>0.50862068965517238</v>
       </c>
       <c r="C28">
-        <v>250900</v>
+        <v>0.51724137931034486</v>
       </c>
       <c r="D28">
-        <v>250900</v>
+        <v>0.52586206896551724</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
-        <v>253833.33333333334</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.51724137931034486</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="2"/>
+        <v>3.7356321839080497E-2</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="3"/>
+        <v>3.7356321839080495</v>
+      </c>
+      <c r="H28" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="4"/>
+        <v>0.10632183908045978</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="5"/>
+        <v>10.632183908045977</v>
+      </c>
+      <c r="K28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B29">
-        <v>26447</v>
-      </c>
-      <c r="C29">
-        <f>C27-C28</f>
-        <v>25525</v>
+        <v>12.829803801816089</v>
+      </c>
+      <c r="C29" s="1">
+        <v>13.84695393052594</v>
       </c>
       <c r="D29">
-        <v>25525</v>
+        <v>12.0599361699203</v>
       </c>
       <c r="E29">
         <f t="shared" si="1"/>
-        <v>25832.333333333332</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>1500</v>
+        <v>12.91223130075411</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="2"/>
+        <v>1.2604106335804381</v>
+      </c>
+      <c r="G29">
+        <f>F29</f>
+        <v>1.2604106335804381</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="4"/>
+        <v>1.4224990633712427</v>
+      </c>
+      <c r="J29">
+        <f>I29</f>
+        <v>1.4224990633712427</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30">
+        <v>0.24309878051280981</v>
+      </c>
+      <c r="C30">
+        <v>0.23840367794036871</v>
+      </c>
+      <c r="D30">
+        <v>0.24638800323009491</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="1"/>
+        <v>0.24263015389442447</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="2"/>
+        <v>-1.1246800422668457E-3</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="3"/>
+        <v>-0.11246800422668457</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="4"/>
+        <v>1.1235088109970204E-2</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="5"/>
+        <v>1.1235088109970204</v>
+      </c>
+      <c r="K30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
       </c>
       <c r="B31">
+        <v>0.19543476402759549</v>
+      </c>
+      <c r="C31">
+        <v>0.18611909449100489</v>
+      </c>
+      <c r="D31">
+        <v>0.19965597987174991</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="1"/>
+        <v>0.19373661279678342</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="2"/>
+        <v>6.5408498048782071E-3</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="3"/>
+        <v>0.65408498048782071</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="4"/>
+        <v>1.3529345393180819E-2</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="5"/>
+        <v>1.3529345393180821</v>
+      </c>
+      <c r="K31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32">
+        <v>0.29144790768623352</v>
+      </c>
+      <c r="C32">
+        <v>0.29186853766441351</v>
+      </c>
+      <c r="D32">
+        <v>0.2941862940788269</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="1"/>
+        <v>0.29250091314315796</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="2"/>
+        <v>-8.5678994655609686E-3</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="3"/>
+        <v>-0.85678994655609686</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="4"/>
+        <v>9.7643733024597723E-3</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="5"/>
+        <v>0.97643733024597723</v>
+      </c>
+      <c r="K32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33">
+        <v>284126</v>
+      </c>
+      <c r="C33" s="1">
+        <v>276230</v>
+      </c>
+      <c r="D33">
+        <v>275657</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="1"/>
+        <v>278671</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="2"/>
+        <v>-994.66666666668607</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="4"/>
+        <v>-3729</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34">
+        <v>258300</v>
+      </c>
+      <c r="C34" s="1">
+        <v>250500</v>
+      </c>
+      <c r="D34">
+        <v>250700</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="1"/>
+        <v>253166.66666666666</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="2"/>
+        <v>-666.66666666668607</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="4"/>
+        <v>-2433.333333333343</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35">
+        <v>25826</v>
+      </c>
+      <c r="C35" s="1">
+        <v>25730</v>
+      </c>
+      <c r="D35">
+        <v>24957</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="1"/>
+        <v>25504.333333333332</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="2"/>
+        <v>-328</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="4"/>
+        <v>-1295.6666666666679</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>1750</v>
+      </c>
+      <c r="B37">
         <v>300</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
         <v>0</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C38" t="s">
         <v>1</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D38" t="s">
         <v>2</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E38" t="s">
         <v>3</v>
       </c>
-      <c r="F32" t="s">
-        <v>27</v>
-      </c>
-      <c r="G32" t="s">
-        <v>14</v>
-      </c>
-      <c r="I32" t="s">
-        <v>28</v>
-      </c>
-      <c r="J32" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>4</v>
       </c>
-      <c r="B33">
-        <v>0.66156887149880894</v>
-      </c>
-      <c r="C33">
-        <v>0.64893983549723122</v>
-      </c>
-      <c r="D33">
-        <v>0.67855384785151796</v>
-      </c>
-      <c r="E33">
-        <f>AVERAGE(B33:D33)</f>
-        <v>0.66302085161585278</v>
-      </c>
-      <c r="F33">
-        <f>E33-E15</f>
-        <v>-2.5500596473455373E-2</v>
-      </c>
-      <c r="G33">
-        <f>F33*100</f>
-        <v>-2.5500596473455373</v>
-      </c>
-      <c r="H33" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33">
-        <f>E33-E51</f>
-        <v>3.0136476105413368E-2</v>
-      </c>
-      <c r="J33">
-        <f>I33*100</f>
-        <v>3.0136476105413368</v>
-      </c>
-      <c r="K33" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B39">
+        <v>0.62963137009189651</v>
+      </c>
+      <c r="C39">
+        <v>0.62900901409001886</v>
+      </c>
+      <c r="D39">
+        <v>0.64001274234940275</v>
+      </c>
+      <c r="E39">
+        <f>AVERAGE(B39:D39)</f>
+        <v>0.63288437551043941</v>
+      </c>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>5</v>
       </c>
-      <c r="B34">
-        <v>0.62444581280788181</v>
-      </c>
-      <c r="C34">
-        <v>0.6359400656814449</v>
-      </c>
-      <c r="D34">
-        <v>0.63349753694581279</v>
-      </c>
-      <c r="E34">
-        <f t="shared" ref="E34:E47" si="2">AVERAGE(B34:D34)</f>
-        <v>0.63129447181171316</v>
-      </c>
-      <c r="F34">
-        <f t="shared" ref="F34:F47" si="3">E34-E16</f>
-        <v>1.8914203612479419E-2</v>
-      </c>
-      <c r="G34">
-        <f t="shared" ref="G34:G44" si="4">F34*100</f>
-        <v>1.8914203612479419</v>
-      </c>
-      <c r="H34" t="s">
-        <v>17</v>
-      </c>
-      <c r="I34">
-        <f t="shared" ref="I34:I47" si="5">E34-E52</f>
-        <v>-3.4325396825396925E-2</v>
-      </c>
-      <c r="J34">
-        <f t="shared" ref="J34:J44" si="6">I34*100</f>
-        <v>-3.4325396825396925</v>
-      </c>
-      <c r="K34" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B40">
+        <v>0.6554187192118226</v>
+      </c>
+      <c r="C40">
+        <v>0.656568144499179</v>
+      </c>
+      <c r="D40">
+        <v>0.68487274220032857</v>
+      </c>
+      <c r="E40">
+        <f t="shared" ref="E40:E53" si="6">AVERAGE(B40:D40)</f>
+        <v>0.66561986863711009</v>
+      </c>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>6</v>
       </c>
-      <c r="B35">
-        <v>0.62411398464630674</v>
-      </c>
-      <c r="C35">
-        <v>0.63705699230932178</v>
-      </c>
-      <c r="D35">
-        <v>0.63023227966371942</v>
-      </c>
-      <c r="E35">
-        <f t="shared" si="2"/>
-        <v>0.63046775220644935</v>
-      </c>
-      <c r="F35">
-        <f t="shared" si="3"/>
-        <v>5.1548531286331079E-2</v>
-      </c>
-      <c r="G35">
-        <f t="shared" si="4"/>
-        <v>5.1548531286331079</v>
-      </c>
-      <c r="H35" t="s">
-        <v>17</v>
-      </c>
-      <c r="I35">
-        <f t="shared" si="5"/>
-        <v>2.7009134319842976E-2</v>
-      </c>
-      <c r="J35">
+      <c r="B41">
+        <v>0.58686542143005738</v>
+      </c>
+      <c r="C41">
+        <v>0.61296695399601808</v>
+      </c>
+      <c r="D41">
+        <v>0.61054347823374377</v>
+      </c>
+      <c r="E41">
         <f t="shared" si="6"/>
-        <v>2.7009134319842976</v>
-      </c>
-      <c r="K35" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+        <v>0.60345861788660637</v>
+      </c>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>7</v>
       </c>
-      <c r="B36">
-        <v>0.75927595016951388</v>
-      </c>
-      <c r="C36">
-        <v>0.75921113559346654</v>
-      </c>
-      <c r="D36">
-        <v>0.7619412322559872</v>
-      </c>
-      <c r="E36">
-        <f t="shared" si="2"/>
-        <v>0.76014277267298924</v>
-      </c>
-      <c r="F36">
-        <f t="shared" si="3"/>
-        <v>-4.3115398351512013E-3</v>
-      </c>
-      <c r="G36">
-        <f t="shared" si="4"/>
-        <v>-0.43115398351512013</v>
-      </c>
-      <c r="I36">
-        <f t="shared" si="5"/>
-        <v>6.8738746768439718E-3</v>
-      </c>
-      <c r="J36">
+      <c r="B42">
+        <v>0.75326889799614516</v>
+      </c>
+      <c r="C42">
+        <v>0.75326889799614549</v>
+      </c>
+      <c r="D42">
+        <v>0.75326889799614549</v>
+      </c>
+      <c r="E42">
         <f t="shared" si="6"/>
-        <v>0.68738746768439718</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+        <v>0.75326889799614527</v>
+      </c>
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>8</v>
       </c>
-      <c r="B37">
-        <v>0.27292447328324371</v>
-      </c>
-      <c r="C37">
-        <v>0.27091359774604223</v>
-      </c>
-      <c r="D37">
-        <v>0.27978722808894224</v>
-      </c>
-      <c r="E37">
-        <f t="shared" si="2"/>
-        <v>0.27454176637274275</v>
-      </c>
-      <c r="F37">
-        <f t="shared" si="3"/>
-        <v>2.2007020392825483E-2</v>
-      </c>
-      <c r="G37">
-        <f t="shared" si="4"/>
-        <v>2.2007020392825485</v>
-      </c>
-      <c r="H37" t="s">
-        <v>17</v>
-      </c>
-      <c r="I37">
-        <f t="shared" si="5"/>
-        <v>2.2588670506993092E-2</v>
-      </c>
-      <c r="J37">
+      <c r="B43">
+        <v>0.24553750941061361</v>
+      </c>
+      <c r="C43">
+        <v>0.26164240439793229</v>
+      </c>
+      <c r="D43">
+        <v>0.24867937378870311</v>
+      </c>
+      <c r="E43">
         <f t="shared" si="6"/>
-        <v>2.2588670506993092</v>
-      </c>
-      <c r="K37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+        <v>0.25195309586574965</v>
+      </c>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>9</v>
       </c>
-      <c r="B38">
-        <v>0.59892572244511921</v>
-      </c>
-      <c r="C38">
-        <v>0.59085822927043607</v>
-      </c>
-      <c r="D38">
-        <v>0.63535731636781256</v>
-      </c>
-      <c r="E38">
-        <f t="shared" si="2"/>
-        <v>0.60838042269445591</v>
-      </c>
-      <c r="F38">
-        <f t="shared" si="3"/>
-        <v>-2.6522567249970264E-3</v>
-      </c>
-      <c r="G38">
-        <f t="shared" si="4"/>
-        <v>-0.26522567249970264</v>
-      </c>
-      <c r="I38">
-        <f t="shared" si="5"/>
-        <v>-1.5621164082773253E-2</v>
-      </c>
-      <c r="J38">
+      <c r="B44">
+        <v>0.60933495101680679</v>
+      </c>
+      <c r="C44">
+        <v>0.63147614145716247</v>
+      </c>
+      <c r="D44">
+        <v>0.63119366785771835</v>
+      </c>
+      <c r="E44">
         <f t="shared" si="6"/>
-        <v>-1.5621164082773253</v>
-      </c>
-      <c r="K38" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+        <v>0.62400158677722917</v>
+      </c>
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>10</v>
       </c>
-      <c r="B39">
-        <v>0.3466954022988506</v>
-      </c>
-      <c r="C39">
-        <v>0.34885057471264369</v>
-      </c>
-      <c r="D39">
-        <v>0.3603448275862069</v>
-      </c>
-      <c r="E39">
-        <f t="shared" si="2"/>
-        <v>0.35196360153256706</v>
-      </c>
-      <c r="F39">
-        <f t="shared" si="3"/>
-        <v>1.7624521072796995E-2</v>
-      </c>
-      <c r="G39">
-        <f t="shared" si="4"/>
-        <v>1.7624521072796995</v>
-      </c>
-      <c r="H39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I39">
-        <f t="shared" si="5"/>
-        <v>9.1762452107279679E-2</v>
-      </c>
-      <c r="J39">
+      <c r="B45">
+        <v>0.26307471264367821</v>
+      </c>
+      <c r="C45">
+        <v>0.25445402298850572</v>
+      </c>
+      <c r="D45">
+        <v>0.26307471264367821</v>
+      </c>
+      <c r="E45">
         <f t="shared" si="6"/>
-        <v>9.1762452107279682</v>
-      </c>
-      <c r="K39" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+        <v>0.26020114942528738</v>
+      </c>
+      <c r="F45" s="2"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>11</v>
       </c>
-      <c r="B40">
-        <v>0.50862068965517238</v>
-      </c>
-      <c r="C40">
-        <v>0.51724137931034486</v>
-      </c>
-      <c r="D40">
-        <v>0.52586206896551724</v>
-      </c>
-      <c r="E40">
-        <f t="shared" si="2"/>
-        <v>0.51724137931034486</v>
-      </c>
-      <c r="F40">
-        <f t="shared" si="3"/>
-        <v>3.7356321839080497E-2</v>
-      </c>
-      <c r="G40">
-        <f t="shared" si="4"/>
-        <v>3.7356321839080495</v>
-      </c>
-      <c r="H40" t="s">
-        <v>17</v>
-      </c>
-      <c r="I40">
-        <f t="shared" si="5"/>
-        <v>0.10632183908045978</v>
-      </c>
-      <c r="J40">
+      <c r="B46">
+        <v>0.41379310344827591</v>
+      </c>
+      <c r="C46">
+        <v>0.40517241379310343</v>
+      </c>
+      <c r="D46">
+        <v>0.41379310344827591</v>
+      </c>
+      <c r="E46">
         <f t="shared" si="6"/>
-        <v>10.632183908045977</v>
-      </c>
-      <c r="K40" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+        <v>0.41091954022988508</v>
+      </c>
+      <c r="F46" s="2"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>12</v>
       </c>
-      <c r="B41">
-        <v>12.829803801816089</v>
-      </c>
-      <c r="C41" s="1">
-        <v>13.84695393052594</v>
-      </c>
-      <c r="D41">
-        <v>12.0599361699203</v>
-      </c>
-      <c r="E41">
-        <f t="shared" si="2"/>
-        <v>12.91223130075411</v>
-      </c>
-      <c r="F41">
-        <f t="shared" si="3"/>
-        <v>1.2604106335804381</v>
-      </c>
-      <c r="G41">
-        <f>F41</f>
-        <v>1.2604106335804381</v>
-      </c>
-      <c r="H41" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41">
-        <f t="shared" si="5"/>
-        <v>1.4224990633712427</v>
-      </c>
-      <c r="J41">
-        <f>I41</f>
-        <v>1.4224990633712427</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B47" s="1">
+        <v>11.927592316578171</v>
+      </c>
+      <c r="C47" s="1">
+        <v>11.35648157267735</v>
+      </c>
+      <c r="D47">
+        <v>11.18512282289308</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="6"/>
+        <v>11.489732237382867</v>
+      </c>
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>21</v>
       </c>
-      <c r="B42">
-        <v>0.24309878051280981</v>
-      </c>
-      <c r="C42">
-        <v>0.23840367794036871</v>
-      </c>
-      <c r="D42">
-        <v>0.24638800323009491</v>
-      </c>
-      <c r="E42">
-        <f t="shared" si="2"/>
-        <v>0.24263015389442447</v>
-      </c>
-      <c r="F42">
-        <f t="shared" si="3"/>
-        <v>-1.1246800422668457E-3</v>
-      </c>
-      <c r="G42">
-        <f t="shared" si="4"/>
-        <v>-0.11246800422668457</v>
-      </c>
-      <c r="I42">
-        <f t="shared" si="5"/>
-        <v>1.1235088109970204E-2</v>
-      </c>
-      <c r="J42">
+      <c r="B48">
+        <v>0.23139506578445429</v>
+      </c>
+      <c r="C48">
+        <v>0.23139506578445429</v>
+      </c>
+      <c r="D48">
+        <v>0.23139506578445429</v>
+      </c>
+      <c r="E48">
         <f t="shared" si="6"/>
-        <v>1.1235088109970204</v>
-      </c>
-      <c r="K42" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+        <v>0.23139506578445426</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>22</v>
       </c>
-      <c r="B43">
-        <v>0.19543476402759549</v>
-      </c>
-      <c r="C43">
-        <v>0.18611909449100489</v>
-      </c>
-      <c r="D43">
-        <v>0.19965597987174991</v>
-      </c>
-      <c r="E43">
-        <f t="shared" si="2"/>
-        <v>0.19373661279678342</v>
-      </c>
-      <c r="F43">
-        <f t="shared" si="3"/>
-        <v>6.5408498048782071E-3</v>
-      </c>
-      <c r="G43">
-        <f t="shared" si="4"/>
-        <v>0.65408498048782071</v>
-      </c>
-      <c r="I43">
-        <f t="shared" si="5"/>
-        <v>1.3529345393180819E-2</v>
-      </c>
-      <c r="J43">
+      <c r="B49">
+        <v>0.1802072674036026</v>
+      </c>
+      <c r="C49">
+        <v>0.1802072674036026</v>
+      </c>
+      <c r="D49">
+        <v>0.1802072674036026</v>
+      </c>
+      <c r="E49">
         <f t="shared" si="6"/>
-        <v>1.3529345393180821</v>
-      </c>
-      <c r="K43" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+        <v>0.1802072674036026</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>23</v>
       </c>
-      <c r="B44">
-        <v>0.29144790768623352</v>
-      </c>
-      <c r="C44">
-        <v>0.29186853766441351</v>
-      </c>
-      <c r="D44">
-        <v>0.2941862940788269</v>
-      </c>
-      <c r="E44">
-        <f t="shared" si="2"/>
-        <v>0.29250091314315796</v>
-      </c>
-      <c r="F44">
-        <f t="shared" si="3"/>
-        <v>-8.5678994655609686E-3</v>
-      </c>
-      <c r="G44">
-        <f t="shared" si="4"/>
-        <v>-0.85678994655609686</v>
-      </c>
-      <c r="I44">
-        <f t="shared" si="5"/>
-        <v>9.7643733024597723E-3</v>
-      </c>
-      <c r="J44">
+      <c r="B50">
+        <v>0.28273653984069819</v>
+      </c>
+      <c r="C50">
+        <v>0.28273653984069819</v>
+      </c>
+      <c r="D50">
+        <v>0.28273653984069819</v>
+      </c>
+      <c r="E50">
         <f t="shared" si="6"/>
-        <v>0.97643733024597723</v>
-      </c>
-      <c r="K44" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+        <v>0.28273653984069819</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>24</v>
       </c>
-      <c r="B45">
-        <v>284126</v>
-      </c>
-      <c r="C45" s="1">
-        <v>276230</v>
-      </c>
-      <c r="D45">
-        <v>275657</v>
-      </c>
-      <c r="E45">
-        <f t="shared" si="2"/>
-        <v>278671</v>
-      </c>
-      <c r="F45">
-        <f t="shared" si="3"/>
-        <v>-994.66666666668607</v>
-      </c>
-      <c r="I45">
-        <f t="shared" si="5"/>
-        <v>-3729</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="B51">
+        <v>282400</v>
+      </c>
+      <c r="C51">
+        <v>282400</v>
+      </c>
+      <c r="D51">
+        <v>282400</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="6"/>
+        <v>282400</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>25</v>
       </c>
-      <c r="B46">
-        <v>258300</v>
-      </c>
-      <c r="C46" s="1">
-        <v>250500</v>
-      </c>
-      <c r="D46">
-        <v>250700</v>
-      </c>
-      <c r="E46">
-        <f t="shared" si="2"/>
-        <v>253166.66666666666</v>
-      </c>
-      <c r="F46">
-        <f t="shared" si="3"/>
-        <v>-666.66666666668607</v>
-      </c>
-      <c r="I46">
-        <f t="shared" si="5"/>
-        <v>-2433.333333333343</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="B52">
+        <v>255600</v>
+      </c>
+      <c r="C52">
+        <v>255600</v>
+      </c>
+      <c r="D52">
+        <v>255600</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="6"/>
+        <v>255600</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>26</v>
       </c>
-      <c r="B47">
-        <v>25826</v>
-      </c>
-      <c r="C47" s="1">
-        <v>25730</v>
-      </c>
-      <c r="D47">
-        <v>24957</v>
-      </c>
-      <c r="E47">
-        <f t="shared" si="2"/>
-        <v>25504.333333333332</v>
-      </c>
-      <c r="F47">
-        <f t="shared" si="3"/>
-        <v>-328</v>
-      </c>
-      <c r="I47">
-        <f t="shared" si="5"/>
-        <v>-1295.6666666666679</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>1750</v>
-      </c>
-      <c r="B49">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
-        <v>0</v>
-      </c>
-      <c r="C50" t="s">
-        <v>1</v>
-      </c>
-      <c r="D50" t="s">
-        <v>2</v>
-      </c>
-      <c r="E50" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>4</v>
-      </c>
-      <c r="B51">
-        <v>0.62963137009189651</v>
-      </c>
-      <c r="C51">
-        <v>0.62900901409001886</v>
-      </c>
-      <c r="D51">
-        <v>0.64001274234940275</v>
-      </c>
-      <c r="E51">
-        <f>AVERAGE(B51:D51)</f>
-        <v>0.63288437551043941</v>
-      </c>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>5</v>
-      </c>
-      <c r="B52">
-        <v>0.6554187192118226</v>
-      </c>
-      <c r="C52">
-        <v>0.656568144499179</v>
-      </c>
-      <c r="D52">
-        <v>0.68487274220032857</v>
-      </c>
-      <c r="E52">
-        <f t="shared" ref="E52:E65" si="7">AVERAGE(B52:D52)</f>
-        <v>0.66561986863711009</v>
-      </c>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>6</v>
-      </c>
       <c r="B53">
-        <v>0.58686542143005738</v>
+        <v>26800</v>
       </c>
       <c r="C53">
-        <v>0.61296695399601808</v>
+        <v>26800</v>
       </c>
       <c r="D53">
-        <v>0.61054347823374377</v>
+        <v>26800</v>
       </c>
       <c r="E53">
-        <f t="shared" si="7"/>
-        <v>0.60345861788660637</v>
-      </c>
-      <c r="F53" s="2"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>7</v>
-      </c>
-      <c r="B54">
-        <v>0.75326889799614516</v>
-      </c>
-      <c r="C54">
-        <v>0.75326889799614549</v>
-      </c>
-      <c r="D54">
-        <v>0.75326889799614549</v>
-      </c>
-      <c r="E54">
-        <f t="shared" si="7"/>
-        <v>0.75326889799614527</v>
-      </c>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>8</v>
-      </c>
-      <c r="B55">
-        <v>0.24553750941061361</v>
-      </c>
-      <c r="C55">
-        <v>0.26164240439793229</v>
-      </c>
-      <c r="D55">
-        <v>0.24867937378870311</v>
-      </c>
-      <c r="E55">
-        <f t="shared" si="7"/>
-        <v>0.25195309586574965</v>
-      </c>
-      <c r="F55" s="2"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>9</v>
-      </c>
-      <c r="B56">
-        <v>0.60933495101680679</v>
-      </c>
-      <c r="C56">
-        <v>0.63147614145716247</v>
-      </c>
-      <c r="D56">
-        <v>0.63119366785771835</v>
-      </c>
-      <c r="E56">
-        <f t="shared" si="7"/>
-        <v>0.62400158677722917</v>
-      </c>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>10</v>
-      </c>
-      <c r="B57">
-        <v>0.26307471264367821</v>
-      </c>
-      <c r="C57">
-        <v>0.25445402298850572</v>
-      </c>
-      <c r="D57">
-        <v>0.26307471264367821</v>
-      </c>
-      <c r="E57">
-        <f t="shared" si="7"/>
-        <v>0.26020114942528738</v>
-      </c>
-      <c r="F57" s="2"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>11</v>
-      </c>
-      <c r="B58">
-        <v>0.41379310344827591</v>
-      </c>
-      <c r="C58">
-        <v>0.40517241379310343</v>
-      </c>
-      <c r="D58">
-        <v>0.41379310344827591</v>
-      </c>
-      <c r="E58">
-        <f t="shared" si="7"/>
-        <v>0.41091954022988508</v>
-      </c>
-      <c r="F58" s="2"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>12</v>
-      </c>
-      <c r="B59" s="1">
-        <v>11.927592316578171</v>
-      </c>
-      <c r="C59" s="1">
-        <v>11.35648157267735</v>
-      </c>
-      <c r="D59">
-        <v>11.18512282289308</v>
-      </c>
-      <c r="E59">
-        <f t="shared" si="7"/>
-        <v>11.489732237382867</v>
-      </c>
-      <c r="F59" s="2"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>21</v>
-      </c>
-      <c r="B60">
-        <v>0.23139506578445429</v>
-      </c>
-      <c r="C60">
-        <v>0.23139506578445429</v>
-      </c>
-      <c r="D60">
-        <v>0.23139506578445429</v>
-      </c>
-      <c r="E60">
-        <f t="shared" si="7"/>
-        <v>0.23139506578445426</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>22</v>
-      </c>
-      <c r="B61">
-        <v>0.1802072674036026</v>
-      </c>
-      <c r="C61">
-        <v>0.1802072674036026</v>
-      </c>
-      <c r="D61">
-        <v>0.1802072674036026</v>
-      </c>
-      <c r="E61">
-        <f t="shared" si="7"/>
-        <v>0.1802072674036026</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>23</v>
-      </c>
-      <c r="B62">
-        <v>0.28273653984069819</v>
-      </c>
-      <c r="C62">
-        <v>0.28273653984069819</v>
-      </c>
-      <c r="D62">
-        <v>0.28273653984069819</v>
-      </c>
-      <c r="E62">
-        <f t="shared" si="7"/>
-        <v>0.28273653984069819</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>24</v>
-      </c>
-      <c r="B63">
-        <v>282400</v>
-      </c>
-      <c r="C63">
-        <v>282400</v>
-      </c>
-      <c r="D63">
-        <v>282400</v>
-      </c>
-      <c r="E63">
-        <f t="shared" si="7"/>
-        <v>282400</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>25</v>
-      </c>
-      <c r="B64">
-        <v>255600</v>
-      </c>
-      <c r="C64">
-        <v>255600</v>
-      </c>
-      <c r="D64">
-        <v>255600</v>
-      </c>
-      <c r="E64">
-        <f t="shared" si="7"/>
-        <v>255600</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>26</v>
-      </c>
-      <c r="B65">
-        <v>26800</v>
-      </c>
-      <c r="C65">
-        <v>26800</v>
-      </c>
-      <c r="D65">
-        <v>26800</v>
-      </c>
-      <c r="E65">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>26800</v>
       </c>
     </row>

</xml_diff>